<commit_message>
#34 Changes to be made
</commit_message>
<xml_diff>
--- a/Deliverables/BOM/PAC5527/eSpark_BOM.xlsx
+++ b/Deliverables/BOM/PAC5527/eSpark_BOM.xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="360" uniqueCount="252">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="412" uniqueCount="266">
   <si>
     <t>Component list</t>
   </si>
@@ -574,15 +574,9 @@
     <t>C105174</t>
   </si>
   <si>
-    <t>C2167787</t>
-  </si>
-  <si>
     <t>C302028</t>
   </si>
   <si>
-    <t>C2176546</t>
-  </si>
-  <si>
     <t>C106204</t>
   </si>
   <si>
@@ -613,12 +607,6 @@
     <t>C185446</t>
   </si>
   <si>
-    <t>C2074203</t>
-  </si>
-  <si>
-    <t>C2074142</t>
-  </si>
-  <si>
     <t>C2828647</t>
   </si>
   <si>
@@ -785,17 +773,72 @@
   </si>
   <si>
     <t>LCSC</t>
+  </si>
+  <si>
+    <t>3mm</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>CC1206KKX7R9BB475</t>
+  </si>
+  <si>
+    <t>C132170</t>
+  </si>
+  <si>
+    <t>CC0402KRX7R0BB102</t>
+  </si>
+  <si>
+    <t>C527013</t>
+  </si>
+  <si>
+    <t>C37208</t>
+  </si>
+  <si>
+    <t>PZ254V-11-02P</t>
+  </si>
+  <si>
+    <t>C492401</t>
+  </si>
+  <si>
+    <t>C441916</t>
+  </si>
+  <si>
+    <t>ERJPA3F1000V</t>
+  </si>
+  <si>
+    <t>AC0603JR-07100KL</t>
+  </si>
+  <si>
+    <t>C144628</t>
+  </si>
+  <si>
+    <t>RC0402FR-071KL</t>
+  </si>
+  <si>
+    <t>C2935237</t>
+  </si>
+  <si>
+    <t>C112005</t>
+  </si>
+  <si>
+    <t>Total Cost</t>
+  </si>
+  <si>
+    <t>Cost per Board</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="[$-409]h:mm:ss\ AM/PM;@"/>
     <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.0000"/>
+    <numFmt numFmtId="170" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="20" x14ac:knownFonts="1">
+  <fonts count="23" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -932,8 +975,31 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <strike/>
+      <sz val="9"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -964,8 +1030,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2" tint="-9.9978637043366805E-2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="28">
+  <borders count="31">
     <border>
       <left/>
       <right/>
@@ -1290,12 +1362,51 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="92">
+  <cellXfs count="100">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1410,24 +1521,6 @@
     <xf numFmtId="0" fontId="11" fillId="3" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="18" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1436,9 +1529,6 @@
     </xf>
     <xf numFmtId="0" fontId="18" fillId="4" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="165" fontId="18" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1467,9 +1557,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="18" fillId="2" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1545,6 +1632,56 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="165" fontId="19" fillId="4" borderId="6" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="6" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="170" fontId="17" fillId="3" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="18" fillId="2" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="170" fontId="17" fillId="3" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1895,9 +2032,9 @@
     <col min="2" max="2" width="3.140625" style="19" customWidth="1"/>
     <col min="3" max="3" width="18" style="19" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="27.42578125" customWidth="1"/>
-    <col min="5" max="5" width="30.85546875" customWidth="1"/>
-    <col min="6" max="6" width="22.28515625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="33.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="43.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="26.5703125" customWidth="1"/>
+    <col min="7" max="7" width="36.140625" customWidth="1"/>
     <col min="8" max="8" width="21.42578125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="29.7109375" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="25.7109375" bestFit="1" customWidth="1"/>
@@ -1923,18 +2060,18 @@
       <c r="H1" s="2"/>
       <c r="I1" s="2"/>
       <c r="J1" s="2"/>
-      <c r="K1" s="41"/>
-      <c r="L1" s="41"/>
-      <c r="M1" s="41"/>
-      <c r="N1" s="41"/>
-      <c r="O1" s="41"/>
-      <c r="P1" s="41"/>
-      <c r="Q1" s="41"/>
-      <c r="R1" s="41"/>
-      <c r="S1" s="41"/>
-      <c r="T1" s="41"/>
-      <c r="U1" s="41"/>
-      <c r="V1" s="42"/>
+      <c r="K1" s="84"/>
+      <c r="L1" s="84"/>
+      <c r="M1" s="84"/>
+      <c r="N1" s="84"/>
+      <c r="O1" s="84"/>
+      <c r="P1" s="84"/>
+      <c r="Q1" s="84"/>
+      <c r="R1" s="84"/>
+      <c r="S1" s="84"/>
+      <c r="T1" s="84"/>
+      <c r="U1" s="84"/>
+      <c r="V1" s="85"/>
     </row>
     <row r="2" spans="1:22" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
@@ -1943,8 +2080,8 @@
       <c r="D2" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="E2" s="65"/>
-      <c r="F2" s="74" t="s">
+      <c r="E2" s="57"/>
+      <c r="F2" s="66" t="s">
         <v>5</v>
       </c>
       <c r="G2" s="38"/>
@@ -1967,39 +2104,39 @@
     <row r="3" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
       <c r="B3" s="16"/>
-      <c r="C3" s="75"/>
-      <c r="D3" s="67" t="s">
+      <c r="C3" s="67"/>
+      <c r="D3" s="59" t="s">
         <v>1</v>
       </c>
-      <c r="E3" s="67"/>
-      <c r="F3" s="66" t="s">
+      <c r="E3" s="59"/>
+      <c r="F3" s="58" t="s">
         <v>6</v>
       </c>
-      <c r="G3" s="67"/>
-      <c r="H3" s="56"/>
-      <c r="I3" s="67"/>
-      <c r="J3" s="56"/>
+      <c r="G3" s="59"/>
+      <c r="H3" s="49"/>
+      <c r="I3" s="59"/>
+      <c r="J3" s="49"/>
       <c r="K3" s="5"/>
-      <c r="L3" s="56"/>
-      <c r="M3" s="56"/>
-      <c r="N3" s="56"/>
-      <c r="O3" s="56"/>
-      <c r="P3" s="56"/>
-      <c r="Q3" s="56"/>
-      <c r="R3" s="56"/>
-      <c r="S3" s="56"/>
-      <c r="T3" s="56"/>
-      <c r="U3" s="56"/>
-      <c r="V3" s="43"/>
+      <c r="L3" s="49"/>
+      <c r="M3" s="49"/>
+      <c r="N3" s="49"/>
+      <c r="O3" s="49"/>
+      <c r="P3" s="49"/>
+      <c r="Q3" s="49"/>
+      <c r="R3" s="49"/>
+      <c r="S3" s="49"/>
+      <c r="T3" s="49"/>
+      <c r="U3" s="49"/>
+      <c r="V3" s="86"/>
     </row>
     <row r="4" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
       <c r="B4" s="16"/>
-      <c r="C4" s="75"/>
-      <c r="D4" s="67" t="s">
+      <c r="C4" s="67"/>
+      <c r="D4" s="59" t="s">
         <v>2</v>
       </c>
-      <c r="E4" s="67"/>
+      <c r="E4" s="59"/>
       <c r="F4" s="39" t="s">
         <v>6</v>
       </c>
@@ -2017,17 +2154,17 @@
       <c r="R4" s="6"/>
       <c r="S4" s="6"/>
       <c r="T4" s="6"/>
-      <c r="U4" s="83"/>
-      <c r="V4" s="44"/>
+      <c r="U4" s="75"/>
+      <c r="V4" s="87"/>
     </row>
     <row r="5" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
       <c r="B5" s="16"/>
-      <c r="C5" s="75"/>
-      <c r="D5" s="67" t="s">
+      <c r="C5" s="67"/>
+      <c r="D5" s="59" t="s">
         <v>3</v>
       </c>
-      <c r="E5" s="67"/>
+      <c r="E5" s="59"/>
       <c r="F5" s="40" t="s">
         <v>7</v>
       </c>
@@ -2046,14 +2183,14 @@
       <c r="S5" s="5"/>
       <c r="T5" s="5"/>
       <c r="U5" s="5"/>
-      <c r="V5" s="44"/>
+      <c r="V5" s="87"/>
     </row>
     <row r="6" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
       <c r="B6" s="16"/>
-      <c r="C6" s="75"/>
-      <c r="D6" s="67"/>
-      <c r="E6" s="67"/>
+      <c r="C6" s="67"/>
+      <c r="D6" s="59"/>
+      <c r="E6" s="59"/>
       <c r="F6" s="12"/>
       <c r="G6" s="11"/>
       <c r="H6" s="5"/>
@@ -2070,55 +2207,55 @@
       <c r="S6" s="5"/>
       <c r="T6" s="5"/>
       <c r="U6" s="5"/>
-      <c r="V6" s="44"/>
+      <c r="V6" s="87"/>
     </row>
     <row r="7" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
       <c r="B7" s="17"/>
-      <c r="C7" s="76"/>
-      <c r="D7" s="68"/>
-      <c r="E7" s="68"/>
+      <c r="C7" s="68"/>
+      <c r="D7" s="60"/>
+      <c r="E7" s="60"/>
       <c r="F7" s="13"/>
-      <c r="G7" s="68"/>
-      <c r="H7" s="57"/>
-      <c r="I7" s="68"/>
-      <c r="J7" s="57"/>
-      <c r="K7" s="57"/>
-      <c r="L7" s="57"/>
-      <c r="M7" s="57"/>
-      <c r="N7" s="57"/>
-      <c r="O7" s="57"/>
-      <c r="P7" s="57"/>
-      <c r="Q7" s="57"/>
-      <c r="R7" s="57"/>
-      <c r="S7" s="57"/>
-      <c r="T7" s="57"/>
-      <c r="U7" s="57"/>
-      <c r="V7" s="44"/>
+      <c r="G7" s="60"/>
+      <c r="H7" s="50"/>
+      <c r="I7" s="60"/>
+      <c r="J7" s="50"/>
+      <c r="K7" s="50"/>
+      <c r="L7" s="50"/>
+      <c r="M7" s="50"/>
+      <c r="N7" s="50"/>
+      <c r="O7" s="50"/>
+      <c r="P7" s="50"/>
+      <c r="Q7" s="50"/>
+      <c r="R7" s="50"/>
+      <c r="S7" s="50"/>
+      <c r="T7" s="50"/>
+      <c r="U7" s="50"/>
+      <c r="V7" s="87"/>
     </row>
     <row r="8" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
-      <c r="B8" s="77"/>
-      <c r="C8" s="78"/>
-      <c r="D8" s="79"/>
-      <c r="E8" s="79"/>
-      <c r="F8" s="80"/>
-      <c r="G8" s="81"/>
-      <c r="H8" s="82"/>
-      <c r="I8" s="81"/>
-      <c r="J8" s="82"/>
-      <c r="K8" s="82"/>
-      <c r="L8" s="82"/>
-      <c r="M8" s="82"/>
-      <c r="N8" s="82"/>
-      <c r="O8" s="82"/>
-      <c r="P8" s="82"/>
-      <c r="Q8" s="82"/>
-      <c r="R8" s="82"/>
-      <c r="S8" s="82"/>
-      <c r="T8" s="82"/>
-      <c r="U8" s="82"/>
-      <c r="V8" s="50"/>
+      <c r="B8" s="69"/>
+      <c r="C8" s="70"/>
+      <c r="D8" s="71"/>
+      <c r="E8" s="71"/>
+      <c r="F8" s="72"/>
+      <c r="G8" s="73"/>
+      <c r="H8" s="74"/>
+      <c r="I8" s="73"/>
+      <c r="J8" s="74"/>
+      <c r="K8" s="74"/>
+      <c r="L8" s="74"/>
+      <c r="M8" s="74"/>
+      <c r="N8" s="74"/>
+      <c r="O8" s="74"/>
+      <c r="P8" s="74"/>
+      <c r="Q8" s="74"/>
+      <c r="R8" s="74"/>
+      <c r="S8" s="74"/>
+      <c r="T8" s="74"/>
+      <c r="U8" s="74"/>
+      <c r="V8" s="88"/>
     </row>
     <row r="9" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
@@ -2128,10 +2265,10 @@
       <c r="C9" s="20" t="s">
         <v>8</v>
       </c>
-      <c r="D9" s="48" t="s">
+      <c r="D9" s="42" t="s">
         <v>13</v>
       </c>
-      <c r="E9" s="53" t="s">
+      <c r="E9" s="46" t="s">
         <v>53</v>
       </c>
       <c r="F9" s="20" t="s">
@@ -2144,46 +2281,46 @@
         <v>150</v>
       </c>
       <c r="I9" s="20" t="s">
-        <v>234</v>
+        <v>230</v>
       </c>
       <c r="J9" s="21" t="s">
         <v>173</v>
       </c>
       <c r="K9" s="20" t="s">
+        <v>231</v>
+      </c>
+      <c r="L9" s="20" t="s">
+        <v>222</v>
+      </c>
+      <c r="M9" s="20" t="s">
+        <v>233</v>
+      </c>
+      <c r="N9" s="42" t="s">
         <v>235</v>
       </c>
-      <c r="L9" s="20" t="s">
-        <v>226</v>
-      </c>
-      <c r="M9" s="20" t="s">
+      <c r="O9" s="20" t="s">
+        <v>232</v>
+      </c>
+      <c r="P9" s="20" t="s">
+        <v>234</v>
+      </c>
+      <c r="Q9" s="46" t="s">
+        <v>236</v>
+      </c>
+      <c r="R9" s="20" t="s">
+        <v>240</v>
+      </c>
+      <c r="S9" s="20" t="s">
+        <v>241</v>
+      </c>
+      <c r="T9" s="20" t="s">
         <v>237</v>
       </c>
-      <c r="N9" s="48" t="s">
+      <c r="U9" s="20" t="s">
+        <v>238</v>
+      </c>
+      <c r="V9" s="42" t="s">
         <v>239</v>
-      </c>
-      <c r="O9" s="20" t="s">
-        <v>236</v>
-      </c>
-      <c r="P9" s="20" t="s">
-        <v>238</v>
-      </c>
-      <c r="Q9" s="53" t="s">
-        <v>240</v>
-      </c>
-      <c r="R9" s="20" t="s">
-        <v>244</v>
-      </c>
-      <c r="S9" s="20" t="s">
-        <v>245</v>
-      </c>
-      <c r="T9" s="20" t="s">
-        <v>241</v>
-      </c>
-      <c r="U9" s="20" t="s">
-        <v>242</v>
-      </c>
-      <c r="V9" s="48" t="s">
-        <v>243</v>
       </c>
     </row>
     <row r="10" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -2193,29 +2330,29 @@
         <v>1</v>
       </c>
       <c r="C10" s="30" t="s">
-        <v>227</v>
+        <v>223</v>
       </c>
       <c r="D10" s="31" t="s">
         <v>14</v>
       </c>
-      <c r="E10" s="63" t="s">
-        <v>246</v>
+      <c r="E10" s="55" t="s">
+        <v>242</v>
       </c>
       <c r="F10" s="37" t="s">
-        <v>247</v>
+        <v>243</v>
       </c>
       <c r="G10" s="31" t="s">
-        <v>248</v>
+        <v>244</v>
       </c>
       <c r="H10" s="30" t="s">
-        <v>249</v>
+        <v>245</v>
       </c>
       <c r="I10" s="31"/>
       <c r="J10" s="30" t="s">
-        <v>250</v>
+        <v>246</v>
       </c>
       <c r="K10" s="31" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
       <c r="L10" s="37">
         <v>2</v>
@@ -2233,20 +2370,20 @@
       <c r="P10" s="37">
         <v>20</v>
       </c>
-      <c r="Q10" s="90" t="s">
-        <v>251</v>
+      <c r="Q10" s="82" t="s">
+        <v>247</v>
       </c>
       <c r="R10" s="35">
         <v>0.29630000000000001</v>
       </c>
       <c r="S10" s="35">
-        <v>1.48</v>
+        <v>2.96</v>
       </c>
       <c r="T10" s="35">
         <v>0.29630000000000001</v>
       </c>
       <c r="U10" s="35">
-        <v>2.96</v>
+        <v>5.93</v>
       </c>
       <c r="V10" s="32"/>
     </row>
@@ -2257,12 +2394,12 @@
         <v>2</v>
       </c>
       <c r="C11" s="33" t="s">
-        <v>227</v>
+        <v>223</v>
       </c>
       <c r="D11" s="34" t="s">
         <v>15</v>
       </c>
-      <c r="E11" s="55" t="s">
+      <c r="E11" s="48" t="s">
         <v>54</v>
       </c>
       <c r="F11" s="33" t="s">
@@ -2279,13 +2416,13 @@
         <v>174</v>
       </c>
       <c r="K11" s="34" t="s">
-        <v>205</v>
+        <v>201</v>
       </c>
       <c r="L11" s="33">
         <v>2</v>
       </c>
-      <c r="M11" s="58">
-        <f t="shared" ref="M11" si="1">L11*5</f>
+      <c r="M11" s="51">
+        <f>L11*5</f>
         <v>10</v>
       </c>
       <c r="N11" s="34">
@@ -2294,11 +2431,11 @@
       <c r="O11" s="33">
         <v>20</v>
       </c>
-      <c r="P11" s="84">
+      <c r="P11" s="76">
         <v>100</v>
       </c>
-      <c r="Q11" s="91" t="s">
-        <v>251</v>
+      <c r="Q11" s="83" t="s">
+        <v>247</v>
       </c>
       <c r="R11" s="36">
         <v>5.1000000000000004E-3</v>
@@ -2312,7 +2449,7 @@
       <c r="U11" s="36">
         <v>0.51</v>
       </c>
-      <c r="V11" s="58"/>
+      <c r="V11" s="51"/>
     </row>
     <row r="12" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="1"/>
@@ -2321,12 +2458,12 @@
         <v>3</v>
       </c>
       <c r="C12" s="30" t="s">
-        <v>227</v>
+        <v>223</v>
       </c>
       <c r="D12" s="31" t="s">
         <v>16</v>
       </c>
-      <c r="E12" s="63" t="s">
+      <c r="E12" s="55" t="s">
         <v>55</v>
       </c>
       <c r="F12" s="30" t="s">
@@ -2343,9 +2480,9 @@
         <v>175</v>
       </c>
       <c r="K12" s="31" t="s">
-        <v>206</v>
-      </c>
-      <c r="L12" s="61">
+        <v>202</v>
+      </c>
+      <c r="L12" s="54">
         <v>2</v>
       </c>
       <c r="M12" s="32">
@@ -2358,11 +2495,11 @@
       <c r="O12" s="30">
         <v>20</v>
       </c>
-      <c r="P12" s="85">
+      <c r="P12" s="77">
         <v>50</v>
       </c>
-      <c r="Q12" s="90" t="s">
-        <v>251</v>
+      <c r="Q12" s="82" t="s">
+        <v>247</v>
       </c>
       <c r="R12" s="35">
         <v>1.78E-2</v>
@@ -2385,12 +2522,12 @@
         <v>4</v>
       </c>
       <c r="C13" s="33" t="s">
-        <v>227</v>
+        <v>223</v>
       </c>
       <c r="D13" s="34" t="s">
         <v>17</v>
       </c>
-      <c r="E13" s="55" t="s">
+      <c r="E13" s="48" t="s">
         <v>56</v>
       </c>
       <c r="F13" s="33" t="s">
@@ -2407,13 +2544,13 @@
         <v>176</v>
       </c>
       <c r="K13" s="34" t="s">
-        <v>207</v>
+        <v>203</v>
       </c>
       <c r="L13" s="33">
         <v>1</v>
       </c>
-      <c r="M13" s="58">
-        <f t="shared" ref="M13" si="2">L13*5</f>
+      <c r="M13" s="51">
+        <f t="shared" ref="M13" si="1">L13*5</f>
         <v>5</v>
       </c>
       <c r="N13" s="34">
@@ -2422,11 +2559,11 @@
       <c r="O13" s="33">
         <v>10</v>
       </c>
-      <c r="P13" s="84">
+      <c r="P13" s="76">
         <v>50</v>
       </c>
-      <c r="Q13" s="91" t="s">
-        <v>251</v>
+      <c r="Q13" s="83" t="s">
+        <v>247</v>
       </c>
       <c r="R13" s="36">
         <v>1.7100000000000001E-2</v>
@@ -2440,7 +2577,7 @@
       <c r="U13" s="36">
         <v>0.86</v>
       </c>
-      <c r="V13" s="58"/>
+      <c r="V13" s="51"/>
     </row>
     <row r="14" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="1"/>
@@ -2449,12 +2586,12 @@
         <v>5</v>
       </c>
       <c r="C14" s="30" t="s">
-        <v>227</v>
+        <v>223</v>
       </c>
       <c r="D14" s="31" t="s">
         <v>18</v>
       </c>
-      <c r="E14" s="63" t="s">
+      <c r="E14" s="55" t="s">
         <v>57</v>
       </c>
       <c r="F14" s="30" t="s">
@@ -2471,9 +2608,9 @@
         <v>177</v>
       </c>
       <c r="K14" s="31" t="s">
-        <v>208</v>
-      </c>
-      <c r="L14" s="61">
+        <v>204</v>
+      </c>
+      <c r="L14" s="54">
         <v>1</v>
       </c>
       <c r="M14" s="32">
@@ -2486,11 +2623,11 @@
       <c r="O14" s="30">
         <v>10</v>
       </c>
-      <c r="P14" s="85">
+      <c r="P14" s="77">
         <v>20</v>
       </c>
-      <c r="Q14" s="90" t="s">
-        <v>251</v>
+      <c r="Q14" s="82" t="s">
+        <v>247</v>
       </c>
       <c r="R14" s="35">
         <v>1.3299999999999999E-2</v>
@@ -2513,12 +2650,12 @@
         <v>6</v>
       </c>
       <c r="C15" s="33" t="s">
-        <v>227</v>
+        <v>223</v>
       </c>
       <c r="D15" s="34" t="s">
         <v>19</v>
       </c>
-      <c r="E15" s="55" t="s">
+      <c r="E15" s="48" t="s">
         <v>55</v>
       </c>
       <c r="F15" s="33" t="s">
@@ -2535,13 +2672,13 @@
         <v>178</v>
       </c>
       <c r="K15" s="34" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
       <c r="L15" s="33">
         <v>2</v>
       </c>
-      <c r="M15" s="58">
-        <f t="shared" ref="M15" si="3">L15*5</f>
+      <c r="M15" s="51">
+        <f t="shared" ref="M15" si="2">L15*5</f>
         <v>10</v>
       </c>
       <c r="N15" s="34">
@@ -2550,11 +2687,11 @@
       <c r="O15" s="33">
         <v>20</v>
       </c>
-      <c r="P15" s="84">
+      <c r="P15" s="76">
         <v>50</v>
       </c>
-      <c r="Q15" s="91" t="s">
-        <v>251</v>
+      <c r="Q15" s="83" t="s">
+        <v>247</v>
       </c>
       <c r="R15" s="36">
         <v>7.1999999999999998E-3</v>
@@ -2568,7 +2705,7 @@
       <c r="U15" s="36">
         <v>0.36</v>
       </c>
-      <c r="V15" s="58"/>
+      <c r="V15" s="51"/>
     </row>
     <row r="16" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="1"/>
@@ -2577,12 +2714,12 @@
         <v>7</v>
       </c>
       <c r="C16" s="30" t="s">
-        <v>227</v>
+        <v>223</v>
       </c>
       <c r="D16" s="31" t="s">
         <v>20</v>
       </c>
-      <c r="E16" s="63" t="s">
+      <c r="E16" s="55" t="s">
         <v>58</v>
       </c>
       <c r="F16" s="30" t="s">
@@ -2599,9 +2736,9 @@
         <v>179</v>
       </c>
       <c r="K16" s="31" t="s">
-        <v>205</v>
-      </c>
-      <c r="L16" s="61">
+        <v>201</v>
+      </c>
+      <c r="L16" s="54">
         <v>1</v>
       </c>
       <c r="M16" s="32">
@@ -2614,11 +2751,11 @@
       <c r="O16" s="30">
         <v>10</v>
       </c>
-      <c r="P16" s="85">
+      <c r="P16" s="77">
         <v>100</v>
       </c>
-      <c r="Q16" s="90" t="s">
-        <v>251</v>
+      <c r="Q16" s="82" t="s">
+        <v>247</v>
       </c>
       <c r="R16" s="35">
         <v>2.5999999999999999E-3</v>
@@ -2641,12 +2778,12 @@
         <v>8</v>
       </c>
       <c r="C17" s="33" t="s">
-        <v>227</v>
+        <v>223</v>
       </c>
       <c r="D17" s="34" t="s">
         <v>21</v>
       </c>
-      <c r="E17" s="55" t="s">
+      <c r="E17" s="48" t="s">
         <v>59</v>
       </c>
       <c r="F17" s="33" t="s">
@@ -2663,13 +2800,13 @@
         <v>180</v>
       </c>
       <c r="K17" s="34" t="s">
-        <v>209</v>
+        <v>205</v>
       </c>
       <c r="L17" s="33">
         <v>1</v>
       </c>
-      <c r="M17" s="58">
-        <f t="shared" ref="M17" si="4">L17*5</f>
+      <c r="M17" s="51">
+        <f t="shared" ref="M17" si="3">L17*5</f>
         <v>5</v>
       </c>
       <c r="N17" s="34">
@@ -2678,11 +2815,11 @@
       <c r="O17" s="33">
         <v>10</v>
       </c>
-      <c r="P17" s="84">
+      <c r="P17" s="76">
         <v>20</v>
       </c>
-      <c r="Q17" s="91" t="s">
-        <v>251</v>
+      <c r="Q17" s="83" t="s">
+        <v>247</v>
       </c>
       <c r="R17" s="36">
         <v>2.7199999999999998E-2</v>
@@ -2696,7 +2833,7 @@
       <c r="U17" s="36">
         <v>0.54</v>
       </c>
-      <c r="V17" s="58"/>
+      <c r="V17" s="51"/>
     </row>
     <row r="18" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="1"/>
@@ -2705,47 +2842,63 @@
         <v>9</v>
       </c>
       <c r="C18" s="30" t="s">
-        <v>227</v>
+        <v>223</v>
       </c>
       <c r="D18" s="31" t="s">
         <v>22</v>
       </c>
-      <c r="E18" s="63" t="s">
+      <c r="E18" s="55" t="s">
         <v>60</v>
       </c>
       <c r="F18" s="30" t="s">
         <v>94</v>
       </c>
-      <c r="G18" s="31" t="s">
+      <c r="G18" s="91" t="s">
         <v>126</v>
       </c>
       <c r="H18" s="30" t="s">
         <v>154</v>
       </c>
-      <c r="I18" s="31"/>
+      <c r="I18" s="30" t="s">
+        <v>250</v>
+      </c>
       <c r="J18" s="30" t="s">
-        <v>181</v>
+        <v>251</v>
       </c>
       <c r="K18" s="31" t="s">
-        <v>207</v>
-      </c>
-      <c r="L18" s="61">
+        <v>203</v>
+      </c>
+      <c r="L18" s="54">
         <v>3</v>
       </c>
       <c r="M18" s="32">
         <f>L18*5</f>
         <v>15</v>
       </c>
-      <c r="N18" s="31"/>
-      <c r="O18" s="30"/>
-      <c r="P18" s="85"/>
-      <c r="Q18" s="51" t="s">
-        <v>251</v>
-      </c>
-      <c r="R18" s="35"/>
-      <c r="S18" s="35"/>
-      <c r="T18" s="35"/>
-      <c r="U18" s="35"/>
+      <c r="N18" s="31">
+        <v>20</v>
+      </c>
+      <c r="O18" s="30">
+        <v>30</v>
+      </c>
+      <c r="P18" s="77">
+        <v>30</v>
+      </c>
+      <c r="Q18" s="82" t="s">
+        <v>247</v>
+      </c>
+      <c r="R18" s="35">
+        <v>6.0299999999999999E-2</v>
+      </c>
+      <c r="S18" s="35">
+        <v>1.21</v>
+      </c>
+      <c r="T18" s="35">
+        <v>6.0299999999999999E-2</v>
+      </c>
+      <c r="U18" s="35">
+        <v>1.81</v>
+      </c>
       <c r="V18" s="32"/>
     </row>
     <row r="19" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -2755,12 +2908,12 @@
         <v>10</v>
       </c>
       <c r="C19" s="33" t="s">
-        <v>227</v>
+        <v>223</v>
       </c>
       <c r="D19" s="34" t="s">
         <v>23</v>
       </c>
-      <c r="E19" s="55" t="s">
+      <c r="E19" s="48" t="s">
         <v>61</v>
       </c>
       <c r="F19" s="33" t="s">
@@ -2774,16 +2927,16 @@
       </c>
       <c r="I19" s="34"/>
       <c r="J19" s="33" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="K19" s="34" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="L19" s="33">
         <v>3</v>
       </c>
-      <c r="M19" s="58">
-        <f t="shared" ref="M19" si="5">L19*5</f>
+      <c r="M19" s="51">
+        <f t="shared" ref="M19" si="4">L19*5</f>
         <v>15</v>
       </c>
       <c r="N19" s="34">
@@ -2792,11 +2945,11 @@
       <c r="O19" s="33">
         <v>30</v>
       </c>
-      <c r="P19" s="84">
+      <c r="P19" s="76">
         <v>50</v>
       </c>
-      <c r="Q19" s="91" t="s">
-        <v>251</v>
+      <c r="Q19" s="83" t="s">
+        <v>247</v>
       </c>
       <c r="R19" s="36">
         <v>7.0000000000000001E-3</v>
@@ -2810,7 +2963,7 @@
       <c r="U19" s="36">
         <v>0.35</v>
       </c>
-      <c r="V19" s="58"/>
+      <c r="V19" s="51"/>
     </row>
     <row r="20" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="1"/>
@@ -2819,49 +2972,63 @@
         <v>11</v>
       </c>
       <c r="C20" s="30" t="s">
-        <v>227</v>
+        <v>223</v>
       </c>
       <c r="D20" s="31" t="s">
         <v>24</v>
       </c>
-      <c r="E20" s="63" t="s">
+      <c r="E20" s="55" t="s">
         <v>62</v>
       </c>
       <c r="F20" s="30" t="s">
         <v>95</v>
       </c>
-      <c r="G20" s="31">
+      <c r="G20" s="91">
         <v>885012205080</v>
       </c>
       <c r="H20" s="30" t="s">
         <v>156</v>
       </c>
-      <c r="I20" s="31"/>
+      <c r="I20" s="30" t="s">
+        <v>252</v>
+      </c>
       <c r="J20" s="30" t="s">
-        <v>183</v>
+        <v>253</v>
       </c>
       <c r="K20" s="31" t="s">
-        <v>211</v>
-      </c>
-      <c r="L20" s="61">
+        <v>207</v>
+      </c>
+      <c r="L20" s="54">
         <v>3</v>
       </c>
       <c r="M20" s="32">
         <f>L20*5</f>
         <v>15</v>
       </c>
-      <c r="N20" s="31"/>
+      <c r="N20" s="31">
+        <v>100</v>
+      </c>
       <c r="O20" s="30">
         <v>30</v>
       </c>
-      <c r="P20" s="85"/>
-      <c r="Q20" s="51" t="s">
-        <v>251</v>
-      </c>
-      <c r="R20" s="35"/>
-      <c r="S20" s="35"/>
-      <c r="T20" s="35"/>
-      <c r="U20" s="35"/>
+      <c r="P20" s="77">
+        <v>100</v>
+      </c>
+      <c r="Q20" s="82" t="s">
+        <v>247</v>
+      </c>
+      <c r="R20" s="35">
+        <v>4.1999999999999997E-3</v>
+      </c>
+      <c r="S20" s="35">
+        <v>0.42</v>
+      </c>
+      <c r="T20" s="35">
+        <v>4.1999999999999997E-3</v>
+      </c>
+      <c r="U20" s="35">
+        <v>0.42</v>
+      </c>
       <c r="V20" s="32"/>
     </row>
     <row r="21" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -2871,12 +3038,12 @@
         <v>12</v>
       </c>
       <c r="C21" s="33" t="s">
-        <v>227</v>
+        <v>223</v>
       </c>
       <c r="D21" s="34" t="s">
         <v>25</v>
       </c>
-      <c r="E21" s="55" t="s">
+      <c r="E21" s="48" t="s">
         <v>63</v>
       </c>
       <c r="F21" s="33" t="s">
@@ -2890,31 +3057,43 @@
       </c>
       <c r="I21" s="34"/>
       <c r="J21" s="33" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="K21" s="34" t="s">
-        <v>205</v>
+        <v>201</v>
       </c>
       <c r="L21" s="33">
         <v>1</v>
       </c>
-      <c r="M21" s="58">
-        <f t="shared" ref="M21" si="6">L21*5</f>
+      <c r="M21" s="51">
+        <f t="shared" ref="M21" si="5">L21*5</f>
         <v>5</v>
       </c>
-      <c r="N21" s="34"/>
+      <c r="N21" s="34">
+        <v>100</v>
+      </c>
       <c r="O21" s="33">
         <v>10</v>
       </c>
-      <c r="P21" s="84"/>
-      <c r="Q21" s="52" t="s">
-        <v>251</v>
-      </c>
-      <c r="R21" s="36"/>
-      <c r="S21" s="36"/>
-      <c r="T21" s="36"/>
-      <c r="U21" s="36"/>
-      <c r="V21" s="58"/>
+      <c r="P21" s="76">
+        <v>100</v>
+      </c>
+      <c r="Q21" s="83" t="s">
+        <v>247</v>
+      </c>
+      <c r="R21" s="36">
+        <v>8.9999999999999998E-4</v>
+      </c>
+      <c r="S21" s="36">
+        <v>0.09</v>
+      </c>
+      <c r="T21" s="36">
+        <v>8.9999999999999998E-4</v>
+      </c>
+      <c r="U21" s="36">
+        <v>0.09</v>
+      </c>
+      <c r="V21" s="51"/>
     </row>
     <row r="22" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="1"/>
@@ -2922,13 +3101,13 @@
         <f>ROW(B22) - ROW($B$9)</f>
         <v>13</v>
       </c>
-      <c r="C22" s="61" t="s">
-        <v>228</v>
+      <c r="C22" s="54" t="s">
+        <v>224</v>
       </c>
       <c r="D22" s="31" t="s">
         <v>26</v>
       </c>
-      <c r="E22" s="63" t="s">
+      <c r="E22" s="55" t="s">
         <v>64</v>
       </c>
       <c r="F22" s="30" t="s">
@@ -2942,30 +3121,42 @@
       </c>
       <c r="I22" s="31"/>
       <c r="J22" s="30" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="K22" s="31" t="s">
-        <v>129</v>
-      </c>
-      <c r="L22" s="61">
+        <v>249</v>
+      </c>
+      <c r="L22" s="54">
         <v>1</v>
       </c>
       <c r="M22" s="32">
         <f>L22*5</f>
         <v>5</v>
       </c>
-      <c r="N22" s="31"/>
+      <c r="N22" s="31">
+        <v>5</v>
+      </c>
       <c r="O22" s="30">
         <v>10</v>
       </c>
-      <c r="P22" s="85"/>
-      <c r="Q22" s="51" t="s">
-        <v>251</v>
-      </c>
-      <c r="R22" s="35"/>
-      <c r="S22" s="35"/>
-      <c r="T22" s="35"/>
-      <c r="U22" s="35"/>
+      <c r="P22" s="77">
+        <v>10</v>
+      </c>
+      <c r="Q22" s="82" t="s">
+        <v>247</v>
+      </c>
+      <c r="R22" s="35">
+        <v>6.1699999999999998E-2</v>
+      </c>
+      <c r="S22" s="35">
+        <v>0.31</v>
+      </c>
+      <c r="T22" s="35">
+        <v>6.1699999999999998E-2</v>
+      </c>
+      <c r="U22" s="35">
+        <v>0.62</v>
+      </c>
       <c r="V22" s="32"/>
     </row>
     <row r="23" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -2975,12 +3166,12 @@
         <v>14</v>
       </c>
       <c r="C23" s="33" t="s">
-        <v>228</v>
+        <v>224</v>
       </c>
       <c r="D23" s="34" t="s">
         <v>27</v>
       </c>
-      <c r="E23" s="55" t="s">
+      <c r="E23" s="48" t="s">
         <v>65</v>
       </c>
       <c r="F23" s="33" t="s">
@@ -2994,31 +3185,43 @@
       </c>
       <c r="I23" s="34"/>
       <c r="J23" s="33" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="K23" s="34" t="s">
-        <v>130</v>
+        <v>249</v>
       </c>
       <c r="L23" s="33">
         <v>3</v>
       </c>
-      <c r="M23" s="58">
-        <f t="shared" ref="M23" si="7">L23*5</f>
+      <c r="M23" s="51">
+        <f t="shared" ref="M23" si="6">L23*5</f>
         <v>15</v>
       </c>
-      <c r="N23" s="34"/>
-      <c r="O23" s="49">
+      <c r="N23" s="34">
+        <v>20</v>
+      </c>
+      <c r="O23" s="43">
         <v>30</v>
       </c>
-      <c r="P23" s="86"/>
-      <c r="Q23" s="52" t="s">
-        <v>251</v>
-      </c>
-      <c r="R23" s="36"/>
-      <c r="S23" s="36"/>
-      <c r="T23" s="36"/>
-      <c r="U23" s="36"/>
-      <c r="V23" s="58"/>
+      <c r="P23" s="78">
+        <v>40</v>
+      </c>
+      <c r="Q23" s="83" t="s">
+        <v>247</v>
+      </c>
+      <c r="R23" s="36">
+        <v>2.2800000000000001E-2</v>
+      </c>
+      <c r="S23" s="36">
+        <v>0.46</v>
+      </c>
+      <c r="T23" s="36">
+        <v>2.2800000000000001E-2</v>
+      </c>
+      <c r="U23" s="36">
+        <v>0.91</v>
+      </c>
+      <c r="V23" s="51"/>
     </row>
     <row r="24" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="1"/>
@@ -3026,49 +3229,65 @@
         <f>ROW(B24) - ROW($B$9)</f>
         <v>15</v>
       </c>
-      <c r="C24" s="61" t="s">
-        <v>229</v>
-      </c>
-      <c r="D24" s="54" t="s">
+      <c r="C24" s="54" t="s">
+        <v>225</v>
+      </c>
+      <c r="D24" s="47" t="s">
         <v>33</v>
       </c>
-      <c r="E24" s="73" t="s">
+      <c r="E24" s="65" t="s">
         <v>70</v>
       </c>
-      <c r="F24" s="61" t="s">
+      <c r="F24" s="54" t="s">
         <v>103</v>
       </c>
-      <c r="G24" s="54">
+      <c r="G24" s="91">
         <v>61300611121</v>
       </c>
-      <c r="H24" s="61" t="s">
+      <c r="H24" s="54" t="s">
         <v>156</v>
       </c>
-      <c r="I24" s="54"/>
-      <c r="J24" s="61"/>
-      <c r="K24" s="54">
-        <v>61300611121</v>
-      </c>
-      <c r="L24" s="61">
+      <c r="I24" s="54" t="s">
+        <v>254</v>
+      </c>
+      <c r="J24" s="54" t="s">
+        <v>254</v>
+      </c>
+      <c r="K24" s="47" t="s">
+        <v>249</v>
+      </c>
+      <c r="L24" s="54">
         <v>1</v>
       </c>
-      <c r="M24" s="59">
+      <c r="M24" s="52">
         <f>L24*5</f>
         <v>5</v>
       </c>
-      <c r="N24" s="54"/>
-      <c r="O24" s="61">
+      <c r="N24" s="47">
+        <v>20</v>
+      </c>
+      <c r="O24" s="54">
         <v>10</v>
       </c>
-      <c r="P24" s="87"/>
-      <c r="Q24" s="51" t="s">
-        <v>251</v>
-      </c>
-      <c r="R24" s="61"/>
-      <c r="S24" s="61"/>
-      <c r="T24" s="61"/>
-      <c r="U24" s="61"/>
-      <c r="V24" s="59"/>
+      <c r="P24" s="79">
+        <v>20</v>
+      </c>
+      <c r="Q24" s="82" t="s">
+        <v>247</v>
+      </c>
+      <c r="R24" s="35">
+        <v>2.75E-2</v>
+      </c>
+      <c r="S24" s="35">
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="T24" s="35">
+        <v>2.75E-2</v>
+      </c>
+      <c r="U24" s="35">
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="V24" s="52"/>
     </row>
     <row r="25" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="1"/>
@@ -3077,48 +3296,64 @@
         <v>16</v>
       </c>
       <c r="C25" s="33" t="s">
-        <v>229</v>
+        <v>225</v>
       </c>
       <c r="D25" s="34" t="s">
         <v>35</v>
       </c>
-      <c r="E25" s="55" t="s">
+      <c r="E25" s="48" t="s">
         <v>72</v>
       </c>
       <c r="F25" s="33" t="s">
         <v>105</v>
       </c>
-      <c r="G25" s="34">
+      <c r="G25" s="92">
         <v>61300211121</v>
       </c>
       <c r="H25" s="33" t="s">
         <v>156</v>
       </c>
-      <c r="I25" s="34"/>
-      <c r="J25" s="33"/>
-      <c r="K25" s="34">
-        <v>61300211121</v>
+      <c r="I25" s="33" t="s">
+        <v>255</v>
+      </c>
+      <c r="J25" s="33" t="s">
+        <v>256</v>
+      </c>
+      <c r="K25" s="34" t="s">
+        <v>249</v>
       </c>
       <c r="L25" s="33">
         <v>1</v>
       </c>
-      <c r="M25" s="58">
-        <f t="shared" ref="M25" si="8">L25*5</f>
+      <c r="M25" s="51">
+        <f t="shared" ref="M25" si="7">L25*5</f>
         <v>5</v>
       </c>
-      <c r="N25" s="34"/>
-      <c r="O25" s="47">
+      <c r="N25" s="34">
+        <v>50</v>
+      </c>
+      <c r="O25" s="41">
         <v>10</v>
       </c>
-      <c r="P25" s="88"/>
-      <c r="Q25" s="52" t="s">
-        <v>251</v>
-      </c>
-      <c r="R25" s="36"/>
-      <c r="S25" s="36"/>
-      <c r="T25" s="36"/>
-      <c r="U25" s="36"/>
-      <c r="V25" s="58"/>
+      <c r="P25" s="80">
+        <v>50</v>
+      </c>
+      <c r="Q25" s="83" t="s">
+        <v>247</v>
+      </c>
+      <c r="R25" s="36">
+        <v>1.38E-2</v>
+      </c>
+      <c r="S25" s="36">
+        <v>0.69</v>
+      </c>
+      <c r="T25" s="36">
+        <v>1.38E-2</v>
+      </c>
+      <c r="U25" s="36">
+        <v>0.69</v>
+      </c>
+      <c r="V25" s="51"/>
     </row>
     <row r="26" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="1"/>
@@ -3126,13 +3361,13 @@
         <f>ROW(B26) - ROW($B$9)</f>
         <v>17</v>
       </c>
-      <c r="C26" s="61" t="s">
-        <v>229</v>
+      <c r="C26" s="54" t="s">
+        <v>225</v>
       </c>
       <c r="D26" s="31" t="s">
         <v>28</v>
       </c>
-      <c r="E26" s="63" t="s">
+      <c r="E26" s="55" t="s">
         <v>66</v>
       </c>
       <c r="F26" s="30" t="s">
@@ -3146,30 +3381,42 @@
       </c>
       <c r="I26" s="31"/>
       <c r="J26" s="30" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="K26" s="31" t="s">
-        <v>131</v>
-      </c>
-      <c r="L26" s="61">
+        <v>249</v>
+      </c>
+      <c r="L26" s="54">
         <v>1</v>
       </c>
       <c r="M26" s="32">
         <f>L26*5</f>
         <v>5</v>
       </c>
-      <c r="N26" s="31"/>
+      <c r="N26" s="31">
+        <v>10</v>
+      </c>
       <c r="O26" s="30">
         <v>10</v>
       </c>
-      <c r="P26" s="85"/>
-      <c r="Q26" s="51" t="s">
-        <v>251</v>
-      </c>
-      <c r="R26" s="35"/>
-      <c r="S26" s="35"/>
-      <c r="T26" s="35"/>
-      <c r="U26" s="35"/>
+      <c r="P26" s="77">
+        <v>10</v>
+      </c>
+      <c r="Q26" s="82" t="s">
+        <v>247</v>
+      </c>
+      <c r="R26" s="35">
+        <v>4.9399999999999999E-2</v>
+      </c>
+      <c r="S26" s="35">
+        <v>0.49</v>
+      </c>
+      <c r="T26" s="35">
+        <v>4.9399999999999999E-2</v>
+      </c>
+      <c r="U26" s="35">
+        <v>0.49</v>
+      </c>
       <c r="V26" s="32"/>
     </row>
     <row r="27" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -3179,12 +3426,12 @@
         <v>18</v>
       </c>
       <c r="C27" s="33" t="s">
-        <v>229</v>
+        <v>225</v>
       </c>
       <c r="D27" s="34" t="s">
         <v>29</v>
       </c>
-      <c r="E27" s="55" t="s">
+      <c r="E27" s="48" t="s">
         <v>67</v>
       </c>
       <c r="F27" s="33" t="s">
@@ -3198,31 +3445,43 @@
       </c>
       <c r="I27" s="34"/>
       <c r="J27" s="33" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="K27" s="34" t="s">
-        <v>132</v>
+        <v>249</v>
       </c>
       <c r="L27" s="33">
         <v>1</v>
       </c>
-      <c r="M27" s="58">
-        <f t="shared" ref="M27" si="9">L27*5</f>
+      <c r="M27" s="51">
+        <f t="shared" ref="M27" si="8">L27*5</f>
         <v>5</v>
       </c>
-      <c r="N27" s="34"/>
+      <c r="N27" s="34">
+        <v>10</v>
+      </c>
       <c r="O27" s="33">
         <v>10</v>
       </c>
-      <c r="P27" s="84"/>
-      <c r="Q27" s="52" t="s">
-        <v>251</v>
-      </c>
-      <c r="R27" s="36"/>
-      <c r="S27" s="36"/>
-      <c r="T27" s="36"/>
-      <c r="U27" s="36"/>
-      <c r="V27" s="58"/>
+      <c r="P27" s="76">
+        <v>10</v>
+      </c>
+      <c r="Q27" s="83" t="s">
+        <v>247</v>
+      </c>
+      <c r="R27" s="36">
+        <v>4.0599999999999997E-2</v>
+      </c>
+      <c r="S27" s="36">
+        <v>0.41</v>
+      </c>
+      <c r="T27" s="36">
+        <v>4.0599999999999997E-2</v>
+      </c>
+      <c r="U27" s="36">
+        <v>0.41</v>
+      </c>
+      <c r="V27" s="51"/>
     </row>
     <row r="28" spans="1:22" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="1"/>
@@ -3236,7 +3495,7 @@
       <c r="D28" s="31" t="s">
         <v>30</v>
       </c>
-      <c r="E28" s="63" t="s">
+      <c r="E28" s="55" t="s">
         <v>68</v>
       </c>
       <c r="F28" s="30" t="s">
@@ -3250,30 +3509,42 @@
       </c>
       <c r="I28" s="31"/>
       <c r="J28" s="30" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="K28" s="31" t="s">
-        <v>212</v>
-      </c>
-      <c r="L28" s="61">
+        <v>208</v>
+      </c>
+      <c r="L28" s="54">
         <v>1</v>
       </c>
       <c r="M28" s="32">
         <f>L28*5</f>
         <v>5</v>
       </c>
-      <c r="N28" s="31"/>
+      <c r="N28" s="31">
+        <v>5</v>
+      </c>
       <c r="O28" s="30">
         <v>10</v>
       </c>
-      <c r="P28" s="85"/>
-      <c r="Q28" s="51" t="s">
-        <v>251</v>
-      </c>
-      <c r="R28" s="35"/>
-      <c r="S28" s="35"/>
-      <c r="T28" s="35"/>
-      <c r="U28" s="35"/>
+      <c r="P28" s="77">
+        <v>10</v>
+      </c>
+      <c r="Q28" s="82" t="s">
+        <v>247</v>
+      </c>
+      <c r="R28" s="35">
+        <v>0.26819999999999999</v>
+      </c>
+      <c r="S28" s="35">
+        <v>1.34</v>
+      </c>
+      <c r="T28" s="35">
+        <v>0.26819999999999999</v>
+      </c>
+      <c r="U28" s="35">
+        <v>2.68</v>
+      </c>
       <c r="V28" s="32"/>
     </row>
     <row r="29" spans="1:22" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -3283,12 +3554,12 @@
         <v>20</v>
       </c>
       <c r="C29" s="33" t="s">
-        <v>230</v>
+        <v>226</v>
       </c>
       <c r="D29" s="34" t="s">
         <v>31</v>
       </c>
-      <c r="E29" s="55" t="s">
+      <c r="E29" s="48" t="s">
         <v>69</v>
       </c>
       <c r="F29" s="33" t="s">
@@ -3302,31 +3573,43 @@
       </c>
       <c r="I29" s="34"/>
       <c r="J29" s="33" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="K29" s="34" t="s">
-        <v>213</v>
+        <v>209</v>
       </c>
       <c r="L29" s="33">
         <v>2</v>
       </c>
-      <c r="M29" s="58">
-        <f t="shared" ref="M29" si="10">L29*5</f>
+      <c r="M29" s="51">
+        <f t="shared" ref="M29" si="9">L29*5</f>
         <v>10</v>
       </c>
-      <c r="N29" s="34"/>
+      <c r="N29" s="34">
+        <v>10</v>
+      </c>
       <c r="O29" s="33">
         <v>20</v>
       </c>
-      <c r="P29" s="84"/>
-      <c r="Q29" s="52" t="s">
-        <v>251</v>
-      </c>
-      <c r="R29" s="36"/>
-      <c r="S29" s="36"/>
-      <c r="T29" s="36"/>
-      <c r="U29" s="36"/>
-      <c r="V29" s="58"/>
+      <c r="P29" s="76">
+        <v>20</v>
+      </c>
+      <c r="Q29" s="83" t="s">
+        <v>247</v>
+      </c>
+      <c r="R29" s="36">
+        <v>7.3200000000000001E-2</v>
+      </c>
+      <c r="S29" s="36">
+        <v>0.73</v>
+      </c>
+      <c r="T29" s="36">
+        <v>7.3200000000000001E-2</v>
+      </c>
+      <c r="U29" s="36">
+        <v>1.46</v>
+      </c>
+      <c r="V29" s="51"/>
     </row>
     <row r="30" spans="1:22" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="1"/>
@@ -3335,139 +3618,189 @@
         <v>21</v>
       </c>
       <c r="C30" s="30" t="s">
-        <v>231</v>
+        <v>10</v>
       </c>
       <c r="D30" s="31" t="s">
-        <v>32</v>
-      </c>
-      <c r="E30" s="63"/>
+        <v>36</v>
+      </c>
+      <c r="E30" s="55" t="s">
+        <v>73</v>
+      </c>
       <c r="F30" s="30" t="s">
-        <v>102</v>
-      </c>
-      <c r="G30" s="31"/>
-      <c r="H30" s="30"/>
+        <v>106</v>
+      </c>
+      <c r="G30" s="31" t="s">
+        <v>134</v>
+      </c>
+      <c r="H30" s="30" t="s">
+        <v>161</v>
+      </c>
       <c r="I30" s="31"/>
-      <c r="J30" s="30"/>
+      <c r="J30" s="30" t="s">
+        <v>189</v>
+      </c>
       <c r="K30" s="31" t="s">
-        <v>214</v>
-      </c>
-      <c r="L30" s="61">
-        <v>5</v>
+        <v>249</v>
+      </c>
+      <c r="L30" s="54">
+        <v>6</v>
       </c>
       <c r="M30" s="32">
         <f>L30*5</f>
-        <v>25</v>
-      </c>
-      <c r="N30" s="31"/>
+        <v>30</v>
+      </c>
+      <c r="N30" s="31">
+        <v>30</v>
+      </c>
       <c r="O30" s="30">
-        <v>50</v>
-      </c>
-      <c r="P30" s="85"/>
-      <c r="Q30" s="51" t="s">
-        <v>251</v>
-      </c>
-      <c r="R30" s="35"/>
-      <c r="S30" s="35"/>
-      <c r="T30" s="35"/>
-      <c r="U30" s="35"/>
+        <v>60</v>
+      </c>
+      <c r="P30" s="77">
+        <v>60</v>
+      </c>
+      <c r="Q30" s="82" t="s">
+        <v>247</v>
+      </c>
+      <c r="R30" s="35">
+        <v>0.1668</v>
+      </c>
+      <c r="S30" s="35">
+        <v>5</v>
+      </c>
+      <c r="T30" s="35">
+        <v>0.13439999999999999</v>
+      </c>
+      <c r="U30" s="35">
+        <v>8.06</v>
+      </c>
       <c r="V30" s="32"/>
     </row>
-    <row r="31" spans="1:22" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="1"/>
       <c r="B31" s="26">
-        <f>ROW(B31) - ROW($B$9)</f>
+        <f t="shared" si="0"/>
         <v>22</v>
       </c>
       <c r="C31" s="33" t="s">
-        <v>232</v>
+        <v>11</v>
       </c>
       <c r="D31" s="34" t="s">
-        <v>34</v>
-      </c>
-      <c r="E31" s="55" t="s">
-        <v>71</v>
+        <v>37</v>
+      </c>
+      <c r="E31" s="48" t="s">
+        <v>74</v>
       </c>
       <c r="F31" s="33" t="s">
-        <v>104</v>
-      </c>
-      <c r="G31" s="34"/>
-      <c r="H31" s="33"/>
+        <v>107</v>
+      </c>
+      <c r="G31" s="34" t="s">
+        <v>135</v>
+      </c>
+      <c r="H31" s="33" t="s">
+        <v>151</v>
+      </c>
       <c r="I31" s="34"/>
-      <c r="J31" s="33"/>
+      <c r="J31" s="33" t="s">
+        <v>190</v>
+      </c>
       <c r="K31" s="34" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="L31" s="33">
+        <v>2</v>
+      </c>
+      <c r="M31" s="51">
+        <f t="shared" ref="M31" si="10">L31*5</f>
         <v>10</v>
       </c>
-      <c r="M31" s="58">
-        <f>L31*5</f>
-        <v>50</v>
-      </c>
-      <c r="N31" s="34"/>
+      <c r="N31" s="34">
+        <v>100</v>
+      </c>
       <c r="O31" s="33">
+        <v>20</v>
+      </c>
+      <c r="P31" s="76">
         <v>100</v>
       </c>
-      <c r="P31" s="84"/>
-      <c r="Q31" s="52" t="s">
-        <v>251</v>
-      </c>
-      <c r="R31" s="33"/>
-      <c r="S31" s="33"/>
-      <c r="T31" s="33"/>
-      <c r="U31" s="33"/>
-      <c r="V31" s="58"/>
+      <c r="Q31" s="83" t="s">
+        <v>247</v>
+      </c>
+      <c r="R31" s="36">
+        <v>1E-3</v>
+      </c>
+      <c r="S31" s="36">
+        <v>0.1</v>
+      </c>
+      <c r="T31" s="36">
+        <v>1E-3</v>
+      </c>
+      <c r="U31" s="36">
+        <v>0.1</v>
+      </c>
+      <c r="V31" s="51"/>
     </row>
-    <row r="32" spans="1:22" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="1"/>
       <c r="B32" s="26">
         <f>ROW(B32) - ROW($B$9)</f>
         <v>23</v>
       </c>
-      <c r="C32" s="30" t="s">
-        <v>10</v>
+      <c r="C32" s="54" t="s">
+        <v>11</v>
       </c>
       <c r="D32" s="31" t="s">
-        <v>36</v>
-      </c>
-      <c r="E32" s="63" t="s">
-        <v>73</v>
+        <v>38</v>
+      </c>
+      <c r="E32" s="55" t="s">
+        <v>75</v>
       </c>
       <c r="F32" s="30" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="G32" s="31" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="H32" s="30" t="s">
-        <v>161</v>
+        <v>151</v>
       </c>
       <c r="I32" s="31"/>
       <c r="J32" s="30" t="s">
         <v>191</v>
       </c>
       <c r="K32" s="31" t="s">
-        <v>134</v>
-      </c>
-      <c r="L32" s="61">
-        <v>6</v>
+        <v>213</v>
+      </c>
+      <c r="L32" s="54">
+        <v>3</v>
       </c>
       <c r="M32" s="32">
         <f>L32*5</f>
+        <v>15</v>
+      </c>
+      <c r="N32" s="31">
+        <v>100</v>
+      </c>
+      <c r="O32" s="30">
         <v>30</v>
       </c>
-      <c r="N32" s="31"/>
-      <c r="O32" s="30">
-        <v>60</v>
-      </c>
-      <c r="P32" s="85"/>
-      <c r="Q32" s="51" t="s">
-        <v>251</v>
-      </c>
-      <c r="R32" s="35"/>
-      <c r="S32" s="35"/>
-      <c r="T32" s="35"/>
-      <c r="U32" s="35"/>
+      <c r="P32" s="77">
+        <v>100</v>
+      </c>
+      <c r="Q32" s="82" t="s">
+        <v>247</v>
+      </c>
+      <c r="R32" s="35">
+        <v>1.5E-3</v>
+      </c>
+      <c r="S32" s="35">
+        <v>0.15</v>
+      </c>
+      <c r="T32" s="35">
+        <v>1.5E-3</v>
+      </c>
+      <c r="U32" s="35">
+        <v>0.15</v>
+      </c>
       <c r="V32" s="32"/>
     </row>
     <row r="33" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -3480,47 +3813,61 @@
         <v>11</v>
       </c>
       <c r="D33" s="34" t="s">
-        <v>37</v>
-      </c>
-      <c r="E33" s="55" t="s">
-        <v>74</v>
+        <v>39</v>
+      </c>
+      <c r="E33" s="48" t="s">
+        <v>76</v>
       </c>
       <c r="F33" s="33" t="s">
-        <v>107</v>
-      </c>
-      <c r="G33" s="34" t="s">
-        <v>135</v>
+        <v>109</v>
+      </c>
+      <c r="G33" s="92" t="s">
+        <v>137</v>
       </c>
       <c r="H33" s="33" t="s">
-        <v>151</v>
-      </c>
-      <c r="I33" s="34"/>
+        <v>162</v>
+      </c>
+      <c r="I33" s="33" t="s">
+        <v>258</v>
+      </c>
       <c r="J33" s="33" t="s">
-        <v>192</v>
-      </c>
-      <c r="K33" s="34" t="s">
-        <v>216</v>
+        <v>257</v>
+      </c>
+      <c r="K33" s="33" t="s">
+        <v>214</v>
       </c>
       <c r="L33" s="33">
-        <v>2</v>
-      </c>
-      <c r="M33" s="58">
+        <v>6</v>
+      </c>
+      <c r="M33" s="33">
         <f t="shared" ref="M33" si="11">L33*5</f>
-        <v>10</v>
-      </c>
-      <c r="N33" s="34"/>
+        <v>30</v>
+      </c>
+      <c r="N33" s="33">
+        <v>40</v>
+      </c>
       <c r="O33" s="33">
-        <v>20</v>
-      </c>
-      <c r="P33" s="84"/>
-      <c r="Q33" s="52" t="s">
-        <v>251</v>
-      </c>
-      <c r="R33" s="36"/>
-      <c r="S33" s="36"/>
-      <c r="T33" s="36"/>
-      <c r="U33" s="36"/>
-      <c r="V33" s="58"/>
+        <v>60</v>
+      </c>
+      <c r="P33" s="33">
+        <v>60</v>
+      </c>
+      <c r="Q33" s="83" t="s">
+        <v>247</v>
+      </c>
+      <c r="R33" s="36">
+        <v>3.1600000000000003E-2</v>
+      </c>
+      <c r="S33" s="36">
+        <v>1.26</v>
+      </c>
+      <c r="T33" s="36">
+        <v>3.1600000000000003E-2</v>
+      </c>
+      <c r="U33" s="36">
+        <v>1.9</v>
+      </c>
+      <c r="V33" s="51"/>
     </row>
     <row r="34" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="1"/>
@@ -3528,50 +3875,64 @@
         <f>ROW(B34) - ROW($B$9)</f>
         <v>25</v>
       </c>
-      <c r="C34" s="61" t="s">
+      <c r="C34" s="54" t="s">
         <v>11</v>
       </c>
       <c r="D34" s="31" t="s">
-        <v>38</v>
-      </c>
-      <c r="E34" s="63" t="s">
-        <v>75</v>
+        <v>40</v>
+      </c>
+      <c r="E34" s="55" t="s">
+        <v>77</v>
       </c>
       <c r="F34" s="30" t="s">
-        <v>108</v>
-      </c>
-      <c r="G34" s="31" t="s">
-        <v>136</v>
+        <v>109</v>
+      </c>
+      <c r="G34" s="91" t="s">
+        <v>138</v>
       </c>
       <c r="H34" s="30" t="s">
-        <v>151</v>
-      </c>
-      <c r="I34" s="31"/>
+        <v>163</v>
+      </c>
+      <c r="I34" s="31" t="s">
+        <v>259</v>
+      </c>
       <c r="J34" s="30" t="s">
-        <v>193</v>
+        <v>260</v>
       </c>
       <c r="K34" s="31" t="s">
-        <v>217</v>
-      </c>
-      <c r="L34" s="61">
-        <v>3</v>
+        <v>215</v>
+      </c>
+      <c r="L34" s="54">
+        <v>4</v>
       </c>
       <c r="M34" s="32">
         <f>L34*5</f>
-        <v>15</v>
-      </c>
-      <c r="N34" s="31"/>
+        <v>20</v>
+      </c>
+      <c r="N34" s="31">
+        <v>100</v>
+      </c>
       <c r="O34" s="30">
-        <v>30</v>
-      </c>
-      <c r="P34" s="85"/>
-      <c r="Q34" s="51" t="s">
-        <v>251</v>
-      </c>
-      <c r="R34" s="35"/>
-      <c r="S34" s="35"/>
-      <c r="T34" s="35"/>
-      <c r="U34" s="35"/>
+        <v>40</v>
+      </c>
+      <c r="P34" s="77">
+        <v>100</v>
+      </c>
+      <c r="Q34" s="82" t="s">
+        <v>247</v>
+      </c>
+      <c r="R34" s="35">
+        <v>1.6999999999999999E-3</v>
+      </c>
+      <c r="S34" s="35">
+        <v>0.17</v>
+      </c>
+      <c r="T34" s="35">
+        <v>1.6999999999999999E-3</v>
+      </c>
+      <c r="U34" s="35">
+        <v>0.17</v>
+      </c>
       <c r="V34" s="32"/>
     </row>
     <row r="35" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -3584,98 +3945,122 @@
         <v>11</v>
       </c>
       <c r="D35" s="34" t="s">
-        <v>39</v>
-      </c>
-      <c r="E35" s="55" t="s">
-        <v>76</v>
+        <v>41</v>
+      </c>
+      <c r="E35" s="48" t="s">
+        <v>78</v>
       </c>
       <c r="F35" s="33" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="G35" s="34" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="H35" s="33" t="s">
-        <v>162</v>
-      </c>
-      <c r="I35" s="34"/>
+        <v>164</v>
+      </c>
+      <c r="I35" s="33"/>
       <c r="J35" s="33" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="K35" s="34" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="L35" s="33">
-        <v>6</v>
-      </c>
-      <c r="M35" s="58">
+        <v>3</v>
+      </c>
+      <c r="M35" s="51">
         <f t="shared" ref="M35" si="12">L35*5</f>
+        <v>15</v>
+      </c>
+      <c r="N35" s="34">
+        <v>20</v>
+      </c>
+      <c r="O35" s="33">
         <v>30</v>
       </c>
-      <c r="N35" s="34"/>
-      <c r="O35" s="33">
-        <v>60</v>
-      </c>
-      <c r="P35" s="84"/>
-      <c r="Q35" s="52" t="s">
-        <v>251</v>
-      </c>
-      <c r="R35" s="36"/>
-      <c r="S35" s="36"/>
-      <c r="T35" s="36"/>
-      <c r="U35" s="36"/>
-      <c r="V35" s="58"/>
+      <c r="P35" s="76">
+        <v>40</v>
+      </c>
+      <c r="Q35" s="83" t="s">
+        <v>247</v>
+      </c>
+      <c r="R35" s="36">
+        <v>2.7900000000000001E-2</v>
+      </c>
+      <c r="S35" s="36">
+        <v>0.56000000000000005</v>
+      </c>
+      <c r="T35" s="36">
+        <v>2.7900000000000001E-2</v>
+      </c>
+      <c r="U35" s="36">
+        <v>1.1200000000000001</v>
+      </c>
+      <c r="V35" s="51"/>
     </row>
-    <row r="36" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:22" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A36" s="1"/>
       <c r="B36" s="26">
         <f>ROW(B36) - ROW($B$9)</f>
         <v>27</v>
       </c>
-      <c r="C36" s="61" t="s">
+      <c r="C36" s="30" t="s">
         <v>11</v>
       </c>
       <c r="D36" s="31" t="s">
-        <v>40</v>
-      </c>
-      <c r="E36" s="63" t="s">
-        <v>77</v>
+        <v>42</v>
+      </c>
+      <c r="E36" s="55" t="s">
+        <v>79</v>
       </c>
       <c r="F36" s="30" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="G36" s="31" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="H36" s="30" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="I36" s="31"/>
       <c r="J36" s="30" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="K36" s="31" t="s">
-        <v>219</v>
-      </c>
-      <c r="L36" s="61">
-        <v>4</v>
+        <v>217</v>
+      </c>
+      <c r="L36" s="54">
+        <v>3</v>
       </c>
       <c r="M36" s="32">
         <f>L36*5</f>
-        <v>20</v>
-      </c>
-      <c r="N36" s="31"/>
+        <v>15</v>
+      </c>
+      <c r="N36" s="31">
+        <v>50</v>
+      </c>
       <c r="O36" s="30">
-        <v>40</v>
-      </c>
-      <c r="P36" s="85"/>
-      <c r="Q36" s="51" t="s">
-        <v>251</v>
-      </c>
-      <c r="R36" s="35"/>
-      <c r="S36" s="35"/>
-      <c r="T36" s="35"/>
-      <c r="U36" s="35"/>
+        <v>30</v>
+      </c>
+      <c r="P36" s="77">
+        <v>50</v>
+      </c>
+      <c r="Q36" s="82" t="s">
+        <v>247</v>
+      </c>
+      <c r="R36" s="35">
+        <v>7.1999999999999998E-3</v>
+      </c>
+      <c r="S36" s="35">
+        <v>0.36</v>
+      </c>
+      <c r="T36" s="35">
+        <v>7.1999999999999998E-3</v>
+      </c>
+      <c r="U36" s="35">
+        <v>0.36</v>
+      </c>
       <c r="V36" s="32"/>
     </row>
     <row r="37" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -3688,49 +4073,61 @@
         <v>11</v>
       </c>
       <c r="D37" s="34" t="s">
-        <v>41</v>
-      </c>
-      <c r="E37" s="55" t="s">
-        <v>78</v>
+        <v>43</v>
+      </c>
+      <c r="E37" s="48" t="s">
+        <v>80</v>
       </c>
       <c r="F37" s="33" t="s">
         <v>107</v>
       </c>
       <c r="G37" s="34" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="H37" s="33" t="s">
-        <v>164</v>
+        <v>151</v>
       </c>
       <c r="I37" s="34"/>
       <c r="J37" s="33" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="K37" s="34" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="L37" s="33">
-        <v>3</v>
-      </c>
-      <c r="M37" s="58">
+        <v>1</v>
+      </c>
+      <c r="M37" s="51">
         <f t="shared" ref="M37" si="13">L37*5</f>
-        <v>15</v>
-      </c>
-      <c r="N37" s="34"/>
+        <v>5</v>
+      </c>
+      <c r="N37" s="34">
+        <v>50</v>
+      </c>
       <c r="O37" s="33">
-        <v>30</v>
-      </c>
-      <c r="P37" s="84"/>
-      <c r="Q37" s="52" t="s">
-        <v>251</v>
-      </c>
-      <c r="R37" s="36"/>
-      <c r="S37" s="36"/>
-      <c r="T37" s="36"/>
-      <c r="U37" s="36"/>
-      <c r="V37" s="58"/>
+        <v>10</v>
+      </c>
+      <c r="P37" s="76">
+        <v>50</v>
+      </c>
+      <c r="Q37" s="83" t="s">
+        <v>247</v>
+      </c>
+      <c r="R37" s="36">
+        <v>1.1599999999999999E-2</v>
+      </c>
+      <c r="S37" s="36">
+        <v>0.57999999999999996</v>
+      </c>
+      <c r="T37" s="36">
+        <v>1.1599999999999999E-2</v>
+      </c>
+      <c r="U37" s="36">
+        <v>0.57999999999999996</v>
+      </c>
+      <c r="V37" s="51"/>
     </row>
-    <row r="38" spans="1:22" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A38" s="1"/>
       <c r="B38" s="26">
         <f>ROW(B38) - ROW($B$9)</f>
@@ -3740,49 +4137,63 @@
         <v>11</v>
       </c>
       <c r="D38" s="31" t="s">
-        <v>42</v>
-      </c>
-      <c r="E38" s="63" t="s">
-        <v>79</v>
+        <v>44</v>
+      </c>
+      <c r="E38" s="55" t="s">
+        <v>81</v>
       </c>
       <c r="F38" s="30" t="s">
-        <v>107</v>
-      </c>
-      <c r="G38" s="31" t="s">
-        <v>140</v>
+        <v>110</v>
+      </c>
+      <c r="G38" s="91" t="s">
+        <v>142</v>
       </c>
       <c r="H38" s="30" t="s">
-        <v>165</v>
-      </c>
-      <c r="I38" s="31"/>
+        <v>166</v>
+      </c>
+      <c r="I38" s="31" t="s">
+        <v>261</v>
+      </c>
       <c r="J38" s="30" t="s">
-        <v>197</v>
+        <v>262</v>
       </c>
       <c r="K38" s="31" t="s">
-        <v>221</v>
-      </c>
-      <c r="L38" s="61">
-        <v>3</v>
+        <v>219</v>
+      </c>
+      <c r="L38" s="54">
+        <v>1</v>
       </c>
       <c r="M38" s="32">
         <f>L38*5</f>
-        <v>15</v>
-      </c>
-      <c r="N38" s="31"/>
+        <v>5</v>
+      </c>
+      <c r="N38" s="31">
+        <v>100</v>
+      </c>
       <c r="O38" s="30">
-        <v>30</v>
-      </c>
-      <c r="P38" s="85"/>
-      <c r="Q38" s="51" t="s">
-        <v>251</v>
-      </c>
-      <c r="R38" s="35"/>
-      <c r="S38" s="35"/>
-      <c r="T38" s="35"/>
-      <c r="U38" s="35"/>
+        <v>10</v>
+      </c>
+      <c r="P38" s="77">
+        <v>100</v>
+      </c>
+      <c r="Q38" s="82" t="s">
+        <v>247</v>
+      </c>
+      <c r="R38" s="35">
+        <v>5.9999999999999995E-4</v>
+      </c>
+      <c r="S38" s="35">
+        <v>0.06</v>
+      </c>
+      <c r="T38" s="35">
+        <v>5.9999999999999995E-4</v>
+      </c>
+      <c r="U38" s="35">
+        <v>0.06</v>
+      </c>
       <c r="V38" s="32"/>
     </row>
-    <row r="39" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:22" ht="36.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A39" s="1"/>
       <c r="B39" s="26">
         <f t="shared" si="0"/>
@@ -3792,47 +4203,59 @@
         <v>11</v>
       </c>
       <c r="D39" s="34" t="s">
-        <v>43</v>
-      </c>
-      <c r="E39" s="55" t="s">
-        <v>80</v>
+        <v>45</v>
+      </c>
+      <c r="E39" s="48" t="s">
+        <v>82</v>
       </c>
       <c r="F39" s="33" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="G39" s="34" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="H39" s="33" t="s">
-        <v>151</v>
+        <v>167</v>
       </c>
       <c r="I39" s="34"/>
       <c r="J39" s="33" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="K39" s="34" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="L39" s="33">
         <v>1</v>
       </c>
-      <c r="M39" s="58">
+      <c r="M39" s="51">
         <f t="shared" ref="M39" si="14">L39*5</f>
         <v>5</v>
       </c>
-      <c r="N39" s="34"/>
+      <c r="N39" s="34">
+        <v>10</v>
+      </c>
       <c r="O39" s="33">
         <v>10</v>
       </c>
-      <c r="P39" s="84"/>
-      <c r="Q39" s="52" t="s">
-        <v>251</v>
-      </c>
-      <c r="R39" s="36"/>
-      <c r="S39" s="36"/>
-      <c r="T39" s="36"/>
-      <c r="U39" s="36"/>
-      <c r="V39" s="58"/>
+      <c r="P39" s="76">
+        <v>10</v>
+      </c>
+      <c r="Q39" s="83" t="s">
+        <v>247</v>
+      </c>
+      <c r="R39" s="36">
+        <v>6.4399999999999999E-2</v>
+      </c>
+      <c r="S39" s="36">
+        <v>0.64</v>
+      </c>
+      <c r="T39" s="36">
+        <v>6.4399999999999999E-2</v>
+      </c>
+      <c r="U39" s="36">
+        <v>0.64</v>
+      </c>
+      <c r="V39" s="51"/>
     </row>
     <row r="40" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A40" s="1"/>
@@ -3844,95 +4267,122 @@
         <v>11</v>
       </c>
       <c r="D40" s="31" t="s">
-        <v>44</v>
-      </c>
-      <c r="E40" s="63" t="s">
-        <v>81</v>
+        <v>46</v>
+      </c>
+      <c r="E40" s="55" t="s">
+        <v>83</v>
       </c>
       <c r="F40" s="30" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="G40" s="31" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="H40" s="30" t="s">
-        <v>166</v>
+        <v>151</v>
       </c>
       <c r="I40" s="31"/>
-      <c r="J40" s="30"/>
+      <c r="J40" s="30" t="s">
+        <v>196</v>
+      </c>
       <c r="K40" s="31" t="s">
-        <v>223</v>
-      </c>
-      <c r="L40" s="61">
+        <v>221</v>
+      </c>
+      <c r="L40" s="54">
         <v>1</v>
       </c>
       <c r="M40" s="32">
         <f>L40*5</f>
         <v>5</v>
       </c>
-      <c r="N40" s="31"/>
+      <c r="N40" s="31">
+        <v>100</v>
+      </c>
       <c r="O40" s="30">
         <v>10</v>
       </c>
-      <c r="P40" s="85"/>
-      <c r="Q40" s="51" t="s">
-        <v>251</v>
-      </c>
-      <c r="R40" s="35"/>
-      <c r="S40" s="35"/>
-      <c r="T40" s="35"/>
-      <c r="U40" s="35"/>
+      <c r="P40" s="77">
+        <v>100</v>
+      </c>
+      <c r="Q40" s="82" t="s">
+        <v>247</v>
+      </c>
+      <c r="R40" s="35">
+        <v>1.1999999999999999E-3</v>
+      </c>
+      <c r="S40" s="35">
+        <v>0.12</v>
+      </c>
+      <c r="T40" s="35">
+        <v>1.1999999999999999E-3</v>
+      </c>
+      <c r="U40" s="35">
+        <v>0.12</v>
+      </c>
       <c r="V40" s="32"/>
     </row>
-    <row r="41" spans="1:22" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A41" s="1"/>
       <c r="B41" s="26">
         <f t="shared" si="0"/>
         <v>32</v>
       </c>
       <c r="C41" s="33" t="s">
-        <v>11</v>
+        <v>112</v>
       </c>
       <c r="D41" s="34" t="s">
-        <v>45</v>
-      </c>
-      <c r="E41" s="55" t="s">
-        <v>82</v>
+        <v>47</v>
+      </c>
+      <c r="E41" s="48" t="s">
+        <v>84</v>
       </c>
       <c r="F41" s="33" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="G41" s="34" t="s">
-        <v>143</v>
+        <v>249</v>
       </c>
       <c r="H41" s="33" t="s">
-        <v>167</v>
+        <v>249</v>
       </c>
       <c r="I41" s="34"/>
       <c r="J41" s="33" t="s">
-        <v>199</v>
+        <v>249</v>
       </c>
       <c r="K41" s="34" t="s">
-        <v>224</v>
-      </c>
-      <c r="L41" s="33">
-        <v>1</v>
-      </c>
-      <c r="M41" s="58">
-        <f t="shared" ref="M41" si="15">L41*5</f>
-        <v>5</v>
-      </c>
-      <c r="N41" s="34"/>
-      <c r="O41" s="33"/>
-      <c r="P41" s="84"/>
-      <c r="Q41" s="52" t="s">
-        <v>251</v>
-      </c>
-      <c r="R41" s="36"/>
-      <c r="S41" s="36"/>
-      <c r="T41" s="36"/>
-      <c r="U41" s="36"/>
-      <c r="V41" s="58"/>
+        <v>112</v>
+      </c>
+      <c r="L41" s="33" t="s">
+        <v>249</v>
+      </c>
+      <c r="M41" s="51" t="s">
+        <v>249</v>
+      </c>
+      <c r="N41" s="34" t="s">
+        <v>249</v>
+      </c>
+      <c r="O41" s="33" t="s">
+        <v>249</v>
+      </c>
+      <c r="P41" s="76" t="s">
+        <v>249</v>
+      </c>
+      <c r="Q41" s="45" t="s">
+        <v>249</v>
+      </c>
+      <c r="R41" s="36" t="s">
+        <v>249</v>
+      </c>
+      <c r="S41" s="36" t="s">
+        <v>249</v>
+      </c>
+      <c r="T41" s="36" t="s">
+        <v>249</v>
+      </c>
+      <c r="U41" s="36" t="s">
+        <v>249</v>
+      </c>
+      <c r="V41" s="51"/>
     </row>
     <row r="42" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A42" s="1"/>
@@ -3941,106 +4391,138 @@
         <v>33</v>
       </c>
       <c r="C42" s="30" t="s">
-        <v>11</v>
+        <v>227</v>
       </c>
       <c r="D42" s="31" t="s">
-        <v>46</v>
-      </c>
-      <c r="E42" s="63" t="s">
-        <v>83</v>
+        <v>32</v>
+      </c>
+      <c r="E42" s="55" t="s">
+        <v>248</v>
       </c>
       <c r="F42" s="30" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="G42" s="31" t="s">
-        <v>144</v>
+        <v>249</v>
       </c>
       <c r="H42" s="30" t="s">
-        <v>151</v>
+        <v>249</v>
       </c>
       <c r="I42" s="31"/>
       <c r="J42" s="30" t="s">
-        <v>200</v>
+        <v>249</v>
       </c>
       <c r="K42" s="31" t="s">
-        <v>225</v>
-      </c>
-      <c r="L42" s="61">
-        <v>1</v>
-      </c>
-      <c r="M42" s="32">
-        <f>L42*5</f>
-        <v>5</v>
-      </c>
-      <c r="N42" s="31"/>
-      <c r="O42" s="30"/>
-      <c r="P42" s="85"/>
-      <c r="Q42" s="51" t="s">
-        <v>251</v>
-      </c>
-      <c r="R42" s="35"/>
-      <c r="S42" s="35"/>
-      <c r="T42" s="35"/>
-      <c r="U42" s="35"/>
+        <v>210</v>
+      </c>
+      <c r="L42" s="54" t="s">
+        <v>249</v>
+      </c>
+      <c r="M42" s="32" t="s">
+        <v>249</v>
+      </c>
+      <c r="N42" s="31" t="s">
+        <v>249</v>
+      </c>
+      <c r="O42" s="30" t="s">
+        <v>249</v>
+      </c>
+      <c r="P42" s="77" t="s">
+        <v>249</v>
+      </c>
+      <c r="Q42" s="44" t="s">
+        <v>249</v>
+      </c>
+      <c r="R42" s="35" t="s">
+        <v>249</v>
+      </c>
+      <c r="S42" s="35" t="s">
+        <v>249</v>
+      </c>
+      <c r="T42" s="35" t="s">
+        <v>249</v>
+      </c>
+      <c r="U42" s="35" t="s">
+        <v>249</v>
+      </c>
       <c r="V42" s="32"/>
     </row>
-    <row r="43" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:22" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A43" s="1"/>
       <c r="B43" s="26">
-        <f t="shared" si="0"/>
+        <f>ROW(B43) - ROW($B$9)</f>
         <v>34</v>
       </c>
       <c r="C43" s="33" t="s">
-        <v>112</v>
+        <v>228</v>
       </c>
       <c r="D43" s="34" t="s">
-        <v>47</v>
-      </c>
-      <c r="E43" s="55" t="s">
-        <v>84</v>
+        <v>34</v>
+      </c>
+      <c r="E43" s="48" t="s">
+        <v>71</v>
       </c>
       <c r="F43" s="33" t="s">
-        <v>112</v>
-      </c>
-      <c r="G43" s="34"/>
-      <c r="H43" s="33"/>
+        <v>104</v>
+      </c>
+      <c r="G43" s="34" t="s">
+        <v>249</v>
+      </c>
+      <c r="H43" s="33" t="s">
+        <v>249</v>
+      </c>
       <c r="I43" s="34"/>
-      <c r="J43" s="33"/>
+      <c r="J43" s="33" t="s">
+        <v>249</v>
+      </c>
       <c r="K43" s="34" t="s">
-        <v>112</v>
-      </c>
-      <c r="L43" s="33">
-        <v>1</v>
-      </c>
-      <c r="M43" s="58">
-        <f t="shared" ref="M43" si="16">L43*5</f>
-        <v>5</v>
-      </c>
-      <c r="N43" s="34"/>
-      <c r="O43" s="33"/>
-      <c r="P43" s="84"/>
-      <c r="Q43" s="52" t="s">
-        <v>251</v>
-      </c>
-      <c r="R43" s="36"/>
-      <c r="S43" s="36"/>
-      <c r="T43" s="36"/>
-      <c r="U43" s="36"/>
-      <c r="V43" s="58"/>
+        <v>211</v>
+      </c>
+      <c r="L43" s="33" t="s">
+        <v>249</v>
+      </c>
+      <c r="M43" s="51" t="s">
+        <v>249</v>
+      </c>
+      <c r="N43" s="34" t="s">
+        <v>249</v>
+      </c>
+      <c r="O43" s="33" t="s">
+        <v>249</v>
+      </c>
+      <c r="P43" s="76" t="s">
+        <v>249</v>
+      </c>
+      <c r="Q43" s="45" t="s">
+        <v>249</v>
+      </c>
+      <c r="R43" s="33" t="s">
+        <v>249</v>
+      </c>
+      <c r="S43" s="33" t="s">
+        <v>249</v>
+      </c>
+      <c r="T43" s="33" t="s">
+        <v>249</v>
+      </c>
+      <c r="U43" s="33" t="s">
+        <v>249</v>
+      </c>
+      <c r="V43" s="51"/>
     </row>
-    <row r="44" spans="1:22" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:22" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A44" s="1"/>
       <c r="B44" s="26">
         <f>ROW(B44) - ROW($B$9)</f>
         <v>35</v>
       </c>
       <c r="C44" s="30" t="s">
-        <v>233</v>
+        <v>229</v>
       </c>
       <c r="D44" s="31" t="s">
         <v>48</v>
       </c>
-      <c r="E44" s="63" t="s">
+      <c r="E44" s="55" t="s">
         <v>85</v>
       </c>
       <c r="F44" s="30" t="s">
@@ -4054,28 +4536,42 @@
       </c>
       <c r="I44" s="31"/>
       <c r="J44" s="30" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
       <c r="K44" s="31" t="s">
-        <v>145</v>
-      </c>
-      <c r="L44" s="61">
+        <v>249</v>
+      </c>
+      <c r="L44" s="54">
         <v>1</v>
       </c>
       <c r="M44" s="32">
         <f>L44*5</f>
         <v>5</v>
       </c>
-      <c r="N44" s="31"/>
-      <c r="O44" s="30"/>
-      <c r="P44" s="85"/>
-      <c r="Q44" s="51" t="s">
-        <v>251</v>
-      </c>
-      <c r="R44" s="35"/>
-      <c r="S44" s="35"/>
-      <c r="T44" s="35"/>
-      <c r="U44" s="35"/>
+      <c r="N44" s="31">
+        <v>10</v>
+      </c>
+      <c r="O44" s="30">
+        <v>10</v>
+      </c>
+      <c r="P44" s="77">
+        <v>10</v>
+      </c>
+      <c r="Q44" s="82" t="s">
+        <v>247</v>
+      </c>
+      <c r="R44" s="35">
+        <v>5.8200000000000002E-2</v>
+      </c>
+      <c r="S44" s="35">
+        <v>0.57999999999999996</v>
+      </c>
+      <c r="T44" s="35">
+        <v>5.8200000000000002E-2</v>
+      </c>
+      <c r="U44" s="35">
+        <v>0.57999999999999996</v>
+      </c>
       <c r="V44" s="32"/>
     </row>
     <row r="45" spans="1:22" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -4090,7 +4586,7 @@
       <c r="D45" s="34" t="s">
         <v>49</v>
       </c>
-      <c r="E45" s="55" t="s">
+      <c r="E45" s="48" t="s">
         <v>86</v>
       </c>
       <c r="F45" s="33" t="s">
@@ -4105,26 +4601,26 @@
       <c r="I45" s="34"/>
       <c r="J45" s="33"/>
       <c r="K45" s="34" t="s">
-        <v>146</v>
+        <v>249</v>
       </c>
       <c r="L45" s="33">
         <v>1</v>
       </c>
-      <c r="M45" s="58">
-        <f t="shared" ref="M45" si="17">L45*5</f>
+      <c r="M45" s="51">
+        <f t="shared" ref="M45" si="15">L45*5</f>
         <v>5</v>
       </c>
       <c r="N45" s="34"/>
       <c r="O45" s="33"/>
-      <c r="P45" s="84"/>
-      <c r="Q45" s="52" t="s">
-        <v>251</v>
+      <c r="P45" s="76"/>
+      <c r="Q45" s="45" t="s">
+        <v>247</v>
       </c>
       <c r="R45" s="36"/>
       <c r="S45" s="36"/>
       <c r="T45" s="36"/>
       <c r="U45" s="36"/>
-      <c r="V45" s="58"/>
+      <c r="V45" s="51"/>
     </row>
     <row r="46" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A46" s="1"/>
@@ -4138,7 +4634,7 @@
       <c r="D46" s="31" t="s">
         <v>50</v>
       </c>
-      <c r="E46" s="63" t="s">
+      <c r="E46" s="55" t="s">
         <v>87</v>
       </c>
       <c r="F46" s="30" t="s">
@@ -4152,28 +4648,42 @@
       </c>
       <c r="I46" s="31"/>
       <c r="J46" s="30" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
       <c r="K46" s="31" t="s">
-        <v>147</v>
-      </c>
-      <c r="L46" s="61">
+        <v>249</v>
+      </c>
+      <c r="L46" s="54">
         <v>1</v>
       </c>
       <c r="M46" s="32">
         <f>L46*5</f>
         <v>5</v>
       </c>
-      <c r="N46" s="31"/>
-      <c r="O46" s="30"/>
-      <c r="P46" s="85"/>
-      <c r="Q46" s="51" t="s">
-        <v>251</v>
-      </c>
-      <c r="R46" s="35"/>
-      <c r="S46" s="35"/>
-      <c r="T46" s="35"/>
-      <c r="U46" s="35"/>
+      <c r="N46" s="31">
+        <v>5</v>
+      </c>
+      <c r="O46" s="30">
+        <v>10</v>
+      </c>
+      <c r="P46" s="77">
+        <v>10</v>
+      </c>
+      <c r="Q46" s="82" t="s">
+        <v>247</v>
+      </c>
+      <c r="R46" s="35">
+        <v>2.2324000000000002</v>
+      </c>
+      <c r="S46" s="35">
+        <v>11.16</v>
+      </c>
+      <c r="T46" s="35">
+        <v>1.9319999999999999</v>
+      </c>
+      <c r="U46" s="35">
+        <v>19.32</v>
+      </c>
       <c r="V46" s="32"/>
     </row>
     <row r="47" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -4188,7 +4698,7 @@
       <c r="D47" s="34" t="s">
         <v>51</v>
       </c>
-      <c r="E47" s="55" t="s">
+      <c r="E47" s="48" t="s">
         <v>88</v>
       </c>
       <c r="F47" s="33" t="s">
@@ -4201,109 +4711,147 @@
         <v>171</v>
       </c>
       <c r="I47" s="34"/>
-      <c r="J47" s="33"/>
+      <c r="J47" s="33" t="s">
+        <v>263</v>
+      </c>
       <c r="K47" s="34" t="s">
-        <v>148</v>
+        <v>249</v>
       </c>
       <c r="L47" s="33">
         <v>1</v>
       </c>
-      <c r="M47" s="58">
-        <f t="shared" ref="M47" si="18">L47*5</f>
+      <c r="M47" s="51">
+        <f t="shared" ref="M47" si="16">L47*5</f>
         <v>5</v>
       </c>
-      <c r="N47" s="34"/>
-      <c r="O47" s="33"/>
-      <c r="P47" s="84"/>
-      <c r="Q47" s="52" t="s">
-        <v>251</v>
-      </c>
-      <c r="R47" s="36"/>
-      <c r="S47" s="36"/>
-      <c r="T47" s="36"/>
-      <c r="U47" s="36"/>
-      <c r="V47" s="58"/>
+      <c r="N47" s="34">
+        <v>5</v>
+      </c>
+      <c r="O47" s="33">
+        <v>10</v>
+      </c>
+      <c r="P47" s="76">
+        <v>10</v>
+      </c>
+      <c r="Q47" s="83" t="s">
+        <v>247</v>
+      </c>
+      <c r="R47" s="36">
+        <v>1.2198</v>
+      </c>
+      <c r="S47" s="36">
+        <v>6.1</v>
+      </c>
+      <c r="T47" s="36">
+        <v>1.0928</v>
+      </c>
+      <c r="U47" s="36">
+        <v>10.93</v>
+      </c>
+      <c r="V47" s="51"/>
     </row>
-    <row r="48" spans="1:22" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:22" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A48" s="1"/>
       <c r="B48" s="26">
         <f>ROW(B48) - ROW($B$9)</f>
         <v>39</v>
       </c>
-      <c r="C48" s="64" t="s">
+      <c r="C48" s="56" t="s">
         <v>12</v>
       </c>
       <c r="D48" s="31" t="s">
         <v>52</v>
       </c>
-      <c r="E48" s="63" t="s">
+      <c r="E48" s="55" t="s">
         <v>89</v>
       </c>
-      <c r="F48" s="64" t="s">
+      <c r="F48" s="56" t="s">
         <v>117</v>
       </c>
       <c r="G48" s="31" t="s">
         <v>149</v>
       </c>
-      <c r="H48" s="64" t="s">
+      <c r="H48" s="56" t="s">
         <v>172</v>
       </c>
       <c r="I48" s="31"/>
-      <c r="J48" s="64" t="s">
-        <v>203</v>
+      <c r="J48" s="56" t="s">
+        <v>199</v>
       </c>
       <c r="K48" s="31" t="s">
-        <v>149</v>
-      </c>
-      <c r="L48" s="72">
+        <v>249</v>
+      </c>
+      <c r="L48" s="64">
         <v>1</v>
       </c>
-      <c r="M48" s="60">
+      <c r="M48" s="53">
         <f>L48*5</f>
         <v>5</v>
       </c>
-      <c r="N48" s="31"/>
-      <c r="O48" s="64"/>
-      <c r="P48" s="89"/>
-      <c r="Q48" s="51" t="s">
-        <v>251</v>
-      </c>
-      <c r="R48" s="62"/>
-      <c r="S48" s="62"/>
-      <c r="T48" s="62"/>
-      <c r="U48" s="62"/>
+      <c r="N48" s="31">
+        <v>5</v>
+      </c>
+      <c r="O48" s="56">
+        <v>10</v>
+      </c>
+      <c r="P48" s="81">
+        <v>10</v>
+      </c>
+      <c r="Q48" s="82" t="s">
+        <v>247</v>
+      </c>
+      <c r="R48" s="35">
+        <v>6.83E-2</v>
+      </c>
+      <c r="S48" s="98">
+        <v>0.34</v>
+      </c>
+      <c r="T48" s="35">
+        <v>6.83E-2</v>
+      </c>
+      <c r="U48" s="98">
+        <v>0.68</v>
+      </c>
       <c r="V48" s="32"/>
     </row>
-    <row r="49" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:22" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A49" s="1"/>
       <c r="B49" s="22"/>
       <c r="C49" s="28"/>
       <c r="D49" s="23"/>
-      <c r="E49" s="69"/>
+      <c r="E49" s="61"/>
       <c r="F49" s="24"/>
       <c r="G49" s="25"/>
       <c r="H49" s="24"/>
       <c r="I49" s="25"/>
       <c r="J49" s="24"/>
       <c r="K49" s="25"/>
-      <c r="L49" s="71"/>
+      <c r="L49" s="63"/>
       <c r="M49" s="25"/>
       <c r="N49" s="25"/>
       <c r="O49" s="25"/>
       <c r="P49" s="25"/>
-      <c r="Q49" s="25"/>
-      <c r="R49" s="25"/>
-      <c r="S49" s="25"/>
+      <c r="Q49" s="93" t="s">
+        <v>264</v>
+      </c>
+      <c r="R49" s="94"/>
+      <c r="S49" s="97">
+        <f>SUM(S10:S48)</f>
+        <v>40.880000000000003</v>
+      </c>
       <c r="T49" s="25"/>
-      <c r="U49" s="25"/>
-      <c r="V49" s="45"/>
+      <c r="U49" s="97">
+        <f>SUM(U10:U48)</f>
+        <v>64.87</v>
+      </c>
+      <c r="V49" s="89"/>
     </row>
-    <row r="50" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:22" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A50" s="1"/>
       <c r="B50" s="18"/>
       <c r="C50" s="29"/>
       <c r="D50" s="7"/>
-      <c r="E50" s="70"/>
+      <c r="E50" s="62"/>
       <c r="F50" s="8"/>
       <c r="G50" s="8"/>
       <c r="H50" s="8"/>
@@ -4315,18 +4863,28 @@
       <c r="N50" s="8"/>
       <c r="O50" s="8"/>
       <c r="P50" s="8"/>
-      <c r="Q50" s="8"/>
-      <c r="R50" s="8"/>
-      <c r="S50" s="8"/>
+      <c r="Q50" s="95" t="s">
+        <v>265</v>
+      </c>
+      <c r="R50" s="96"/>
+      <c r="S50" s="99">
+        <f>(S49/5)</f>
+        <v>8.1760000000000002</v>
+      </c>
       <c r="T50" s="8"/>
-      <c r="U50" s="8"/>
-      <c r="V50" s="46"/>
+      <c r="U50" s="99">
+        <f>(U49/10)</f>
+        <v>6.4870000000000001</v>
+      </c>
+      <c r="V50" s="90"/>
     </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="5">
     <mergeCell ref="K1:V1"/>
     <mergeCell ref="V3:V8"/>
     <mergeCell ref="V49:V50"/>
+    <mergeCell ref="Q49:R49"/>
+    <mergeCell ref="Q50:R50"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="H10" r:id="rId1" display="https://www.lcsc.com/brand-detail/994.html"/>
@@ -4339,9 +4897,35 @@
     <hyperlink ref="Q16" r:id="rId8"/>
     <hyperlink ref="Q17" r:id="rId9"/>
     <hyperlink ref="Q19" r:id="rId10"/>
+    <hyperlink ref="Q21" r:id="rId11"/>
+    <hyperlink ref="Q22" r:id="rId12"/>
+    <hyperlink ref="Q23" r:id="rId13"/>
+    <hyperlink ref="Q18" r:id="rId14"/>
+    <hyperlink ref="Q20" r:id="rId15"/>
+    <hyperlink ref="Q24" r:id="rId16"/>
+    <hyperlink ref="Q25" r:id="rId17"/>
+    <hyperlink ref="Q26" r:id="rId18"/>
+    <hyperlink ref="Q27" r:id="rId19"/>
+    <hyperlink ref="Q28" r:id="rId20"/>
+    <hyperlink ref="Q30" r:id="rId21"/>
+    <hyperlink ref="Q29" r:id="rId22"/>
+    <hyperlink ref="Q44" r:id="rId23"/>
+    <hyperlink ref="Q31" r:id="rId24"/>
+    <hyperlink ref="Q32" r:id="rId25"/>
+    <hyperlink ref="Q33" r:id="rId26"/>
+    <hyperlink ref="Q34" r:id="rId27"/>
+    <hyperlink ref="Q35" r:id="rId28"/>
+    <hyperlink ref="Q36" r:id="rId29"/>
+    <hyperlink ref="Q37" r:id="rId30"/>
+    <hyperlink ref="Q38" r:id="rId31"/>
+    <hyperlink ref="Q39" r:id="rId32"/>
+    <hyperlink ref="Q40" r:id="rId33"/>
+    <hyperlink ref="Q48" r:id="rId34"/>
+    <hyperlink ref="Q47" r:id="rId35"/>
+    <hyperlink ref="Q46" r:id="rId36"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId11"/>
-  <drawing r:id="rId12"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId37"/>
+  <drawing r:id="rId38"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
#34 BOM completed, 2 parts remaining.
</commit_message>
<xml_diff>
--- a/Deliverables/BOM/PAC5527/eSpark_BOM.xlsx
+++ b/Deliverables/BOM/PAC5527/eSpark_BOM.xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="412" uniqueCount="266">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="373" uniqueCount="251">
   <si>
     <t>Component list</t>
   </si>
@@ -76,9 +76,6 @@
     <t>C1, C2</t>
   </si>
   <si>
-    <t>C3, C12</t>
-  </si>
-  <si>
     <t>C4, C7</t>
   </si>
   <si>
@@ -94,9 +91,6 @@
     <t>C10</t>
   </si>
   <si>
-    <t>C11</t>
-  </si>
-  <si>
     <t>C13, C14, C15</t>
   </si>
   <si>
@@ -109,12 +103,6 @@
     <t>C22</t>
   </si>
   <si>
-    <t>D1</t>
-  </si>
-  <si>
-    <t>D2, D3, D4</t>
-  </si>
-  <si>
     <t>J1</t>
   </si>
   <si>
@@ -142,18 +130,12 @@
     <t>Q1, Q2, Q3, Q4, Q5, Q6</t>
   </si>
   <si>
-    <t>R1, R2</t>
-  </si>
-  <si>
     <t>R3, R4, R5</t>
   </si>
   <si>
     <t>R6, R7, R8, R18, R19, R20</t>
   </si>
   <si>
-    <t>R9, R11, R16, R25</t>
-  </si>
-  <si>
     <t>R10, R12, R17</t>
   </si>
   <si>
@@ -169,12 +151,6 @@
     <t>R23</t>
   </si>
   <si>
-    <t>R24</t>
-  </si>
-  <si>
-    <t>SB1</t>
-  </si>
-  <si>
     <t>SW1</t>
   </si>
   <si>
@@ -223,9 +199,6 @@
     <t>CAP CER 0.1UF 16V X5R 0402</t>
   </si>
   <si>
-    <t>TVS DIODE 5V 9.8V SOD923</t>
-  </si>
-  <si>
     <t>DIODE GEN PURP 75V 150MA SOD323</t>
   </si>
   <si>
@@ -253,9 +226,6 @@
     <t>DFN(3.3x3.3) N 40V 20A  Transistor</t>
   </si>
   <si>
-    <t>RES SMD 5.1K OHM 5% 1/10W 0603</t>
-  </si>
-  <si>
     <t>RES 1 OHM 1% 1/16W 0402</t>
   </si>
   <si>
@@ -283,18 +253,12 @@
     <t>RES 120 OHM 1% 1/10W 0603</t>
   </si>
   <si>
-    <t>Solder Bridge ON</t>
-  </si>
-  <si>
     <t>3mm 2mm Round Button 50mA Top3.65mm SPST 12V SMD Tactile Switches</t>
   </si>
   <si>
     <t>PAC5527 48V BLDC Motor Controller and Driver Evaluation Board</t>
   </si>
   <si>
-    <t>SOP-8 Position Sensor ROHS</t>
-  </si>
-  <si>
     <t>IC TXRX CAN 3.3V SOT23-8</t>
   </si>
   <si>
@@ -319,9 +283,6 @@
     <t>Cap-0402</t>
   </si>
   <si>
-    <t>SOD-923.</t>
-  </si>
-  <si>
     <t>SOD-323</t>
   </si>
   <si>
@@ -367,18 +328,12 @@
     <t>RES-0805</t>
   </si>
   <si>
-    <t>Solder Bridge</t>
-  </si>
-  <si>
     <t>TS-1185EC-C-D-B_</t>
   </si>
   <si>
     <t>48-QFN (6x6)_</t>
   </si>
   <si>
-    <t>SOP-8</t>
-  </si>
-  <si>
     <t>SOT-23-8</t>
   </si>
   <si>
@@ -418,9 +373,6 @@
     <t>CC0402KRX5R7BB104</t>
   </si>
   <si>
-    <t>ESD9L5.0ST5G</t>
-  </si>
-  <si>
     <t>1N4148WS-7-F</t>
   </si>
   <si>
@@ -436,9 +388,6 @@
     <t>YJQ20N04A</t>
   </si>
   <si>
-    <t>RC0603JR-075K1L</t>
-  </si>
-  <si>
     <t>RC0402FR-071RL</t>
   </si>
   <si>
@@ -472,9 +421,6 @@
     <t>PAC5527QMST</t>
   </si>
   <si>
-    <t>MT6701CT-STD-R</t>
-  </si>
-  <si>
     <t>MAX3051EKA+T</t>
   </si>
   <si>
@@ -502,9 +448,6 @@
     <t>Wurth Electronics</t>
   </si>
   <si>
-    <t>ON Semiconductor</t>
-  </si>
-  <si>
     <t>Diodes</t>
   </si>
   <si>
@@ -541,9 +484,6 @@
     <t>Qorvo</t>
   </si>
   <si>
-    <t>Magn Tek</t>
-  </si>
-  <si>
     <t>Maxim</t>
   </si>
   <si>
@@ -580,9 +520,6 @@
     <t>C106204</t>
   </si>
   <si>
-    <t>C82326</t>
-  </si>
-  <si>
     <t>C60580</t>
   </si>
   <si>
@@ -601,9 +538,6 @@
     <t>C919577</t>
   </si>
   <si>
-    <t>C14677</t>
-  </si>
-  <si>
     <t>C185446</t>
   </si>
   <si>
@@ -625,9 +559,6 @@
     <t>C318893</t>
   </si>
   <si>
-    <t>C3003196</t>
-  </si>
-  <si>
     <t>C92102</t>
   </si>
   <si>
@@ -667,9 +598,6 @@
     <t>TEST POINT</t>
   </si>
   <si>
-    <t>5.1K</t>
-  </si>
-  <si>
     <t>1R</t>
   </si>
   <si>
@@ -827,6 +755,33 @@
   </si>
   <si>
     <t>Cost per Board</t>
+  </si>
+  <si>
+    <t>C3</t>
+  </si>
+  <si>
+    <t>C11, C12</t>
+  </si>
+  <si>
+    <t>D1, D2, D3</t>
+  </si>
+  <si>
+    <t>R9, R11, R16, R1</t>
+  </si>
+  <si>
+    <t>R2</t>
+  </si>
+  <si>
+    <t>Digital Contactless Angle Sensor with ABZ Incremental &amp; PWM Outputs 3.3V 12-Bit 16-Pin QFN T/R</t>
+  </si>
+  <si>
+    <t>16-QFN (3x3)</t>
+  </si>
+  <si>
+    <t>MA702GQ-Z</t>
+  </si>
+  <si>
+    <t>Monolithic Power Systems</t>
   </si>
 </sst>
 </file>
@@ -836,9 +791,9 @@
   <numFmts count="3">
     <numFmt numFmtId="164" formatCode="[$-409]h:mm:ss\ AM/PM;@"/>
     <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.0000"/>
-    <numFmt numFmtId="170" formatCode="&quot;$&quot;#,##0.00"/>
+    <numFmt numFmtId="166" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="23" x14ac:knownFonts="1">
+  <fonts count="24" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -998,6 +953,12 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color indexed="13"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="7">
     <fill>
@@ -1037,7 +998,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="31">
+  <borders count="28">
     <border>
       <left/>
       <right/>
@@ -1270,34 +1231,6 @@
       <diagonal/>
     </border>
     <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
       <left/>
       <right style="thin">
         <color indexed="64"/>
@@ -1387,17 +1320,6 @@
       <top style="medium">
         <color indexed="64"/>
       </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top/>
       <bottom/>
       <diagonal/>
     </border>
@@ -1406,7 +1328,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="100">
+  <cellXfs count="88">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1521,48 +1443,24 @@
     <xf numFmtId="0" fontId="11" fillId="3" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="17" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="4" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="18" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="18" fillId="4" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="5" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="5" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="4" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="4" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="10" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="18" fillId="4" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="2" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="4" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="2" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1582,13 +1480,7 @@
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="18" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="24" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="22" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1609,31 +1501,28 @@
     </xf>
     <xf numFmtId="0" fontId="16" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="10" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="18" fillId="4" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="2" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="4" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="2" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="4" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="2" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="165" fontId="19" fillId="2" borderId="5" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="165" fontId="19" fillId="4" borderId="6" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="17" fillId="3" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="17" fillId="3" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1653,12 +1542,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="2" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="6" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1675,13 +1558,14 @@
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="170" fontId="17" fillId="3" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="18" fillId="2" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="170" fontId="17" fillId="3" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="23" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="20" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2026,7 +1910,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:V50"/>
+  <dimension ref="A1:V47"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="3.140625" style="19" customWidth="1"/>
@@ -2060,18 +1944,18 @@
       <c r="H1" s="2"/>
       <c r="I1" s="2"/>
       <c r="J1" s="2"/>
-      <c r="K1" s="84"/>
-      <c r="L1" s="84"/>
-      <c r="M1" s="84"/>
-      <c r="N1" s="84"/>
-      <c r="O1" s="84"/>
-      <c r="P1" s="84"/>
-      <c r="Q1" s="84"/>
-      <c r="R1" s="84"/>
-      <c r="S1" s="84"/>
-      <c r="T1" s="84"/>
-      <c r="U1" s="84"/>
-      <c r="V1" s="85"/>
+      <c r="K1" s="73"/>
+      <c r="L1" s="73"/>
+      <c r="M1" s="73"/>
+      <c r="N1" s="73"/>
+      <c r="O1" s="73"/>
+      <c r="P1" s="73"/>
+      <c r="Q1" s="73"/>
+      <c r="R1" s="73"/>
+      <c r="S1" s="73"/>
+      <c r="T1" s="73"/>
+      <c r="U1" s="73"/>
+      <c r="V1" s="74"/>
     </row>
     <row r="2" spans="1:22" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
@@ -2080,8 +1964,8 @@
       <c r="D2" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="E2" s="57"/>
-      <c r="F2" s="66" t="s">
+      <c r="E2" s="49"/>
+      <c r="F2" s="56" t="s">
         <v>5</v>
       </c>
       <c r="G2" s="38"/>
@@ -2104,39 +1988,39 @@
     <row r="3" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
       <c r="B3" s="16"/>
-      <c r="C3" s="67"/>
-      <c r="D3" s="59" t="s">
+      <c r="C3" s="57"/>
+      <c r="D3" s="51" t="s">
         <v>1</v>
       </c>
-      <c r="E3" s="59"/>
-      <c r="F3" s="58" t="s">
+      <c r="E3" s="51"/>
+      <c r="F3" s="50" t="s">
         <v>6</v>
       </c>
-      <c r="G3" s="59"/>
-      <c r="H3" s="49"/>
-      <c r="I3" s="59"/>
-      <c r="J3" s="49"/>
+      <c r="G3" s="51"/>
+      <c r="H3" s="44"/>
+      <c r="I3" s="51"/>
+      <c r="J3" s="44"/>
       <c r="K3" s="5"/>
-      <c r="L3" s="49"/>
-      <c r="M3" s="49"/>
-      <c r="N3" s="49"/>
-      <c r="O3" s="49"/>
-      <c r="P3" s="49"/>
-      <c r="Q3" s="49"/>
-      <c r="R3" s="49"/>
-      <c r="S3" s="49"/>
-      <c r="T3" s="49"/>
-      <c r="U3" s="49"/>
-      <c r="V3" s="86"/>
+      <c r="L3" s="44"/>
+      <c r="M3" s="44"/>
+      <c r="N3" s="44"/>
+      <c r="O3" s="44"/>
+      <c r="P3" s="44"/>
+      <c r="Q3" s="44"/>
+      <c r="R3" s="44"/>
+      <c r="S3" s="44"/>
+      <c r="T3" s="44"/>
+      <c r="U3" s="44"/>
+      <c r="V3" s="75"/>
     </row>
     <row r="4" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
       <c r="B4" s="16"/>
-      <c r="C4" s="67"/>
-      <c r="D4" s="59" t="s">
+      <c r="C4" s="57"/>
+      <c r="D4" s="51" t="s">
         <v>2</v>
       </c>
-      <c r="E4" s="59"/>
+      <c r="E4" s="51"/>
       <c r="F4" s="39" t="s">
         <v>6</v>
       </c>
@@ -2154,17 +2038,17 @@
       <c r="R4" s="6"/>
       <c r="S4" s="6"/>
       <c r="T4" s="6"/>
-      <c r="U4" s="75"/>
-      <c r="V4" s="87"/>
+      <c r="U4" s="65"/>
+      <c r="V4" s="76"/>
     </row>
     <row r="5" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
       <c r="B5" s="16"/>
-      <c r="C5" s="67"/>
-      <c r="D5" s="59" t="s">
+      <c r="C5" s="57"/>
+      <c r="D5" s="51" t="s">
         <v>3</v>
       </c>
-      <c r="E5" s="59"/>
+      <c r="E5" s="51"/>
       <c r="F5" s="40" t="s">
         <v>7</v>
       </c>
@@ -2183,14 +2067,14 @@
       <c r="S5" s="5"/>
       <c r="T5" s="5"/>
       <c r="U5" s="5"/>
-      <c r="V5" s="87"/>
+      <c r="V5" s="76"/>
     </row>
     <row r="6" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
       <c r="B6" s="16"/>
-      <c r="C6" s="67"/>
-      <c r="D6" s="59"/>
-      <c r="E6" s="59"/>
+      <c r="C6" s="57"/>
+      <c r="D6" s="51"/>
+      <c r="E6" s="51"/>
       <c r="F6" s="12"/>
       <c r="G6" s="11"/>
       <c r="H6" s="5"/>
@@ -2207,55 +2091,55 @@
       <c r="S6" s="5"/>
       <c r="T6" s="5"/>
       <c r="U6" s="5"/>
-      <c r="V6" s="87"/>
+      <c r="V6" s="76"/>
     </row>
     <row r="7" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
       <c r="B7" s="17"/>
-      <c r="C7" s="68"/>
-      <c r="D7" s="60"/>
-      <c r="E7" s="60"/>
+      <c r="C7" s="58"/>
+      <c r="D7" s="52"/>
+      <c r="E7" s="52"/>
       <c r="F7" s="13"/>
-      <c r="G7" s="60"/>
-      <c r="H7" s="50"/>
-      <c r="I7" s="60"/>
-      <c r="J7" s="50"/>
-      <c r="K7" s="50"/>
-      <c r="L7" s="50"/>
-      <c r="M7" s="50"/>
-      <c r="N7" s="50"/>
-      <c r="O7" s="50"/>
-      <c r="P7" s="50"/>
-      <c r="Q7" s="50"/>
-      <c r="R7" s="50"/>
-      <c r="S7" s="50"/>
-      <c r="T7" s="50"/>
-      <c r="U7" s="50"/>
-      <c r="V7" s="87"/>
+      <c r="G7" s="52"/>
+      <c r="H7" s="45"/>
+      <c r="I7" s="52"/>
+      <c r="J7" s="45"/>
+      <c r="K7" s="45"/>
+      <c r="L7" s="45"/>
+      <c r="M7" s="45"/>
+      <c r="N7" s="45"/>
+      <c r="O7" s="45"/>
+      <c r="P7" s="45"/>
+      <c r="Q7" s="45"/>
+      <c r="R7" s="45"/>
+      <c r="S7" s="45"/>
+      <c r="T7" s="45"/>
+      <c r="U7" s="45"/>
+      <c r="V7" s="76"/>
     </row>
     <row r="8" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
-      <c r="B8" s="69"/>
-      <c r="C8" s="70"/>
-      <c r="D8" s="71"/>
-      <c r="E8" s="71"/>
-      <c r="F8" s="72"/>
-      <c r="G8" s="73"/>
-      <c r="H8" s="74"/>
-      <c r="I8" s="73"/>
-      <c r="J8" s="74"/>
-      <c r="K8" s="74"/>
-      <c r="L8" s="74"/>
-      <c r="M8" s="74"/>
-      <c r="N8" s="74"/>
-      <c r="O8" s="74"/>
-      <c r="P8" s="74"/>
-      <c r="Q8" s="74"/>
-      <c r="R8" s="74"/>
-      <c r="S8" s="74"/>
-      <c r="T8" s="74"/>
-      <c r="U8" s="74"/>
-      <c r="V8" s="88"/>
+      <c r="B8" s="59"/>
+      <c r="C8" s="60"/>
+      <c r="D8" s="61"/>
+      <c r="E8" s="61"/>
+      <c r="F8" s="62"/>
+      <c r="G8" s="63"/>
+      <c r="H8" s="64"/>
+      <c r="I8" s="63"/>
+      <c r="J8" s="64"/>
+      <c r="K8" s="64"/>
+      <c r="L8" s="64"/>
+      <c r="M8" s="64"/>
+      <c r="N8" s="64"/>
+      <c r="O8" s="64"/>
+      <c r="P8" s="64"/>
+      <c r="Q8" s="64"/>
+      <c r="R8" s="64"/>
+      <c r="S8" s="64"/>
+      <c r="T8" s="64"/>
+      <c r="U8" s="64"/>
+      <c r="V8" s="77"/>
     </row>
     <row r="9" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
@@ -2265,62 +2149,62 @@
       <c r="C9" s="20" t="s">
         <v>8</v>
       </c>
-      <c r="D9" s="42" t="s">
+      <c r="D9" s="41" t="s">
         <v>13</v>
       </c>
-      <c r="E9" s="46" t="s">
-        <v>53</v>
+      <c r="E9" s="42" t="s">
+        <v>45</v>
       </c>
       <c r="F9" s="20" t="s">
-        <v>90</v>
+        <v>78</v>
       </c>
       <c r="G9" s="21" t="s">
-        <v>118</v>
+        <v>103</v>
       </c>
       <c r="H9" s="20" t="s">
-        <v>150</v>
+        <v>132</v>
       </c>
       <c r="I9" s="20" t="s">
-        <v>230</v>
+        <v>206</v>
       </c>
       <c r="J9" s="21" t="s">
-        <v>173</v>
+        <v>153</v>
       </c>
       <c r="K9" s="20" t="s">
-        <v>231</v>
+        <v>207</v>
       </c>
       <c r="L9" s="20" t="s">
-        <v>222</v>
+        <v>198</v>
       </c>
       <c r="M9" s="20" t="s">
-        <v>233</v>
-      </c>
-      <c r="N9" s="42" t="s">
-        <v>235</v>
+        <v>209</v>
+      </c>
+      <c r="N9" s="41" t="s">
+        <v>211</v>
       </c>
       <c r="O9" s="20" t="s">
-        <v>232</v>
+        <v>208</v>
       </c>
       <c r="P9" s="20" t="s">
-        <v>234</v>
-      </c>
-      <c r="Q9" s="46" t="s">
-        <v>236</v>
+        <v>210</v>
+      </c>
+      <c r="Q9" s="42" t="s">
+        <v>212</v>
       </c>
       <c r="R9" s="20" t="s">
-        <v>240</v>
+        <v>216</v>
       </c>
       <c r="S9" s="20" t="s">
-        <v>241</v>
+        <v>217</v>
       </c>
       <c r="T9" s="20" t="s">
-        <v>237</v>
+        <v>213</v>
       </c>
       <c r="U9" s="20" t="s">
-        <v>238</v>
-      </c>
-      <c r="V9" s="42" t="s">
-        <v>239</v>
+        <v>214</v>
+      </c>
+      <c r="V9" s="41" t="s">
+        <v>215</v>
       </c>
     </row>
     <row r="10" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -2330,29 +2214,29 @@
         <v>1</v>
       </c>
       <c r="C10" s="30" t="s">
-        <v>223</v>
+        <v>199</v>
       </c>
       <c r="D10" s="31" t="s">
         <v>14</v>
       </c>
-      <c r="E10" s="55" t="s">
-        <v>242</v>
+      <c r="E10" s="48" t="s">
+        <v>218</v>
       </c>
       <c r="F10" s="37" t="s">
-        <v>243</v>
+        <v>219</v>
       </c>
       <c r="G10" s="31" t="s">
-        <v>244</v>
+        <v>220</v>
       </c>
       <c r="H10" s="30" t="s">
-        <v>245</v>
+        <v>221</v>
       </c>
       <c r="I10" s="31"/>
       <c r="J10" s="30" t="s">
-        <v>246</v>
+        <v>222</v>
       </c>
       <c r="K10" s="31" t="s">
-        <v>200</v>
+        <v>177</v>
       </c>
       <c r="L10" s="37">
         <v>2</v>
@@ -2370,8 +2254,8 @@
       <c r="P10" s="37">
         <v>20</v>
       </c>
-      <c r="Q10" s="82" t="s">
-        <v>247</v>
+      <c r="Q10" s="68" t="s">
+        <v>223</v>
       </c>
       <c r="R10" s="35">
         <v>0.29630000000000001</v>
@@ -2390,52 +2274,52 @@
     <row r="11" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="1"/>
       <c r="B11" s="26">
-        <f t="shared" ref="B11:B47" si="0">ROW(B11) - ROW($B$9)</f>
+        <f t="shared" ref="B11:B44" si="0">ROW(B11) - ROW($B$9)</f>
         <v>2</v>
       </c>
       <c r="C11" s="33" t="s">
-        <v>223</v>
+        <v>199</v>
       </c>
       <c r="D11" s="34" t="s">
-        <v>15</v>
-      </c>
-      <c r="E11" s="48" t="s">
-        <v>54</v>
+        <v>242</v>
+      </c>
+      <c r="E11" s="43" t="s">
+        <v>46</v>
       </c>
       <c r="F11" s="33" t="s">
-        <v>91</v>
+        <v>79</v>
       </c>
       <c r="G11" s="34" t="s">
-        <v>119</v>
+        <v>104</v>
       </c>
       <c r="H11" s="33" t="s">
-        <v>151</v>
+        <v>133</v>
       </c>
       <c r="I11" s="34"/>
       <c r="J11" s="33" t="s">
-        <v>174</v>
+        <v>154</v>
       </c>
       <c r="K11" s="34" t="s">
-        <v>201</v>
+        <v>178</v>
       </c>
       <c r="L11" s="33">
-        <v>2</v>
-      </c>
-      <c r="M11" s="51">
+        <v>1</v>
+      </c>
+      <c r="M11" s="46">
         <f>L11*5</f>
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="N11" s="34">
         <v>100</v>
       </c>
       <c r="O11" s="33">
-        <v>20</v>
-      </c>
-      <c r="P11" s="76">
+        <v>10</v>
+      </c>
+      <c r="P11" s="66">
         <v>100</v>
       </c>
-      <c r="Q11" s="83" t="s">
-        <v>247</v>
+      <c r="Q11" s="69" t="s">
+        <v>223</v>
       </c>
       <c r="R11" s="36">
         <v>5.1000000000000004E-3</v>
@@ -2449,7 +2333,7 @@
       <c r="U11" s="36">
         <v>0.51</v>
       </c>
-      <c r="V11" s="51"/>
+      <c r="V11" s="46"/>
     </row>
     <row r="12" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="1"/>
@@ -2458,31 +2342,31 @@
         <v>3</v>
       </c>
       <c r="C12" s="30" t="s">
-        <v>223</v>
+        <v>199</v>
       </c>
       <c r="D12" s="31" t="s">
-        <v>16</v>
-      </c>
-      <c r="E12" s="55" t="s">
-        <v>55</v>
+        <v>15</v>
+      </c>
+      <c r="E12" s="48" t="s">
+        <v>47</v>
       </c>
       <c r="F12" s="30" t="s">
-        <v>92</v>
+        <v>80</v>
       </c>
       <c r="G12" s="31" t="s">
-        <v>120</v>
+        <v>105</v>
       </c>
       <c r="H12" s="30" t="s">
-        <v>151</v>
+        <v>133</v>
       </c>
       <c r="I12" s="31"/>
       <c r="J12" s="30" t="s">
-        <v>175</v>
+        <v>155</v>
       </c>
       <c r="K12" s="31" t="s">
-        <v>202</v>
-      </c>
-      <c r="L12" s="54">
+        <v>179</v>
+      </c>
+      <c r="L12" s="47">
         <v>2</v>
       </c>
       <c r="M12" s="32">
@@ -2495,11 +2379,11 @@
       <c r="O12" s="30">
         <v>20</v>
       </c>
-      <c r="P12" s="77">
+      <c r="P12" s="67">
         <v>50</v>
       </c>
-      <c r="Q12" s="82" t="s">
-        <v>247</v>
+      <c r="Q12" s="68" t="s">
+        <v>223</v>
       </c>
       <c r="R12" s="35">
         <v>1.78E-2</v>
@@ -2522,34 +2406,34 @@
         <v>4</v>
       </c>
       <c r="C13" s="33" t="s">
-        <v>223</v>
+        <v>199</v>
       </c>
       <c r="D13" s="34" t="s">
-        <v>17</v>
-      </c>
-      <c r="E13" s="48" t="s">
-        <v>56</v>
+        <v>16</v>
+      </c>
+      <c r="E13" s="43" t="s">
+        <v>48</v>
       </c>
       <c r="F13" s="33" t="s">
-        <v>91</v>
+        <v>79</v>
       </c>
       <c r="G13" s="34" t="s">
-        <v>121</v>
+        <v>106</v>
       </c>
       <c r="H13" s="33" t="s">
-        <v>151</v>
+        <v>133</v>
       </c>
       <c r="I13" s="34"/>
       <c r="J13" s="33" t="s">
-        <v>176</v>
+        <v>156</v>
       </c>
       <c r="K13" s="34" t="s">
-        <v>203</v>
+        <v>180</v>
       </c>
       <c r="L13" s="33">
         <v>1</v>
       </c>
-      <c r="M13" s="51">
+      <c r="M13" s="46">
         <f t="shared" ref="M13" si="1">L13*5</f>
         <v>5</v>
       </c>
@@ -2559,11 +2443,11 @@
       <c r="O13" s="33">
         <v>10</v>
       </c>
-      <c r="P13" s="76">
+      <c r="P13" s="66">
         <v>50</v>
       </c>
-      <c r="Q13" s="83" t="s">
-        <v>247</v>
+      <c r="Q13" s="69" t="s">
+        <v>223</v>
       </c>
       <c r="R13" s="36">
         <v>1.7100000000000001E-2</v>
@@ -2577,7 +2461,7 @@
       <c r="U13" s="36">
         <v>0.86</v>
       </c>
-      <c r="V13" s="51"/>
+      <c r="V13" s="46"/>
     </row>
     <row r="14" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="1"/>
@@ -2586,31 +2470,31 @@
         <v>5</v>
       </c>
       <c r="C14" s="30" t="s">
-        <v>223</v>
+        <v>199</v>
       </c>
       <c r="D14" s="31" t="s">
-        <v>18</v>
-      </c>
-      <c r="E14" s="55" t="s">
-        <v>57</v>
+        <v>17</v>
+      </c>
+      <c r="E14" s="48" t="s">
+        <v>49</v>
       </c>
       <c r="F14" s="30" t="s">
-        <v>93</v>
+        <v>81</v>
       </c>
       <c r="G14" s="31" t="s">
-        <v>122</v>
+        <v>107</v>
       </c>
       <c r="H14" s="30" t="s">
-        <v>152</v>
+        <v>134</v>
       </c>
       <c r="I14" s="31"/>
       <c r="J14" s="30" t="s">
-        <v>177</v>
+        <v>157</v>
       </c>
       <c r="K14" s="31" t="s">
-        <v>204</v>
-      </c>
-      <c r="L14" s="54">
+        <v>181</v>
+      </c>
+      <c r="L14" s="47">
         <v>1</v>
       </c>
       <c r="M14" s="32">
@@ -2623,11 +2507,11 @@
       <c r="O14" s="30">
         <v>10</v>
       </c>
-      <c r="P14" s="77">
+      <c r="P14" s="67">
         <v>20</v>
       </c>
-      <c r="Q14" s="82" t="s">
-        <v>247</v>
+      <c r="Q14" s="68" t="s">
+        <v>223</v>
       </c>
       <c r="R14" s="35">
         <v>1.3299999999999999E-2</v>
@@ -2650,34 +2534,34 @@
         <v>6</v>
       </c>
       <c r="C15" s="33" t="s">
-        <v>223</v>
+        <v>199</v>
       </c>
       <c r="D15" s="34" t="s">
-        <v>19</v>
-      </c>
-      <c r="E15" s="48" t="s">
-        <v>55</v>
+        <v>18</v>
+      </c>
+      <c r="E15" s="43" t="s">
+        <v>47</v>
       </c>
       <c r="F15" s="33" t="s">
-        <v>91</v>
+        <v>79</v>
       </c>
       <c r="G15" s="34" t="s">
-        <v>123</v>
+        <v>108</v>
       </c>
       <c r="H15" s="33" t="s">
-        <v>152</v>
+        <v>134</v>
       </c>
       <c r="I15" s="34"/>
       <c r="J15" s="33" t="s">
-        <v>178</v>
+        <v>158</v>
       </c>
       <c r="K15" s="34" t="s">
-        <v>202</v>
+        <v>179</v>
       </c>
       <c r="L15" s="33">
         <v>2</v>
       </c>
-      <c r="M15" s="51">
+      <c r="M15" s="46">
         <f t="shared" ref="M15" si="2">L15*5</f>
         <v>10</v>
       </c>
@@ -2687,11 +2571,11 @@
       <c r="O15" s="33">
         <v>20</v>
       </c>
-      <c r="P15" s="76">
+      <c r="P15" s="66">
         <v>50</v>
       </c>
-      <c r="Q15" s="83" t="s">
-        <v>247</v>
+      <c r="Q15" s="69" t="s">
+        <v>223</v>
       </c>
       <c r="R15" s="36">
         <v>7.1999999999999998E-3</v>
@@ -2705,7 +2589,7 @@
       <c r="U15" s="36">
         <v>0.36</v>
       </c>
-      <c r="V15" s="51"/>
+      <c r="V15" s="46"/>
     </row>
     <row r="16" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="1"/>
@@ -2714,31 +2598,31 @@
         <v>7</v>
       </c>
       <c r="C16" s="30" t="s">
-        <v>223</v>
+        <v>199</v>
       </c>
       <c r="D16" s="31" t="s">
-        <v>20</v>
-      </c>
-      <c r="E16" s="55" t="s">
-        <v>58</v>
+        <v>19</v>
+      </c>
+      <c r="E16" s="48" t="s">
+        <v>50</v>
       </c>
       <c r="F16" s="30" t="s">
-        <v>91</v>
+        <v>79</v>
       </c>
       <c r="G16" s="31" t="s">
-        <v>124</v>
+        <v>109</v>
       </c>
       <c r="H16" s="30" t="s">
-        <v>151</v>
+        <v>133</v>
       </c>
       <c r="I16" s="31"/>
       <c r="J16" s="30" t="s">
-        <v>179</v>
+        <v>159</v>
       </c>
       <c r="K16" s="31" t="s">
-        <v>201</v>
-      </c>
-      <c r="L16" s="54">
+        <v>178</v>
+      </c>
+      <c r="L16" s="47">
         <v>1</v>
       </c>
       <c r="M16" s="32">
@@ -2751,11 +2635,11 @@
       <c r="O16" s="30">
         <v>10</v>
       </c>
-      <c r="P16" s="77">
+      <c r="P16" s="67">
         <v>100</v>
       </c>
-      <c r="Q16" s="82" t="s">
-        <v>247</v>
+      <c r="Q16" s="68" t="s">
+        <v>223</v>
       </c>
       <c r="R16" s="35">
         <v>2.5999999999999999E-3</v>
@@ -2778,48 +2662,48 @@
         <v>8</v>
       </c>
       <c r="C17" s="33" t="s">
-        <v>223</v>
-      </c>
-      <c r="D17" s="34" t="s">
-        <v>21</v>
-      </c>
-      <c r="E17" s="48" t="s">
-        <v>59</v>
+        <v>199</v>
+      </c>
+      <c r="D17" s="33" t="s">
+        <v>243</v>
+      </c>
+      <c r="E17" s="43" t="s">
+        <v>51</v>
       </c>
       <c r="F17" s="33" t="s">
-        <v>91</v>
+        <v>79</v>
       </c>
       <c r="G17" s="34" t="s">
-        <v>125</v>
+        <v>110</v>
       </c>
       <c r="H17" s="33" t="s">
-        <v>153</v>
+        <v>135</v>
       </c>
       <c r="I17" s="34"/>
       <c r="J17" s="33" t="s">
-        <v>180</v>
+        <v>160</v>
       </c>
       <c r="K17" s="34" t="s">
-        <v>205</v>
+        <v>182</v>
       </c>
       <c r="L17" s="33">
-        <v>1</v>
-      </c>
-      <c r="M17" s="51">
+        <v>2</v>
+      </c>
+      <c r="M17" s="46">
         <f t="shared" ref="M17" si="3">L17*5</f>
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="N17" s="34">
         <v>20</v>
       </c>
       <c r="O17" s="33">
-        <v>10</v>
-      </c>
-      <c r="P17" s="76">
         <v>20</v>
       </c>
-      <c r="Q17" s="83" t="s">
-        <v>247</v>
+      <c r="P17" s="66">
+        <v>20</v>
+      </c>
+      <c r="Q17" s="69" t="s">
+        <v>223</v>
       </c>
       <c r="R17" s="36">
         <v>2.7199999999999998E-2</v>
@@ -2833,7 +2717,7 @@
       <c r="U17" s="36">
         <v>0.54</v>
       </c>
-      <c r="V17" s="51"/>
+      <c r="V17" s="46"/>
     </row>
     <row r="18" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="1"/>
@@ -2842,33 +2726,33 @@
         <v>9</v>
       </c>
       <c r="C18" s="30" t="s">
-        <v>223</v>
+        <v>199</v>
       </c>
       <c r="D18" s="31" t="s">
-        <v>22</v>
-      </c>
-      <c r="E18" s="55" t="s">
-        <v>60</v>
+        <v>20</v>
+      </c>
+      <c r="E18" s="48" t="s">
+        <v>52</v>
       </c>
       <c r="F18" s="30" t="s">
-        <v>94</v>
-      </c>
-      <c r="G18" s="91" t="s">
-        <v>126</v>
+        <v>82</v>
+      </c>
+      <c r="G18" s="70" t="s">
+        <v>111</v>
       </c>
       <c r="H18" s="30" t="s">
-        <v>154</v>
+        <v>136</v>
       </c>
       <c r="I18" s="30" t="s">
-        <v>250</v>
+        <v>226</v>
       </c>
       <c r="J18" s="30" t="s">
-        <v>251</v>
+        <v>227</v>
       </c>
       <c r="K18" s="31" t="s">
-        <v>203</v>
-      </c>
-      <c r="L18" s="54">
+        <v>180</v>
+      </c>
+      <c r="L18" s="47">
         <v>3</v>
       </c>
       <c r="M18" s="32">
@@ -2881,11 +2765,11 @@
       <c r="O18" s="30">
         <v>30</v>
       </c>
-      <c r="P18" s="77">
+      <c r="P18" s="67">
         <v>30</v>
       </c>
-      <c r="Q18" s="82" t="s">
-        <v>247</v>
+      <c r="Q18" s="68" t="s">
+        <v>223</v>
       </c>
       <c r="R18" s="35">
         <v>6.0299999999999999E-2</v>
@@ -2908,34 +2792,34 @@
         <v>10</v>
       </c>
       <c r="C19" s="33" t="s">
-        <v>223</v>
+        <v>199</v>
       </c>
       <c r="D19" s="34" t="s">
-        <v>23</v>
-      </c>
-      <c r="E19" s="48" t="s">
-        <v>61</v>
+        <v>21</v>
+      </c>
+      <c r="E19" s="43" t="s">
+        <v>53</v>
       </c>
       <c r="F19" s="33" t="s">
-        <v>91</v>
+        <v>79</v>
       </c>
       <c r="G19" s="34" t="s">
-        <v>127</v>
+        <v>112</v>
       </c>
       <c r="H19" s="33" t="s">
-        <v>155</v>
+        <v>137</v>
       </c>
       <c r="I19" s="34"/>
       <c r="J19" s="33" t="s">
-        <v>181</v>
+        <v>161</v>
       </c>
       <c r="K19" s="34" t="s">
-        <v>206</v>
+        <v>183</v>
       </c>
       <c r="L19" s="33">
         <v>3</v>
       </c>
-      <c r="M19" s="51">
+      <c r="M19" s="46">
         <f t="shared" ref="M19" si="4">L19*5</f>
         <v>15</v>
       </c>
@@ -2945,11 +2829,11 @@
       <c r="O19" s="33">
         <v>30</v>
       </c>
-      <c r="P19" s="76">
+      <c r="P19" s="66">
         <v>50</v>
       </c>
-      <c r="Q19" s="83" t="s">
-        <v>247</v>
+      <c r="Q19" s="69" t="s">
+        <v>223</v>
       </c>
       <c r="R19" s="36">
         <v>7.0000000000000001E-3</v>
@@ -2963,7 +2847,7 @@
       <c r="U19" s="36">
         <v>0.35</v>
       </c>
-      <c r="V19" s="51"/>
+      <c r="V19" s="46"/>
     </row>
     <row r="20" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="1"/>
@@ -2972,33 +2856,33 @@
         <v>11</v>
       </c>
       <c r="C20" s="30" t="s">
-        <v>223</v>
+        <v>199</v>
       </c>
       <c r="D20" s="31" t="s">
-        <v>24</v>
-      </c>
-      <c r="E20" s="55" t="s">
-        <v>62</v>
+        <v>22</v>
+      </c>
+      <c r="E20" s="48" t="s">
+        <v>54</v>
       </c>
       <c r="F20" s="30" t="s">
-        <v>95</v>
-      </c>
-      <c r="G20" s="91">
+        <v>83</v>
+      </c>
+      <c r="G20" s="70">
         <v>885012205080</v>
       </c>
       <c r="H20" s="30" t="s">
-        <v>156</v>
+        <v>138</v>
       </c>
       <c r="I20" s="30" t="s">
-        <v>252</v>
+        <v>228</v>
       </c>
       <c r="J20" s="30" t="s">
-        <v>253</v>
+        <v>229</v>
       </c>
       <c r="K20" s="31" t="s">
-        <v>207</v>
-      </c>
-      <c r="L20" s="54">
+        <v>184</v>
+      </c>
+      <c r="L20" s="47">
         <v>3</v>
       </c>
       <c r="M20" s="32">
@@ -3011,11 +2895,11 @@
       <c r="O20" s="30">
         <v>30</v>
       </c>
-      <c r="P20" s="77">
+      <c r="P20" s="67">
         <v>100</v>
       </c>
-      <c r="Q20" s="82" t="s">
-        <v>247</v>
+      <c r="Q20" s="68" t="s">
+        <v>223</v>
       </c>
       <c r="R20" s="35">
         <v>4.1999999999999997E-3</v>
@@ -3038,34 +2922,34 @@
         <v>12</v>
       </c>
       <c r="C21" s="33" t="s">
-        <v>223</v>
+        <v>199</v>
       </c>
       <c r="D21" s="34" t="s">
-        <v>25</v>
-      </c>
-      <c r="E21" s="48" t="s">
-        <v>63</v>
+        <v>23</v>
+      </c>
+      <c r="E21" s="43" t="s">
+        <v>55</v>
       </c>
       <c r="F21" s="33" t="s">
-        <v>95</v>
+        <v>83</v>
       </c>
       <c r="G21" s="34" t="s">
-        <v>128</v>
+        <v>113</v>
       </c>
       <c r="H21" s="33" t="s">
-        <v>151</v>
+        <v>133</v>
       </c>
       <c r="I21" s="34"/>
       <c r="J21" s="33" t="s">
-        <v>182</v>
+        <v>162</v>
       </c>
       <c r="K21" s="34" t="s">
-        <v>201</v>
+        <v>178</v>
       </c>
       <c r="L21" s="33">
         <v>1</v>
       </c>
-      <c r="M21" s="51">
+      <c r="M21" s="46">
         <f t="shared" ref="M21" si="5">L21*5</f>
         <v>5</v>
       </c>
@@ -3075,11 +2959,11 @@
       <c r="O21" s="33">
         <v>10</v>
       </c>
-      <c r="P21" s="76">
+      <c r="P21" s="66">
         <v>100</v>
       </c>
-      <c r="Q21" s="83" t="s">
-        <v>247</v>
+      <c r="Q21" s="69" t="s">
+        <v>223</v>
       </c>
       <c r="R21" s="36">
         <v>8.9999999999999998E-4</v>
@@ -3093,135 +2977,137 @@
       <c r="U21" s="36">
         <v>0.09</v>
       </c>
-      <c r="V21" s="51"/>
+      <c r="V21" s="46"/>
     </row>
     <row r="22" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="1"/>
       <c r="B22" s="26">
-        <f>ROW(B22) - ROW($B$9)</f>
+        <f t="shared" si="0"/>
         <v>13</v>
       </c>
-      <c r="C22" s="54" t="s">
-        <v>224</v>
+      <c r="C22" s="30" t="s">
+        <v>200</v>
       </c>
       <c r="D22" s="31" t="s">
-        <v>26</v>
-      </c>
-      <c r="E22" s="55" t="s">
-        <v>64</v>
+        <v>244</v>
+      </c>
+      <c r="E22" s="48" t="s">
+        <v>56</v>
       </c>
       <c r="F22" s="30" t="s">
-        <v>96</v>
+        <v>84</v>
       </c>
       <c r="G22" s="31" t="s">
-        <v>129</v>
+        <v>114</v>
       </c>
       <c r="H22" s="30" t="s">
-        <v>157</v>
+        <v>139</v>
       </c>
       <c r="I22" s="31"/>
       <c r="J22" s="30" t="s">
-        <v>183</v>
+        <v>163</v>
       </c>
       <c r="K22" s="31" t="s">
-        <v>249</v>
-      </c>
-      <c r="L22" s="54">
-        <v>1</v>
+        <v>225</v>
+      </c>
+      <c r="L22" s="47">
+        <v>3</v>
       </c>
       <c r="M22" s="32">
-        <f>L22*5</f>
-        <v>5</v>
+        <f t="shared" ref="M22" si="6">L22*5</f>
+        <v>15</v>
       </c>
       <c r="N22" s="31">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="O22" s="30">
-        <v>10</v>
-      </c>
-      <c r="P22" s="77">
-        <v>10</v>
-      </c>
-      <c r="Q22" s="82" t="s">
-        <v>247</v>
+        <v>30</v>
+      </c>
+      <c r="P22" s="67">
+        <v>40</v>
+      </c>
+      <c r="Q22" s="68" t="s">
+        <v>223</v>
       </c>
       <c r="R22" s="35">
-        <v>6.1699999999999998E-2</v>
+        <v>2.2800000000000001E-2</v>
       </c>
       <c r="S22" s="35">
-        <v>0.31</v>
+        <v>0.46</v>
       </c>
       <c r="T22" s="35">
-        <v>6.1699999999999998E-2</v>
+        <v>2.2800000000000001E-2</v>
       </c>
       <c r="U22" s="35">
-        <v>0.62</v>
+        <v>0.91</v>
       </c>
       <c r="V22" s="32"/>
     </row>
     <row r="23" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="1"/>
       <c r="B23" s="26">
-        <f t="shared" si="0"/>
+        <f>ROW(B23) - ROW($B$9)</f>
         <v>14</v>
       </c>
       <c r="C23" s="33" t="s">
-        <v>224</v>
+        <v>201</v>
       </c>
       <c r="D23" s="34" t="s">
-        <v>27</v>
-      </c>
-      <c r="E23" s="48" t="s">
-        <v>65</v>
+        <v>29</v>
+      </c>
+      <c r="E23" s="43" t="s">
+        <v>61</v>
       </c>
       <c r="F23" s="33" t="s">
-        <v>97</v>
-      </c>
-      <c r="G23" s="34" t="s">
-        <v>130</v>
+        <v>90</v>
+      </c>
+      <c r="G23" s="84">
+        <v>61300611121</v>
       </c>
       <c r="H23" s="33" t="s">
-        <v>158</v>
-      </c>
-      <c r="I23" s="34"/>
+        <v>138</v>
+      </c>
+      <c r="I23" s="34" t="s">
+        <v>230</v>
+      </c>
       <c r="J23" s="33" t="s">
-        <v>184</v>
+        <v>230</v>
       </c>
       <c r="K23" s="34" t="s">
-        <v>249</v>
+        <v>225</v>
       </c>
       <c r="L23" s="33">
-        <v>3</v>
-      </c>
-      <c r="M23" s="51">
-        <f t="shared" ref="M23" si="6">L23*5</f>
-        <v>15</v>
+        <v>1</v>
+      </c>
+      <c r="M23" s="46">
+        <f>L23*5</f>
+        <v>5</v>
       </c>
       <c r="N23" s="34">
         <v>20</v>
       </c>
-      <c r="O23" s="43">
-        <v>30</v>
-      </c>
-      <c r="P23" s="78">
-        <v>40</v>
-      </c>
-      <c r="Q23" s="83" t="s">
-        <v>247</v>
+      <c r="O23" s="33">
+        <v>10</v>
+      </c>
+      <c r="P23" s="66">
+        <v>20</v>
+      </c>
+      <c r="Q23" s="69" t="s">
+        <v>223</v>
       </c>
       <c r="R23" s="36">
-        <v>2.2800000000000001E-2</v>
+        <v>2.75E-2</v>
       </c>
       <c r="S23" s="36">
-        <v>0.46</v>
+        <v>0.55000000000000004</v>
       </c>
       <c r="T23" s="36">
-        <v>2.2800000000000001E-2</v>
+        <v>2.75E-2</v>
       </c>
       <c r="U23" s="36">
-        <v>0.91</v>
-      </c>
-      <c r="V23" s="51"/>
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="V23" s="46"/>
     </row>
     <row r="24" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="1"/>
@@ -3229,65 +3115,65 @@
         <f>ROW(B24) - ROW($B$9)</f>
         <v>15</v>
       </c>
-      <c r="C24" s="54" t="s">
+      <c r="C24" s="30" t="s">
+        <v>201</v>
+      </c>
+      <c r="D24" s="31" t="s">
+        <v>31</v>
+      </c>
+      <c r="E24" s="48" t="s">
+        <v>63</v>
+      </c>
+      <c r="F24" s="30" t="s">
+        <v>92</v>
+      </c>
+      <c r="G24" s="85">
+        <v>61300211121</v>
+      </c>
+      <c r="H24" s="30" t="s">
+        <v>138</v>
+      </c>
+      <c r="I24" s="31" t="s">
+        <v>231</v>
+      </c>
+      <c r="J24" s="30" t="s">
+        <v>232</v>
+      </c>
+      <c r="K24" s="31" t="s">
         <v>225</v>
       </c>
-      <c r="D24" s="47" t="s">
-        <v>33</v>
-      </c>
-      <c r="E24" s="65" t="s">
-        <v>70</v>
-      </c>
-      <c r="F24" s="54" t="s">
-        <v>103</v>
-      </c>
-      <c r="G24" s="91">
-        <v>61300611121</v>
-      </c>
-      <c r="H24" s="54" t="s">
-        <v>156</v>
-      </c>
-      <c r="I24" s="54" t="s">
-        <v>254</v>
-      </c>
-      <c r="J24" s="54" t="s">
-        <v>254</v>
-      </c>
-      <c r="K24" s="47" t="s">
-        <v>249</v>
-      </c>
-      <c r="L24" s="54">
+      <c r="L24" s="47">
         <v>1</v>
       </c>
-      <c r="M24" s="52">
-        <f>L24*5</f>
+      <c r="M24" s="32">
+        <f t="shared" ref="M24" si="7">L24*5</f>
         <v>5</v>
       </c>
-      <c r="N24" s="47">
-        <v>20</v>
-      </c>
-      <c r="O24" s="54">
+      <c r="N24" s="31">
+        <v>50</v>
+      </c>
+      <c r="O24" s="30">
         <v>10</v>
       </c>
-      <c r="P24" s="79">
-        <v>20</v>
-      </c>
-      <c r="Q24" s="82" t="s">
-        <v>247</v>
+      <c r="P24" s="67">
+        <v>50</v>
+      </c>
+      <c r="Q24" s="68" t="s">
+        <v>223</v>
       </c>
       <c r="R24" s="35">
-        <v>2.75E-2</v>
+        <v>1.38E-2</v>
       </c>
       <c r="S24" s="35">
-        <v>0.55000000000000004</v>
+        <v>0.69</v>
       </c>
       <c r="T24" s="35">
-        <v>2.75E-2</v>
+        <v>1.38E-2</v>
       </c>
       <c r="U24" s="35">
-        <v>0.55000000000000004</v>
-      </c>
-      <c r="V24" s="52"/>
+        <v>0.69</v>
+      </c>
+      <c r="V24" s="32"/>
     </row>
     <row r="25" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="1"/>
@@ -3296,101 +3182,99 @@
         <v>16</v>
       </c>
       <c r="C25" s="33" t="s">
+        <v>201</v>
+      </c>
+      <c r="D25" s="34" t="s">
+        <v>24</v>
+      </c>
+      <c r="E25" s="43" t="s">
+        <v>57</v>
+      </c>
+      <c r="F25" s="33" t="s">
+        <v>85</v>
+      </c>
+      <c r="G25" s="34" t="s">
+        <v>115</v>
+      </c>
+      <c r="H25" s="33" t="s">
+        <v>140</v>
+      </c>
+      <c r="I25" s="34"/>
+      <c r="J25" s="33" t="s">
+        <v>164</v>
+      </c>
+      <c r="K25" s="34" t="s">
         <v>225</v>
-      </c>
-      <c r="D25" s="34" t="s">
-        <v>35</v>
-      </c>
-      <c r="E25" s="48" t="s">
-        <v>72</v>
-      </c>
-      <c r="F25" s="33" t="s">
-        <v>105</v>
-      </c>
-      <c r="G25" s="92">
-        <v>61300211121</v>
-      </c>
-      <c r="H25" s="33" t="s">
-        <v>156</v>
-      </c>
-      <c r="I25" s="33" t="s">
-        <v>255</v>
-      </c>
-      <c r="J25" s="33" t="s">
-        <v>256</v>
-      </c>
-      <c r="K25" s="34" t="s">
-        <v>249</v>
       </c>
       <c r="L25" s="33">
         <v>1</v>
       </c>
-      <c r="M25" s="51">
-        <f t="shared" ref="M25" si="7">L25*5</f>
+      <c r="M25" s="46">
+        <f>L25*5</f>
         <v>5</v>
       </c>
       <c r="N25" s="34">
-        <v>50</v>
-      </c>
-      <c r="O25" s="41">
         <v>10</v>
       </c>
-      <c r="P25" s="80">
-        <v>50</v>
-      </c>
-      <c r="Q25" s="83" t="s">
-        <v>247</v>
+      <c r="O25" s="33">
+        <v>10</v>
+      </c>
+      <c r="P25" s="66">
+        <v>10</v>
+      </c>
+      <c r="Q25" s="69" t="s">
+        <v>223</v>
       </c>
       <c r="R25" s="36">
-        <v>1.38E-2</v>
+        <v>4.9399999999999999E-2</v>
       </c>
       <c r="S25" s="36">
-        <v>0.69</v>
+        <v>0.49</v>
       </c>
       <c r="T25" s="36">
-        <v>1.38E-2</v>
+        <v>4.9399999999999999E-2</v>
       </c>
       <c r="U25" s="36">
-        <v>0.69</v>
-      </c>
-      <c r="V25" s="51"/>
+        <v>0.49</v>
+      </c>
+      <c r="V25" s="46"/>
     </row>
     <row r="26" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="1"/>
       <c r="B26" s="26">
-        <f>ROW(B26) - ROW($B$9)</f>
+        <f t="shared" si="0"/>
         <v>17</v>
       </c>
-      <c r="C26" s="54" t="s">
-        <v>225</v>
+      <c r="C26" s="30" t="s">
+        <v>201</v>
       </c>
       <c r="D26" s="31" t="s">
-        <v>28</v>
-      </c>
-      <c r="E26" s="55" t="s">
-        <v>66</v>
+        <v>25</v>
+      </c>
+      <c r="E26" s="48" t="s">
+        <v>58</v>
       </c>
       <c r="F26" s="30" t="s">
-        <v>98</v>
+        <v>86</v>
       </c>
       <c r="G26" s="31" t="s">
-        <v>131</v>
+        <v>116</v>
       </c>
       <c r="H26" s="30" t="s">
-        <v>159</v>
+        <v>140</v>
       </c>
       <c r="I26" s="31"/>
       <c r="J26" s="30" t="s">
-        <v>185</v>
+        <v>165</v>
       </c>
       <c r="K26" s="31" t="s">
-        <v>249</v>
-      </c>
-      <c r="L26" s="54">
+        <v>225</v>
+      </c>
+      <c r="L26" s="47">
         <v>1</v>
       </c>
       <c r="M26" s="32">
-        <f>L26*5</f>
+        <f t="shared" ref="M26" si="8">L26*5</f>
         <v>5</v>
       </c>
       <c r="N26" s="31">
@@ -3399,279 +3283,279 @@
       <c r="O26" s="30">
         <v>10</v>
       </c>
-      <c r="P26" s="77">
+      <c r="P26" s="67">
         <v>10</v>
       </c>
-      <c r="Q26" s="82" t="s">
-        <v>247</v>
+      <c r="Q26" s="68" t="s">
+        <v>223</v>
       </c>
       <c r="R26" s="35">
-        <v>4.9399999999999999E-2</v>
+        <v>4.0599999999999997E-2</v>
       </c>
       <c r="S26" s="35">
-        <v>0.49</v>
+        <v>0.41</v>
       </c>
       <c r="T26" s="35">
-        <v>4.9399999999999999E-2</v>
+        <v>4.0599999999999997E-2</v>
       </c>
       <c r="U26" s="35">
-        <v>0.49</v>
+        <v>0.41</v>
       </c>
       <c r="V26" s="32"/>
     </row>
-    <row r="27" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:22" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="1"/>
       <c r="B27" s="26">
-        <f t="shared" si="0"/>
+        <f>ROW(B27) - ROW($B$9)</f>
         <v>18</v>
       </c>
       <c r="C27" s="33" t="s">
-        <v>225</v>
+        <v>9</v>
       </c>
       <c r="D27" s="34" t="s">
-        <v>29</v>
-      </c>
-      <c r="E27" s="48" t="s">
-        <v>67</v>
+        <v>26</v>
+      </c>
+      <c r="E27" s="43" t="s">
+        <v>59</v>
       </c>
       <c r="F27" s="33" t="s">
-        <v>99</v>
+        <v>87</v>
       </c>
       <c r="G27" s="34" t="s">
-        <v>132</v>
+        <v>87</v>
       </c>
       <c r="H27" s="33" t="s">
-        <v>159</v>
+        <v>136</v>
       </c>
       <c r="I27" s="34"/>
       <c r="J27" s="33" t="s">
-        <v>186</v>
+        <v>166</v>
       </c>
       <c r="K27" s="34" t="s">
-        <v>249</v>
+        <v>185</v>
       </c>
       <c r="L27" s="33">
         <v>1</v>
       </c>
-      <c r="M27" s="51">
-        <f t="shared" ref="M27" si="8">L27*5</f>
+      <c r="M27" s="46">
+        <f>L27*5</f>
         <v>5</v>
       </c>
       <c r="N27" s="34">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="O27" s="33">
         <v>10</v>
       </c>
-      <c r="P27" s="76">
+      <c r="P27" s="66">
         <v>10</v>
       </c>
-      <c r="Q27" s="83" t="s">
-        <v>247</v>
+      <c r="Q27" s="69" t="s">
+        <v>223</v>
       </c>
       <c r="R27" s="36">
-        <v>4.0599999999999997E-2</v>
+        <v>0.26819999999999999</v>
       </c>
       <c r="S27" s="36">
-        <v>0.41</v>
+        <v>1.34</v>
       </c>
       <c r="T27" s="36">
-        <v>4.0599999999999997E-2</v>
+        <v>0.26819999999999999</v>
       </c>
       <c r="U27" s="36">
-        <v>0.41</v>
-      </c>
-      <c r="V27" s="51"/>
+        <v>2.68</v>
+      </c>
+      <c r="V27" s="46"/>
     </row>
-    <row r="28" spans="1:22" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:22" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="1"/>
       <c r="B28" s="26">
-        <f>ROW(B28) - ROW($B$9)</f>
+        <f t="shared" si="0"/>
         <v>19</v>
       </c>
       <c r="C28" s="30" t="s">
-        <v>9</v>
+        <v>202</v>
       </c>
       <c r="D28" s="31" t="s">
-        <v>30</v>
-      </c>
-      <c r="E28" s="55" t="s">
-        <v>68</v>
+        <v>27</v>
+      </c>
+      <c r="E28" s="48" t="s">
+        <v>60</v>
       </c>
       <c r="F28" s="30" t="s">
-        <v>100</v>
+        <v>88</v>
       </c>
       <c r="G28" s="31" t="s">
-        <v>100</v>
+        <v>117</v>
       </c>
       <c r="H28" s="30" t="s">
-        <v>154</v>
+        <v>141</v>
       </c>
       <c r="I28" s="31"/>
       <c r="J28" s="30" t="s">
-        <v>187</v>
+        <v>167</v>
       </c>
       <c r="K28" s="31" t="s">
-        <v>208</v>
-      </c>
-      <c r="L28" s="54">
-        <v>1</v>
+        <v>186</v>
+      </c>
+      <c r="L28" s="47">
+        <v>2</v>
       </c>
       <c r="M28" s="32">
-        <f>L28*5</f>
-        <v>5</v>
+        <f t="shared" ref="M28" si="9">L28*5</f>
+        <v>10</v>
       </c>
       <c r="N28" s="31">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="O28" s="30">
-        <v>10</v>
-      </c>
-      <c r="P28" s="77">
-        <v>10</v>
-      </c>
-      <c r="Q28" s="82" t="s">
-        <v>247</v>
+        <v>20</v>
+      </c>
+      <c r="P28" s="67">
+        <v>20</v>
+      </c>
+      <c r="Q28" s="68" t="s">
+        <v>223</v>
       </c>
       <c r="R28" s="35">
-        <v>0.26819999999999999</v>
+        <v>7.3200000000000001E-2</v>
       </c>
       <c r="S28" s="35">
-        <v>1.34</v>
+        <v>0.73</v>
       </c>
       <c r="T28" s="35">
-        <v>0.26819999999999999</v>
+        <v>7.3200000000000001E-2</v>
       </c>
       <c r="U28" s="35">
-        <v>2.68</v>
+        <v>1.46</v>
       </c>
       <c r="V28" s="32"/>
     </row>
     <row r="29" spans="1:22" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="1"/>
       <c r="B29" s="26">
-        <f t="shared" si="0"/>
+        <f>ROW(B29) - ROW($B$9)</f>
         <v>20</v>
       </c>
       <c r="C29" s="33" t="s">
-        <v>226</v>
+        <v>10</v>
       </c>
       <c r="D29" s="34" t="s">
-        <v>31</v>
-      </c>
-      <c r="E29" s="48" t="s">
-        <v>69</v>
+        <v>32</v>
+      </c>
+      <c r="E29" s="43" t="s">
+        <v>64</v>
       </c>
       <c r="F29" s="33" t="s">
-        <v>101</v>
+        <v>93</v>
       </c>
       <c r="G29" s="34" t="s">
-        <v>133</v>
+        <v>118</v>
       </c>
       <c r="H29" s="33" t="s">
-        <v>160</v>
+        <v>142</v>
       </c>
       <c r="I29" s="34"/>
       <c r="J29" s="33" t="s">
-        <v>188</v>
+        <v>168</v>
       </c>
       <c r="K29" s="34" t="s">
-        <v>209</v>
+        <v>225</v>
       </c>
       <c r="L29" s="33">
-        <v>2</v>
-      </c>
-      <c r="M29" s="51">
-        <f t="shared" ref="M29" si="9">L29*5</f>
-        <v>10</v>
+        <v>6</v>
+      </c>
+      <c r="M29" s="46">
+        <f>L29*5</f>
+        <v>30</v>
       </c>
       <c r="N29" s="34">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="O29" s="33">
-        <v>20</v>
-      </c>
-      <c r="P29" s="76">
-        <v>20</v>
-      </c>
-      <c r="Q29" s="83" t="s">
-        <v>247</v>
+        <v>60</v>
+      </c>
+      <c r="P29" s="66">
+        <v>60</v>
+      </c>
+      <c r="Q29" s="69" t="s">
+        <v>223</v>
       </c>
       <c r="R29" s="36">
-        <v>7.3200000000000001E-2</v>
+        <v>0.1668</v>
       </c>
       <c r="S29" s="36">
-        <v>0.73</v>
+        <v>5</v>
       </c>
       <c r="T29" s="36">
-        <v>7.3200000000000001E-2</v>
+        <v>0.13439999999999999</v>
       </c>
       <c r="U29" s="36">
-        <v>1.46</v>
-      </c>
-      <c r="V29" s="51"/>
+        <v>8.06</v>
+      </c>
+      <c r="V29" s="46"/>
     </row>
-    <row r="30" spans="1:22" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="1"/>
       <c r="B30" s="26">
         <f>ROW(B30) - ROW($B$9)</f>
         <v>21</v>
       </c>
       <c r="C30" s="30" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D30" s="31" t="s">
-        <v>36</v>
-      </c>
-      <c r="E30" s="55" t="s">
-        <v>73</v>
+        <v>33</v>
+      </c>
+      <c r="E30" s="48" t="s">
+        <v>65</v>
       </c>
       <c r="F30" s="30" t="s">
-        <v>106</v>
+        <v>95</v>
       </c>
       <c r="G30" s="31" t="s">
-        <v>134</v>
+        <v>119</v>
       </c>
       <c r="H30" s="30" t="s">
-        <v>161</v>
+        <v>133</v>
       </c>
       <c r="I30" s="31"/>
       <c r="J30" s="30" t="s">
+        <v>169</v>
+      </c>
+      <c r="K30" s="31" t="s">
         <v>189</v>
       </c>
-      <c r="K30" s="31" t="s">
-        <v>249</v>
-      </c>
-      <c r="L30" s="54">
-        <v>6</v>
+      <c r="L30" s="47">
+        <v>3</v>
       </c>
       <c r="M30" s="32">
         <f>L30*5</f>
+        <v>15</v>
+      </c>
+      <c r="N30" s="31">
+        <v>100</v>
+      </c>
+      <c r="O30" s="30">
         <v>30</v>
       </c>
-      <c r="N30" s="31">
-        <v>30</v>
-      </c>
-      <c r="O30" s="30">
-        <v>60</v>
-      </c>
-      <c r="P30" s="77">
-        <v>60</v>
-      </c>
-      <c r="Q30" s="82" t="s">
-        <v>247</v>
+      <c r="P30" s="67">
+        <v>100</v>
+      </c>
+      <c r="Q30" s="68" t="s">
+        <v>223</v>
       </c>
       <c r="R30" s="35">
-        <v>0.1668</v>
+        <v>1.5E-3</v>
       </c>
       <c r="S30" s="35">
-        <v>5</v>
+        <v>0.15</v>
       </c>
       <c r="T30" s="35">
-        <v>0.13439999999999999</v>
+        <v>1.5E-3</v>
       </c>
       <c r="U30" s="35">
-        <v>8.06</v>
+        <v>0.15</v>
       </c>
       <c r="V30" s="32"/>
     </row>
@@ -3685,59 +3569,61 @@
         <v>11</v>
       </c>
       <c r="D31" s="34" t="s">
-        <v>37</v>
-      </c>
-      <c r="E31" s="48" t="s">
-        <v>74</v>
+        <v>34</v>
+      </c>
+      <c r="E31" s="43" t="s">
+        <v>66</v>
       </c>
       <c r="F31" s="33" t="s">
-        <v>107</v>
-      </c>
-      <c r="G31" s="34" t="s">
-        <v>135</v>
+        <v>96</v>
+      </c>
+      <c r="G31" s="87" t="s">
+        <v>120</v>
       </c>
       <c r="H31" s="33" t="s">
-        <v>151</v>
-      </c>
-      <c r="I31" s="34"/>
+        <v>143</v>
+      </c>
+      <c r="I31" s="34" t="s">
+        <v>234</v>
+      </c>
       <c r="J31" s="33" t="s">
+        <v>233</v>
+      </c>
+      <c r="K31" s="34" t="s">
         <v>190</v>
       </c>
-      <c r="K31" s="34" t="s">
-        <v>212</v>
-      </c>
       <c r="L31" s="33">
-        <v>2</v>
-      </c>
-      <c r="M31" s="51">
+        <v>6</v>
+      </c>
+      <c r="M31" s="46">
         <f t="shared" ref="M31" si="10">L31*5</f>
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="N31" s="34">
-        <v>100</v>
+        <v>40</v>
       </c>
       <c r="O31" s="33">
-        <v>20</v>
-      </c>
-      <c r="P31" s="76">
-        <v>100</v>
-      </c>
-      <c r="Q31" s="83" t="s">
-        <v>247</v>
+        <v>60</v>
+      </c>
+      <c r="P31" s="66">
+        <v>60</v>
+      </c>
+      <c r="Q31" s="69" t="s">
+        <v>223</v>
       </c>
       <c r="R31" s="36">
-        <v>1E-3</v>
+        <v>3.1600000000000003E-2</v>
       </c>
       <c r="S31" s="36">
-        <v>0.1</v>
+        <v>1.26</v>
       </c>
       <c r="T31" s="36">
-        <v>1E-3</v>
+        <v>3.1600000000000003E-2</v>
       </c>
       <c r="U31" s="36">
-        <v>0.1</v>
-      </c>
-      <c r="V31" s="51"/>
+        <v>1.9</v>
+      </c>
+      <c r="V31" s="46"/>
     </row>
     <row r="32" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="1"/>
@@ -3745,61 +3631,63 @@
         <f>ROW(B32) - ROW($B$9)</f>
         <v>23</v>
       </c>
-      <c r="C32" s="54" t="s">
+      <c r="C32" s="30" t="s">
         <v>11</v>
       </c>
       <c r="D32" s="31" t="s">
-        <v>38</v>
-      </c>
-      <c r="E32" s="55" t="s">
-        <v>75</v>
+        <v>245</v>
+      </c>
+      <c r="E32" s="48" t="s">
+        <v>67</v>
       </c>
       <c r="F32" s="30" t="s">
-        <v>108</v>
-      </c>
-      <c r="G32" s="31" t="s">
-        <v>136</v>
+        <v>96</v>
+      </c>
+      <c r="G32" s="85" t="s">
+        <v>121</v>
       </c>
       <c r="H32" s="30" t="s">
-        <v>151</v>
-      </c>
-      <c r="I32" s="31"/>
+        <v>144</v>
+      </c>
+      <c r="I32" s="31" t="s">
+        <v>235</v>
+      </c>
       <c r="J32" s="30" t="s">
+        <v>236</v>
+      </c>
+      <c r="K32" s="31" t="s">
         <v>191</v>
       </c>
-      <c r="K32" s="31" t="s">
-        <v>213</v>
-      </c>
-      <c r="L32" s="54">
-        <v>3</v>
+      <c r="L32" s="47">
+        <v>4</v>
       </c>
       <c r="M32" s="32">
         <f>L32*5</f>
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="N32" s="31">
         <v>100</v>
       </c>
       <c r="O32" s="30">
-        <v>30</v>
-      </c>
-      <c r="P32" s="77">
+        <v>40</v>
+      </c>
+      <c r="P32" s="67">
         <v>100</v>
       </c>
-      <c r="Q32" s="82" t="s">
-        <v>247</v>
+      <c r="Q32" s="68" t="s">
+        <v>223</v>
       </c>
       <c r="R32" s="35">
-        <v>1.5E-3</v>
+        <v>1.6999999999999999E-3</v>
       </c>
       <c r="S32" s="35">
-        <v>0.15</v>
+        <v>0.17</v>
       </c>
       <c r="T32" s="35">
-        <v>1.5E-3</v>
+        <v>1.6999999999999999E-3</v>
       </c>
       <c r="U32" s="35">
-        <v>0.15</v>
+        <v>0.17</v>
       </c>
       <c r="V32" s="32"/>
     </row>
@@ -3813,125 +3701,121 @@
         <v>11</v>
       </c>
       <c r="D33" s="34" t="s">
-        <v>39</v>
-      </c>
-      <c r="E33" s="48" t="s">
-        <v>76</v>
+        <v>35</v>
+      </c>
+      <c r="E33" s="43" t="s">
+        <v>68</v>
       </c>
       <c r="F33" s="33" t="s">
-        <v>109</v>
-      </c>
-      <c r="G33" s="92" t="s">
-        <v>137</v>
+        <v>94</v>
+      </c>
+      <c r="G33" s="34" t="s">
+        <v>122</v>
       </c>
       <c r="H33" s="33" t="s">
-        <v>162</v>
-      </c>
-      <c r="I33" s="33" t="s">
-        <v>258</v>
-      </c>
+        <v>145</v>
+      </c>
+      <c r="I33" s="34"/>
       <c r="J33" s="33" t="s">
-        <v>257</v>
-      </c>
-      <c r="K33" s="33" t="s">
-        <v>214</v>
+        <v>170</v>
+      </c>
+      <c r="K33" s="34" t="s">
+        <v>192</v>
       </c>
       <c r="L33" s="33">
-        <v>6</v>
-      </c>
-      <c r="M33" s="33">
+        <v>3</v>
+      </c>
+      <c r="M33" s="46">
         <f t="shared" ref="M33" si="11">L33*5</f>
+        <v>15</v>
+      </c>
+      <c r="N33" s="34">
+        <v>20</v>
+      </c>
+      <c r="O33" s="33">
         <v>30</v>
       </c>
-      <c r="N33" s="33">
+      <c r="P33" s="66">
         <v>40</v>
       </c>
-      <c r="O33" s="33">
-        <v>60</v>
-      </c>
-      <c r="P33" s="33">
-        <v>60</v>
-      </c>
-      <c r="Q33" s="83" t="s">
-        <v>247</v>
+      <c r="Q33" s="69" t="s">
+        <v>223</v>
       </c>
       <c r="R33" s="36">
-        <v>3.1600000000000003E-2</v>
+        <v>2.7900000000000001E-2</v>
       </c>
       <c r="S33" s="36">
-        <v>1.26</v>
+        <v>0.56000000000000005</v>
       </c>
       <c r="T33" s="36">
-        <v>3.1600000000000003E-2</v>
+        <v>2.7900000000000001E-2</v>
       </c>
       <c r="U33" s="36">
-        <v>1.9</v>
-      </c>
-      <c r="V33" s="51"/>
+        <v>1.1200000000000001</v>
+      </c>
+      <c r="V33" s="46"/>
     </row>
-    <row r="34" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:22" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="1"/>
       <c r="B34" s="26">
         <f>ROW(B34) - ROW($B$9)</f>
         <v>25</v>
       </c>
-      <c r="C34" s="54" t="s">
+      <c r="C34" s="30" t="s">
         <v>11</v>
       </c>
       <c r="D34" s="31" t="s">
-        <v>40</v>
-      </c>
-      <c r="E34" s="55" t="s">
-        <v>77</v>
+        <v>36</v>
+      </c>
+      <c r="E34" s="48" t="s">
+        <v>69</v>
       </c>
       <c r="F34" s="30" t="s">
-        <v>109</v>
-      </c>
-      <c r="G34" s="91" t="s">
-        <v>138</v>
+        <v>94</v>
+      </c>
+      <c r="G34" s="31" t="s">
+        <v>123</v>
       </c>
       <c r="H34" s="30" t="s">
-        <v>163</v>
-      </c>
-      <c r="I34" s="31" t="s">
-        <v>259</v>
-      </c>
+        <v>146</v>
+      </c>
+      <c r="I34" s="31"/>
       <c r="J34" s="30" t="s">
-        <v>260</v>
+        <v>171</v>
       </c>
       <c r="K34" s="31" t="s">
-        <v>215</v>
-      </c>
-      <c r="L34" s="54">
-        <v>4</v>
+        <v>193</v>
+      </c>
+      <c r="L34" s="47">
+        <v>3</v>
       </c>
       <c r="M34" s="32">
         <f>L34*5</f>
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="N34" s="31">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="O34" s="30">
-        <v>40</v>
-      </c>
-      <c r="P34" s="77">
-        <v>100</v>
-      </c>
-      <c r="Q34" s="82" t="s">
-        <v>247</v>
+        <v>30</v>
+      </c>
+      <c r="P34" s="67">
+        <v>50</v>
+      </c>
+      <c r="Q34" s="68" t="s">
+        <v>223</v>
       </c>
       <c r="R34" s="35">
-        <v>1.6999999999999999E-3</v>
+        <v>7.1999999999999998E-3</v>
       </c>
       <c r="S34" s="35">
-        <v>0.17</v>
+        <v>0.36</v>
       </c>
       <c r="T34" s="35">
-        <v>1.6999999999999999E-3</v>
+        <v>7.1999999999999998E-3</v>
       </c>
       <c r="U34" s="35">
-        <v>0.17</v>
+        <v>0.36</v>
       </c>
       <c r="V34" s="32"/>
     </row>
@@ -3945,61 +3829,61 @@
         <v>11</v>
       </c>
       <c r="D35" s="34" t="s">
-        <v>41</v>
-      </c>
-      <c r="E35" s="48" t="s">
-        <v>78</v>
+        <v>37</v>
+      </c>
+      <c r="E35" s="43" t="s">
+        <v>70</v>
       </c>
       <c r="F35" s="33" t="s">
-        <v>107</v>
+        <v>94</v>
       </c>
       <c r="G35" s="34" t="s">
-        <v>139</v>
+        <v>124</v>
       </c>
       <c r="H35" s="33" t="s">
-        <v>164</v>
-      </c>
-      <c r="I35" s="33"/>
+        <v>133</v>
+      </c>
+      <c r="I35" s="34"/>
       <c r="J35" s="33" t="s">
-        <v>192</v>
+        <v>172</v>
       </c>
       <c r="K35" s="34" t="s">
-        <v>216</v>
+        <v>194</v>
       </c>
       <c r="L35" s="33">
-        <v>3</v>
-      </c>
-      <c r="M35" s="51">
+        <v>1</v>
+      </c>
+      <c r="M35" s="46">
         <f t="shared" ref="M35" si="12">L35*5</f>
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="N35" s="34">
-        <v>20</v>
+        <v>50</v>
       </c>
       <c r="O35" s="33">
-        <v>30</v>
-      </c>
-      <c r="P35" s="76">
-        <v>40</v>
-      </c>
-      <c r="Q35" s="83" t="s">
-        <v>247</v>
+        <v>10</v>
+      </c>
+      <c r="P35" s="66">
+        <v>50</v>
+      </c>
+      <c r="Q35" s="69" t="s">
+        <v>223</v>
       </c>
       <c r="R35" s="36">
-        <v>2.7900000000000001E-2</v>
+        <v>1.1599999999999999E-2</v>
       </c>
       <c r="S35" s="36">
-        <v>0.56000000000000005</v>
+        <v>0.57999999999999996</v>
       </c>
       <c r="T35" s="36">
-        <v>2.7900000000000001E-2</v>
+        <v>1.1599999999999999E-2</v>
       </c>
       <c r="U35" s="36">
-        <v>1.1200000000000001</v>
-      </c>
-      <c r="V35" s="51"/>
+        <v>0.57999999999999996</v>
+      </c>
+      <c r="V35" s="46"/>
     </row>
-    <row r="36" spans="1:22" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A36" s="1"/>
       <c r="B36" s="26">
         <f>ROW(B36) - ROW($B$9)</f>
@@ -4009,61 +3893,63 @@
         <v>11</v>
       </c>
       <c r="D36" s="31" t="s">
-        <v>42</v>
-      </c>
-      <c r="E36" s="55" t="s">
-        <v>79</v>
+        <v>38</v>
+      </c>
+      <c r="E36" s="48" t="s">
+        <v>71</v>
       </c>
       <c r="F36" s="30" t="s">
-        <v>107</v>
-      </c>
-      <c r="G36" s="31" t="s">
-        <v>140</v>
+        <v>97</v>
+      </c>
+      <c r="G36" s="85" t="s">
+        <v>125</v>
       </c>
       <c r="H36" s="30" t="s">
-        <v>165</v>
-      </c>
-      <c r="I36" s="31"/>
+        <v>147</v>
+      </c>
+      <c r="I36" s="31" t="s">
+        <v>237</v>
+      </c>
       <c r="J36" s="30" t="s">
-        <v>193</v>
+        <v>238</v>
       </c>
       <c r="K36" s="31" t="s">
-        <v>217</v>
-      </c>
-      <c r="L36" s="54">
-        <v>3</v>
+        <v>195</v>
+      </c>
+      <c r="L36" s="47">
+        <v>1</v>
       </c>
       <c r="M36" s="32">
         <f>L36*5</f>
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="N36" s="31">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="O36" s="30">
-        <v>30</v>
-      </c>
-      <c r="P36" s="77">
-        <v>50</v>
-      </c>
-      <c r="Q36" s="82" t="s">
-        <v>247</v>
+        <v>10</v>
+      </c>
+      <c r="P36" s="67">
+        <v>100</v>
+      </c>
+      <c r="Q36" s="68" t="s">
+        <v>223</v>
       </c>
       <c r="R36" s="35">
-        <v>7.1999999999999998E-3</v>
+        <v>5.9999999999999995E-4</v>
       </c>
       <c r="S36" s="35">
-        <v>0.36</v>
+        <v>0.06</v>
       </c>
       <c r="T36" s="35">
-        <v>7.1999999999999998E-3</v>
+        <v>5.9999999999999995E-4</v>
       </c>
       <c r="U36" s="35">
-        <v>0.36</v>
+        <v>0.06</v>
       </c>
       <c r="V36" s="32"/>
     </row>
-    <row r="37" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:22" ht="36.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A37" s="1"/>
       <c r="B37" s="26">
         <f t="shared" si="0"/>
@@ -4073,59 +3959,59 @@
         <v>11</v>
       </c>
       <c r="D37" s="34" t="s">
-        <v>43</v>
-      </c>
-      <c r="E37" s="48" t="s">
-        <v>80</v>
+        <v>39</v>
+      </c>
+      <c r="E37" s="43" t="s">
+        <v>72</v>
       </c>
       <c r="F37" s="33" t="s">
-        <v>107</v>
+        <v>98</v>
       </c>
       <c r="G37" s="34" t="s">
-        <v>141</v>
+        <v>126</v>
       </c>
       <c r="H37" s="33" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="I37" s="34"/>
       <c r="J37" s="33" t="s">
-        <v>194</v>
+        <v>173</v>
       </c>
       <c r="K37" s="34" t="s">
-        <v>218</v>
+        <v>196</v>
       </c>
       <c r="L37" s="33">
         <v>1</v>
       </c>
-      <c r="M37" s="51">
+      <c r="M37" s="46">
         <f t="shared" ref="M37" si="13">L37*5</f>
         <v>5</v>
       </c>
       <c r="N37" s="34">
-        <v>50</v>
+        <v>10</v>
       </c>
       <c r="O37" s="33">
         <v>10</v>
       </c>
-      <c r="P37" s="76">
-        <v>50</v>
-      </c>
-      <c r="Q37" s="83" t="s">
-        <v>247</v>
+      <c r="P37" s="66">
+        <v>10</v>
+      </c>
+      <c r="Q37" s="69" t="s">
+        <v>223</v>
       </c>
       <c r="R37" s="36">
-        <v>1.1599999999999999E-2</v>
+        <v>6.4399999999999999E-2</v>
       </c>
       <c r="S37" s="36">
-        <v>0.57999999999999996</v>
+        <v>0.64</v>
       </c>
       <c r="T37" s="36">
-        <v>1.1599999999999999E-2</v>
+        <v>6.4399999999999999E-2</v>
       </c>
       <c r="U37" s="36">
-        <v>0.57999999999999996</v>
-      </c>
-      <c r="V37" s="51"/>
+        <v>0.64</v>
+      </c>
+      <c r="V37" s="46"/>
     </row>
     <row r="38" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A38" s="1"/>
@@ -4137,30 +4023,28 @@
         <v>11</v>
       </c>
       <c r="D38" s="31" t="s">
-        <v>44</v>
-      </c>
-      <c r="E38" s="55" t="s">
-        <v>81</v>
+        <v>246</v>
+      </c>
+      <c r="E38" s="48" t="s">
+        <v>73</v>
       </c>
       <c r="F38" s="30" t="s">
-        <v>110</v>
-      </c>
-      <c r="G38" s="91" t="s">
-        <v>142</v>
+        <v>94</v>
+      </c>
+      <c r="G38" s="31" t="s">
+        <v>127</v>
       </c>
       <c r="H38" s="30" t="s">
-        <v>166</v>
-      </c>
-      <c r="I38" s="31" t="s">
-        <v>261</v>
-      </c>
+        <v>133</v>
+      </c>
+      <c r="I38" s="31"/>
       <c r="J38" s="30" t="s">
-        <v>262</v>
+        <v>174</v>
       </c>
       <c r="K38" s="31" t="s">
-        <v>219</v>
-      </c>
-      <c r="L38" s="54">
+        <v>197</v>
+      </c>
+      <c r="L38" s="47">
         <v>1</v>
       </c>
       <c r="M38" s="32">
@@ -4173,718 +4057,507 @@
       <c r="O38" s="30">
         <v>10</v>
       </c>
-      <c r="P38" s="77">
+      <c r="P38" s="67">
         <v>100</v>
       </c>
-      <c r="Q38" s="82" t="s">
-        <v>247</v>
+      <c r="Q38" s="68" t="s">
+        <v>223</v>
       </c>
       <c r="R38" s="35">
-        <v>5.9999999999999995E-4</v>
+        <v>1.1999999999999999E-3</v>
       </c>
       <c r="S38" s="35">
-        <v>0.06</v>
+        <v>0.12</v>
       </c>
       <c r="T38" s="35">
-        <v>5.9999999999999995E-4</v>
+        <v>1.1999999999999999E-3</v>
       </c>
       <c r="U38" s="35">
-        <v>0.06</v>
+        <v>0.12</v>
       </c>
       <c r="V38" s="32"/>
     </row>
-    <row r="39" spans="1:22" ht="36.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A39" s="1"/>
       <c r="B39" s="26">
-        <f t="shared" si="0"/>
+        <f>ROW(B39) - ROW($B$9)</f>
         <v>30</v>
       </c>
       <c r="C39" s="33" t="s">
-        <v>11</v>
+        <v>203</v>
       </c>
       <c r="D39" s="34" t="s">
-        <v>45</v>
-      </c>
-      <c r="E39" s="48" t="s">
-        <v>82</v>
+        <v>28</v>
+      </c>
+      <c r="E39" s="43" t="s">
+        <v>224</v>
       </c>
       <c r="F39" s="33" t="s">
-        <v>111</v>
+        <v>89</v>
       </c>
       <c r="G39" s="34" t="s">
-        <v>143</v>
+        <v>225</v>
       </c>
       <c r="H39" s="33" t="s">
-        <v>167</v>
+        <v>225</v>
       </c>
       <c r="I39" s="34"/>
       <c r="J39" s="33" t="s">
-        <v>195</v>
+        <v>225</v>
       </c>
       <c r="K39" s="34" t="s">
-        <v>220</v>
-      </c>
-      <c r="L39" s="33">
-        <v>1</v>
-      </c>
-      <c r="M39" s="51">
-        <f t="shared" ref="M39" si="14">L39*5</f>
-        <v>5</v>
-      </c>
-      <c r="N39" s="34">
-        <v>10</v>
-      </c>
-      <c r="O39" s="33">
-        <v>10</v>
-      </c>
-      <c r="P39" s="76">
-        <v>10</v>
-      </c>
-      <c r="Q39" s="83" t="s">
-        <v>247</v>
-      </c>
-      <c r="R39" s="36">
-        <v>6.4399999999999999E-2</v>
-      </c>
-      <c r="S39" s="36">
-        <v>0.64</v>
-      </c>
-      <c r="T39" s="36">
-        <v>6.4399999999999999E-2</v>
-      </c>
-      <c r="U39" s="36">
-        <v>0.64</v>
-      </c>
-      <c r="V39" s="51"/>
+        <v>187</v>
+      </c>
+      <c r="L39" s="33" t="s">
+        <v>225</v>
+      </c>
+      <c r="M39" s="46" t="s">
+        <v>225</v>
+      </c>
+      <c r="N39" s="34" t="s">
+        <v>225</v>
+      </c>
+      <c r="O39" s="33" t="s">
+        <v>225</v>
+      </c>
+      <c r="P39" s="66" t="s">
+        <v>225</v>
+      </c>
+      <c r="Q39" s="69" t="s">
+        <v>225</v>
+      </c>
+      <c r="R39" s="36" t="s">
+        <v>225</v>
+      </c>
+      <c r="S39" s="36" t="s">
+        <v>225</v>
+      </c>
+      <c r="T39" s="36" t="s">
+        <v>225</v>
+      </c>
+      <c r="U39" s="36" t="s">
+        <v>225</v>
+      </c>
+      <c r="V39" s="46"/>
     </row>
-    <row r="40" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:22" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A40" s="1"/>
       <c r="B40" s="26">
         <f>ROW(B40) - ROW($B$9)</f>
         <v>31</v>
       </c>
       <c r="C40" s="30" t="s">
-        <v>11</v>
+        <v>204</v>
       </c>
       <c r="D40" s="31" t="s">
-        <v>46</v>
-      </c>
-      <c r="E40" s="55" t="s">
-        <v>83</v>
+        <v>30</v>
+      </c>
+      <c r="E40" s="48" t="s">
+        <v>62</v>
       </c>
       <c r="F40" s="30" t="s">
-        <v>107</v>
+        <v>91</v>
       </c>
       <c r="G40" s="31" t="s">
-        <v>144</v>
+        <v>225</v>
       </c>
       <c r="H40" s="30" t="s">
-        <v>151</v>
+        <v>225</v>
       </c>
       <c r="I40" s="31"/>
       <c r="J40" s="30" t="s">
-        <v>196</v>
+        <v>225</v>
       </c>
       <c r="K40" s="31" t="s">
-        <v>221</v>
-      </c>
-      <c r="L40" s="54">
-        <v>1</v>
-      </c>
-      <c r="M40" s="32">
-        <f>L40*5</f>
-        <v>5</v>
-      </c>
-      <c r="N40" s="31">
-        <v>100</v>
-      </c>
-      <c r="O40" s="30">
-        <v>10</v>
-      </c>
-      <c r="P40" s="77">
-        <v>100</v>
-      </c>
-      <c r="Q40" s="82" t="s">
-        <v>247</v>
-      </c>
-      <c r="R40" s="35">
-        <v>1.1999999999999999E-3</v>
-      </c>
-      <c r="S40" s="35">
-        <v>0.12</v>
-      </c>
-      <c r="T40" s="35">
-        <v>1.1999999999999999E-3</v>
-      </c>
-      <c r="U40" s="35">
-        <v>0.12</v>
+        <v>188</v>
+      </c>
+      <c r="L40" s="47" t="s">
+        <v>225</v>
+      </c>
+      <c r="M40" s="32" t="s">
+        <v>225</v>
+      </c>
+      <c r="N40" s="31" t="s">
+        <v>225</v>
+      </c>
+      <c r="O40" s="30" t="s">
+        <v>225</v>
+      </c>
+      <c r="P40" s="67" t="s">
+        <v>225</v>
+      </c>
+      <c r="Q40" s="68" t="s">
+        <v>225</v>
+      </c>
+      <c r="R40" s="35" t="s">
+        <v>225</v>
+      </c>
+      <c r="S40" s="35" t="s">
+        <v>225</v>
+      </c>
+      <c r="T40" s="35" t="s">
+        <v>225</v>
+      </c>
+      <c r="U40" s="35" t="s">
+        <v>225</v>
       </c>
       <c r="V40" s="32"/>
     </row>
-    <row r="41" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:22" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A41" s="1"/>
       <c r="B41" s="26">
-        <f t="shared" si="0"/>
+        <f>ROW(B41) - ROW($B$9)</f>
         <v>32</v>
       </c>
       <c r="C41" s="33" t="s">
-        <v>112</v>
+        <v>205</v>
       </c>
       <c r="D41" s="34" t="s">
-        <v>47</v>
-      </c>
-      <c r="E41" s="48" t="s">
-        <v>84</v>
+        <v>40</v>
+      </c>
+      <c r="E41" s="43" t="s">
+        <v>74</v>
       </c>
       <c r="F41" s="33" t="s">
-        <v>112</v>
+        <v>99</v>
       </c>
       <c r="G41" s="34" t="s">
-        <v>249</v>
+        <v>128</v>
       </c>
       <c r="H41" s="33" t="s">
-        <v>249</v>
+        <v>149</v>
       </c>
       <c r="I41" s="34"/>
       <c r="J41" s="33" t="s">
-        <v>249</v>
+        <v>175</v>
       </c>
       <c r="K41" s="34" t="s">
-        <v>112</v>
-      </c>
-      <c r="L41" s="33" t="s">
-        <v>249</v>
-      </c>
-      <c r="M41" s="51" t="s">
-        <v>249</v>
-      </c>
-      <c r="N41" s="34" t="s">
-        <v>249</v>
-      </c>
-      <c r="O41" s="33" t="s">
-        <v>249</v>
-      </c>
-      <c r="P41" s="76" t="s">
-        <v>249</v>
-      </c>
-      <c r="Q41" s="45" t="s">
-        <v>249</v>
-      </c>
-      <c r="R41" s="36" t="s">
-        <v>249</v>
-      </c>
-      <c r="S41" s="36" t="s">
-        <v>249</v>
-      </c>
-      <c r="T41" s="36" t="s">
-        <v>249</v>
-      </c>
-      <c r="U41" s="36" t="s">
-        <v>249</v>
-      </c>
-      <c r="V41" s="51"/>
+        <v>225</v>
+      </c>
+      <c r="L41" s="33">
+        <v>1</v>
+      </c>
+      <c r="M41" s="46">
+        <f>L41*5</f>
+        <v>5</v>
+      </c>
+      <c r="N41" s="34">
+        <v>10</v>
+      </c>
+      <c r="O41" s="33">
+        <v>10</v>
+      </c>
+      <c r="P41" s="66">
+        <v>10</v>
+      </c>
+      <c r="Q41" s="69" t="s">
+        <v>223</v>
+      </c>
+      <c r="R41" s="36">
+        <v>5.8200000000000002E-2</v>
+      </c>
+      <c r="S41" s="36">
+        <v>0.57999999999999996</v>
+      </c>
+      <c r="T41" s="36">
+        <v>5.8200000000000002E-2</v>
+      </c>
+      <c r="U41" s="36">
+        <v>0.57999999999999996</v>
+      </c>
+      <c r="V41" s="46"/>
     </row>
-    <row r="42" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:22" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A42" s="1"/>
       <c r="B42" s="26">
-        <f>ROW(B42) - ROW($B$9)</f>
+        <f t="shared" si="0"/>
         <v>33</v>
       </c>
       <c r="C42" s="30" t="s">
-        <v>227</v>
+        <v>12</v>
       </c>
       <c r="D42" s="31" t="s">
-        <v>32</v>
-      </c>
-      <c r="E42" s="55" t="s">
-        <v>248</v>
+        <v>41</v>
+      </c>
+      <c r="E42" s="48" t="s">
+        <v>75</v>
       </c>
       <c r="F42" s="30" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="G42" s="31" t="s">
-        <v>249</v>
+        <v>129</v>
       </c>
       <c r="H42" s="30" t="s">
-        <v>249</v>
+        <v>150</v>
       </c>
       <c r="I42" s="31"/>
-      <c r="J42" s="30" t="s">
-        <v>249</v>
-      </c>
+      <c r="J42" s="30"/>
       <c r="K42" s="31" t="s">
-        <v>210</v>
-      </c>
-      <c r="L42" s="54" t="s">
-        <v>249</v>
-      </c>
-      <c r="M42" s="32" t="s">
-        <v>249</v>
-      </c>
-      <c r="N42" s="31" t="s">
-        <v>249</v>
-      </c>
-      <c r="O42" s="30" t="s">
-        <v>249</v>
-      </c>
-      <c r="P42" s="77" t="s">
-        <v>249</v>
-      </c>
-      <c r="Q42" s="44" t="s">
-        <v>249</v>
-      </c>
-      <c r="R42" s="35" t="s">
-        <v>249</v>
-      </c>
-      <c r="S42" s="35" t="s">
-        <v>249</v>
-      </c>
-      <c r="T42" s="35" t="s">
-        <v>249</v>
-      </c>
-      <c r="U42" s="35" t="s">
-        <v>249</v>
-      </c>
+        <v>225</v>
+      </c>
+      <c r="L42" s="47">
+        <v>1</v>
+      </c>
+      <c r="M42" s="32">
+        <f t="shared" ref="M42:M43" si="14">L42*5</f>
+        <v>5</v>
+      </c>
+      <c r="N42" s="31"/>
+      <c r="O42" s="30"/>
+      <c r="P42" s="67"/>
+      <c r="Q42" s="68"/>
+      <c r="R42" s="35"/>
+      <c r="S42" s="35"/>
+      <c r="T42" s="35"/>
+      <c r="U42" s="35"/>
       <c r="V42" s="32"/>
     </row>
-    <row r="43" spans="1:22" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A43" s="1"/>
+    <row r="43" spans="1:22" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A43" s="86"/>
       <c r="B43" s="26">
-        <f>ROW(B43) - ROW($B$9)</f>
+        <f t="shared" si="0"/>
         <v>34</v>
       </c>
       <c r="C43" s="33" t="s">
-        <v>228</v>
+        <v>12</v>
       </c>
       <c r="D43" s="34" t="s">
-        <v>34</v>
-      </c>
-      <c r="E43" s="48" t="s">
-        <v>71</v>
+        <v>42</v>
+      </c>
+      <c r="E43" s="43" t="s">
+        <v>247</v>
       </c>
       <c r="F43" s="33" t="s">
-        <v>104</v>
+        <v>248</v>
       </c>
       <c r="G43" s="34" t="s">
         <v>249</v>
       </c>
       <c r="H43" s="33" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="I43" s="34"/>
-      <c r="J43" s="33" t="s">
-        <v>249</v>
-      </c>
+      <c r="J43" s="33"/>
       <c r="K43" s="34" t="s">
-        <v>211</v>
-      </c>
-      <c r="L43" s="33" t="s">
-        <v>249</v>
-      </c>
-      <c r="M43" s="51" t="s">
-        <v>249</v>
-      </c>
-      <c r="N43" s="34" t="s">
-        <v>249</v>
-      </c>
-      <c r="O43" s="33" t="s">
-        <v>249</v>
-      </c>
-      <c r="P43" s="76" t="s">
-        <v>249</v>
-      </c>
-      <c r="Q43" s="45" t="s">
-        <v>249</v>
-      </c>
-      <c r="R43" s="33" t="s">
-        <v>249</v>
-      </c>
-      <c r="S43" s="33" t="s">
-        <v>249</v>
-      </c>
-      <c r="T43" s="33" t="s">
-        <v>249</v>
-      </c>
-      <c r="U43" s="33" t="s">
-        <v>249</v>
-      </c>
-      <c r="V43" s="51"/>
+        <v>225</v>
+      </c>
+      <c r="L43" s="33">
+        <v>1</v>
+      </c>
+      <c r="M43" s="46">
+        <f t="shared" si="14"/>
+        <v>5</v>
+      </c>
+      <c r="N43" s="34"/>
+      <c r="O43" s="33"/>
+      <c r="P43" s="66"/>
+      <c r="Q43" s="69"/>
+      <c r="R43" s="36"/>
+      <c r="S43" s="36"/>
+      <c r="T43" s="36"/>
+      <c r="U43" s="36"/>
+      <c r="V43" s="46"/>
     </row>
-    <row r="44" spans="1:22" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A44" s="1"/>
       <c r="B44" s="26">
-        <f>ROW(B44) - ROW($B$9)</f>
+        <f t="shared" si="0"/>
         <v>35</v>
       </c>
       <c r="C44" s="30" t="s">
-        <v>229</v>
+        <v>12</v>
       </c>
       <c r="D44" s="31" t="s">
-        <v>48</v>
-      </c>
-      <c r="E44" s="55" t="s">
-        <v>85</v>
+        <v>43</v>
+      </c>
+      <c r="E44" s="48" t="s">
+        <v>76</v>
       </c>
       <c r="F44" s="30" t="s">
-        <v>113</v>
+        <v>101</v>
       </c>
       <c r="G44" s="31" t="s">
-        <v>145</v>
+        <v>130</v>
       </c>
       <c r="H44" s="30" t="s">
-        <v>168</v>
+        <v>151</v>
       </c>
       <c r="I44" s="31"/>
       <c r="J44" s="30" t="s">
-        <v>197</v>
+        <v>239</v>
       </c>
       <c r="K44" s="31" t="s">
-        <v>249</v>
-      </c>
-      <c r="L44" s="54">
+        <v>225</v>
+      </c>
+      <c r="L44" s="47">
         <v>1</v>
       </c>
       <c r="M44" s="32">
-        <f>L44*5</f>
+        <f t="shared" ref="M44" si="15">L44*5</f>
         <v>5</v>
       </c>
       <c r="N44" s="31">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="O44" s="30">
         <v>10</v>
       </c>
-      <c r="P44" s="77">
+      <c r="P44" s="67">
         <v>10</v>
       </c>
-      <c r="Q44" s="82" t="s">
-        <v>247</v>
+      <c r="Q44" s="68" t="s">
+        <v>223</v>
       </c>
       <c r="R44" s="35">
-        <v>5.8200000000000002E-2</v>
+        <v>1.2198</v>
       </c>
       <c r="S44" s="35">
-        <v>0.57999999999999996</v>
+        <v>6.1</v>
       </c>
       <c r="T44" s="35">
-        <v>5.8200000000000002E-2</v>
+        <v>1.0928</v>
       </c>
       <c r="U44" s="35">
-        <v>0.57999999999999996</v>
+        <v>10.93</v>
       </c>
       <c r="V44" s="32"/>
     </row>
     <row r="45" spans="1:22" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A45" s="1"/>
       <c r="B45" s="26">
-        <f t="shared" si="0"/>
+        <f>ROW(B45) - ROW($B$9)</f>
         <v>36</v>
       </c>
       <c r="C45" s="33" t="s">
         <v>12</v>
       </c>
       <c r="D45" s="34" t="s">
-        <v>49</v>
-      </c>
-      <c r="E45" s="48" t="s">
-        <v>86</v>
+        <v>44</v>
+      </c>
+      <c r="E45" s="43" t="s">
+        <v>77</v>
       </c>
       <c r="F45" s="33" t="s">
-        <v>114</v>
+        <v>102</v>
       </c>
       <c r="G45" s="34" t="s">
-        <v>146</v>
+        <v>131</v>
       </c>
       <c r="H45" s="33" t="s">
-        <v>169</v>
+        <v>152</v>
       </c>
       <c r="I45" s="34"/>
-      <c r="J45" s="33"/>
+      <c r="J45" s="33" t="s">
+        <v>176</v>
+      </c>
       <c r="K45" s="34" t="s">
-        <v>249</v>
+        <v>225</v>
       </c>
       <c r="L45" s="33">
         <v>1</v>
       </c>
-      <c r="M45" s="51">
-        <f t="shared" ref="M45" si="15">L45*5</f>
+      <c r="M45" s="46">
+        <f>L45*5</f>
         <v>5</v>
       </c>
-      <c r="N45" s="34"/>
-      <c r="O45" s="33"/>
-      <c r="P45" s="76"/>
-      <c r="Q45" s="45" t="s">
-        <v>247</v>
-      </c>
-      <c r="R45" s="36"/>
-      <c r="S45" s="36"/>
-      <c r="T45" s="36"/>
-      <c r="U45" s="36"/>
-      <c r="V45" s="51"/>
+      <c r="N45" s="34">
+        <v>5</v>
+      </c>
+      <c r="O45" s="33">
+        <v>10</v>
+      </c>
+      <c r="P45" s="66">
+        <v>10</v>
+      </c>
+      <c r="Q45" s="69" t="s">
+        <v>223</v>
+      </c>
+      <c r="R45" s="36">
+        <v>6.83E-2</v>
+      </c>
+      <c r="S45" s="36">
+        <v>0.34</v>
+      </c>
+      <c r="T45" s="36">
+        <v>6.83E-2</v>
+      </c>
+      <c r="U45" s="36">
+        <v>0.68</v>
+      </c>
+      <c r="V45" s="46"/>
     </row>
-    <row r="46" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:22" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A46" s="1"/>
-      <c r="B46" s="26">
-        <f>ROW(B46) - ROW($B$9)</f>
-        <v>37</v>
-      </c>
-      <c r="C46" s="30" t="s">
-        <v>12</v>
-      </c>
-      <c r="D46" s="31" t="s">
-        <v>50</v>
-      </c>
-      <c r="E46" s="55" t="s">
-        <v>87</v>
-      </c>
-      <c r="F46" s="30" t="s">
-        <v>115</v>
-      </c>
-      <c r="G46" s="31" t="s">
-        <v>147</v>
-      </c>
-      <c r="H46" s="30" t="s">
-        <v>170</v>
-      </c>
-      <c r="I46" s="31"/>
-      <c r="J46" s="30" t="s">
-        <v>198</v>
-      </c>
-      <c r="K46" s="31" t="s">
-        <v>249</v>
-      </c>
-      <c r="L46" s="54">
-        <v>1</v>
-      </c>
-      <c r="M46" s="32">
-        <f>L46*5</f>
-        <v>5</v>
-      </c>
-      <c r="N46" s="31">
-        <v>5</v>
-      </c>
-      <c r="O46" s="30">
-        <v>10</v>
-      </c>
-      <c r="P46" s="77">
-        <v>10</v>
-      </c>
-      <c r="Q46" s="82" t="s">
-        <v>247</v>
-      </c>
-      <c r="R46" s="35">
-        <v>2.2324000000000002</v>
-      </c>
-      <c r="S46" s="35">
-        <v>11.16</v>
-      </c>
-      <c r="T46" s="35">
-        <v>1.9319999999999999</v>
-      </c>
-      <c r="U46" s="35">
-        <v>19.32</v>
-      </c>
-      <c r="V46" s="32"/>
+      <c r="B46" s="22"/>
+      <c r="C46" s="28"/>
+      <c r="D46" s="23"/>
+      <c r="E46" s="53"/>
+      <c r="F46" s="24"/>
+      <c r="G46" s="25"/>
+      <c r="H46" s="24"/>
+      <c r="I46" s="25"/>
+      <c r="J46" s="24"/>
+      <c r="K46" s="25"/>
+      <c r="L46" s="55"/>
+      <c r="M46" s="25"/>
+      <c r="N46" s="25"/>
+      <c r="O46" s="25"/>
+      <c r="P46" s="25"/>
+      <c r="Q46" s="80" t="s">
+        <v>240</v>
+      </c>
+      <c r="R46" s="81"/>
+      <c r="S46" s="71">
+        <f>SUM(S10:S45)</f>
+        <v>29.31</v>
+      </c>
+      <c r="T46" s="25"/>
+      <c r="U46" s="71">
+        <f>SUM(U10:U45)</f>
+        <v>44.829999999999991</v>
+      </c>
+      <c r="V46" s="78"/>
     </row>
-    <row r="47" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:22" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A47" s="1"/>
-      <c r="B47" s="26">
-        <f t="shared" si="0"/>
-        <v>38</v>
-      </c>
-      <c r="C47" s="33" t="s">
-        <v>12</v>
-      </c>
-      <c r="D47" s="34" t="s">
-        <v>51</v>
-      </c>
-      <c r="E47" s="48" t="s">
-        <v>88</v>
-      </c>
-      <c r="F47" s="33" t="s">
-        <v>116</v>
-      </c>
-      <c r="G47" s="34" t="s">
-        <v>148</v>
-      </c>
-      <c r="H47" s="33" t="s">
-        <v>171</v>
-      </c>
-      <c r="I47" s="34"/>
-      <c r="J47" s="33" t="s">
-        <v>263</v>
-      </c>
-      <c r="K47" s="34" t="s">
-        <v>249</v>
-      </c>
-      <c r="L47" s="33">
-        <v>1</v>
-      </c>
-      <c r="M47" s="51">
-        <f t="shared" ref="M47" si="16">L47*5</f>
-        <v>5</v>
-      </c>
-      <c r="N47" s="34">
-        <v>5</v>
-      </c>
-      <c r="O47" s="33">
-        <v>10</v>
-      </c>
-      <c r="P47" s="76">
-        <v>10</v>
-      </c>
-      <c r="Q47" s="83" t="s">
-        <v>247</v>
-      </c>
-      <c r="R47" s="36">
-        <v>1.2198</v>
-      </c>
-      <c r="S47" s="36">
-        <v>6.1</v>
-      </c>
-      <c r="T47" s="36">
-        <v>1.0928</v>
-      </c>
-      <c r="U47" s="36">
-        <v>10.93</v>
-      </c>
-      <c r="V47" s="51"/>
-    </row>
-    <row r="48" spans="1:22" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A48" s="1"/>
-      <c r="B48" s="26">
-        <f>ROW(B48) - ROW($B$9)</f>
-        <v>39</v>
-      </c>
-      <c r="C48" s="56" t="s">
-        <v>12</v>
-      </c>
-      <c r="D48" s="31" t="s">
-        <v>52</v>
-      </c>
-      <c r="E48" s="55" t="s">
-        <v>89</v>
-      </c>
-      <c r="F48" s="56" t="s">
-        <v>117</v>
-      </c>
-      <c r="G48" s="31" t="s">
-        <v>149</v>
-      </c>
-      <c r="H48" s="56" t="s">
-        <v>172</v>
-      </c>
-      <c r="I48" s="31"/>
-      <c r="J48" s="56" t="s">
-        <v>199</v>
-      </c>
-      <c r="K48" s="31" t="s">
-        <v>249</v>
-      </c>
-      <c r="L48" s="64">
-        <v>1</v>
-      </c>
-      <c r="M48" s="53">
-        <f>L48*5</f>
-        <v>5</v>
-      </c>
-      <c r="N48" s="31">
-        <v>5</v>
-      </c>
-      <c r="O48" s="56">
-        <v>10</v>
-      </c>
-      <c r="P48" s="81">
-        <v>10</v>
-      </c>
-      <c r="Q48" s="82" t="s">
-        <v>247</v>
-      </c>
-      <c r="R48" s="35">
-        <v>6.83E-2</v>
-      </c>
-      <c r="S48" s="98">
-        <v>0.34</v>
-      </c>
-      <c r="T48" s="35">
-        <v>6.83E-2</v>
-      </c>
-      <c r="U48" s="98">
-        <v>0.68</v>
-      </c>
-      <c r="V48" s="32"/>
-    </row>
-    <row r="49" spans="1:22" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A49" s="1"/>
-      <c r="B49" s="22"/>
-      <c r="C49" s="28"/>
-      <c r="D49" s="23"/>
-      <c r="E49" s="61"/>
-      <c r="F49" s="24"/>
-      <c r="G49" s="25"/>
-      <c r="H49" s="24"/>
-      <c r="I49" s="25"/>
-      <c r="J49" s="24"/>
-      <c r="K49" s="25"/>
-      <c r="L49" s="63"/>
-      <c r="M49" s="25"/>
-      <c r="N49" s="25"/>
-      <c r="O49" s="25"/>
-      <c r="P49" s="25"/>
-      <c r="Q49" s="93" t="s">
-        <v>264</v>
-      </c>
-      <c r="R49" s="94"/>
-      <c r="S49" s="97">
-        <f>SUM(S10:S48)</f>
-        <v>40.880000000000003</v>
-      </c>
-      <c r="T49" s="25"/>
-      <c r="U49" s="97">
-        <f>SUM(U10:U48)</f>
-        <v>64.87</v>
-      </c>
-      <c r="V49" s="89"/>
-    </row>
-    <row r="50" spans="1:22" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A50" s="1"/>
-      <c r="B50" s="18"/>
-      <c r="C50" s="29"/>
-      <c r="D50" s="7"/>
-      <c r="E50" s="62"/>
-      <c r="F50" s="8"/>
-      <c r="G50" s="8"/>
-      <c r="H50" s="8"/>
-      <c r="I50" s="8"/>
-      <c r="J50" s="8"/>
-      <c r="K50" s="8"/>
-      <c r="L50" s="8"/>
-      <c r="M50" s="8"/>
-      <c r="N50" s="8"/>
-      <c r="O50" s="8"/>
-      <c r="P50" s="8"/>
-      <c r="Q50" s="95" t="s">
-        <v>265</v>
-      </c>
-      <c r="R50" s="96"/>
-      <c r="S50" s="99">
-        <f>(S49/5)</f>
-        <v>8.1760000000000002</v>
-      </c>
-      <c r="T50" s="8"/>
-      <c r="U50" s="99">
-        <f>(U49/10)</f>
-        <v>6.4870000000000001</v>
-      </c>
-      <c r="V50" s="90"/>
+      <c r="B47" s="18"/>
+      <c r="C47" s="29"/>
+      <c r="D47" s="7"/>
+      <c r="E47" s="54"/>
+      <c r="F47" s="8"/>
+      <c r="G47" s="8"/>
+      <c r="H47" s="8"/>
+      <c r="I47" s="8"/>
+      <c r="J47" s="8"/>
+      <c r="K47" s="8"/>
+      <c r="L47" s="8"/>
+      <c r="M47" s="8"/>
+      <c r="N47" s="8"/>
+      <c r="O47" s="8"/>
+      <c r="P47" s="8"/>
+      <c r="Q47" s="82" t="s">
+        <v>241</v>
+      </c>
+      <c r="R47" s="83"/>
+      <c r="S47" s="72">
+        <f>(S46/5)</f>
+        <v>5.8620000000000001</v>
+      </c>
+      <c r="T47" s="8"/>
+      <c r="U47" s="72">
+        <f>(U46/10)</f>
+        <v>4.4829999999999988</v>
+      </c>
+      <c r="V47" s="79"/>
     </row>
   </sheetData>
   <mergeCells count="5">
     <mergeCell ref="K1:V1"/>
     <mergeCell ref="V3:V8"/>
-    <mergeCell ref="V49:V50"/>
-    <mergeCell ref="Q49:R49"/>
-    <mergeCell ref="Q50:R50"/>
+    <mergeCell ref="V46:V47"/>
+    <mergeCell ref="Q46:R46"/>
+    <mergeCell ref="Q47:R47"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="H10" r:id="rId1" display="https://www.lcsc.com/brand-detail/994.html"/>
@@ -4899,17 +4572,17 @@
     <hyperlink ref="Q19" r:id="rId10"/>
     <hyperlink ref="Q21" r:id="rId11"/>
     <hyperlink ref="Q22" r:id="rId12"/>
-    <hyperlink ref="Q23" r:id="rId13"/>
-    <hyperlink ref="Q18" r:id="rId14"/>
-    <hyperlink ref="Q20" r:id="rId15"/>
+    <hyperlink ref="Q18" r:id="rId13"/>
+    <hyperlink ref="Q20" r:id="rId14"/>
+    <hyperlink ref="Q23" r:id="rId15"/>
     <hyperlink ref="Q24" r:id="rId16"/>
     <hyperlink ref="Q25" r:id="rId17"/>
     <hyperlink ref="Q26" r:id="rId18"/>
     <hyperlink ref="Q27" r:id="rId19"/>
-    <hyperlink ref="Q28" r:id="rId20"/>
-    <hyperlink ref="Q30" r:id="rId21"/>
-    <hyperlink ref="Q29" r:id="rId22"/>
-    <hyperlink ref="Q44" r:id="rId23"/>
+    <hyperlink ref="Q29" r:id="rId20"/>
+    <hyperlink ref="Q28" r:id="rId21"/>
+    <hyperlink ref="Q41" r:id="rId22"/>
+    <hyperlink ref="Q30" r:id="rId23"/>
     <hyperlink ref="Q31" r:id="rId24"/>
     <hyperlink ref="Q32" r:id="rId25"/>
     <hyperlink ref="Q33" r:id="rId26"/>
@@ -4918,14 +4591,11 @@
     <hyperlink ref="Q36" r:id="rId29"/>
     <hyperlink ref="Q37" r:id="rId30"/>
     <hyperlink ref="Q38" r:id="rId31"/>
-    <hyperlink ref="Q39" r:id="rId32"/>
-    <hyperlink ref="Q40" r:id="rId33"/>
-    <hyperlink ref="Q48" r:id="rId34"/>
-    <hyperlink ref="Q47" r:id="rId35"/>
-    <hyperlink ref="Q46" r:id="rId36"/>
+    <hyperlink ref="Q45" r:id="rId32"/>
+    <hyperlink ref="Q44" r:id="rId33"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId37"/>
-  <drawing r:id="rId38"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId34"/>
+  <drawing r:id="rId35"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
#34 BOM updated with price changes
</commit_message>
<xml_diff>
--- a/Deliverables/BOM/PAC5527/eSpark_BOM.xlsx
+++ b/Deliverables/BOM/PAC5527/eSpark_BOM.xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="373" uniqueCount="251">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="383" uniqueCount="257">
   <si>
     <t>Component list</t>
   </si>
@@ -535,21 +535,12 @@
     <t>C74338</t>
   </si>
   <si>
-    <t>C919577</t>
-  </si>
-  <si>
-    <t>C185446</t>
-  </si>
-  <si>
     <t>C2828647</t>
   </si>
   <si>
     <t>C620909</t>
   </si>
   <si>
-    <t>C136943</t>
-  </si>
-  <si>
     <t>C313926</t>
   </si>
   <si>
@@ -782,6 +773,33 @@
   </si>
   <si>
     <t>Monolithic Power Systems</t>
+  </si>
+  <si>
+    <t>R24</t>
+  </si>
+  <si>
+    <t>RES 0 OHM JUMPER 1/10W 0603</t>
+  </si>
+  <si>
+    <t>RC0603JR-070RL</t>
+  </si>
+  <si>
+    <t>0R</t>
+  </si>
+  <si>
+    <t>C95177</t>
+  </si>
+  <si>
+    <t>BSC0702LS</t>
+  </si>
+  <si>
+    <t>C501503</t>
+  </si>
+  <si>
+    <t>C137904</t>
+  </si>
+  <si>
+    <t>C105574</t>
   </si>
 </sst>
 </file>
@@ -1328,7 +1346,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="88">
+  <cellXfs count="91">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1523,6 +1541,16 @@
     <xf numFmtId="166" fontId="17" fillId="3" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="20" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="20" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1558,14 +1586,13 @@
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="19" fillId="4" borderId="17" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="16" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="20" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="4" borderId="17" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1910,7 +1937,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:V47"/>
+  <dimension ref="A1:V48"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="3.140625" style="19" customWidth="1"/>
@@ -1944,18 +1971,18 @@
       <c r="H1" s="2"/>
       <c r="I1" s="2"/>
       <c r="J1" s="2"/>
-      <c r="K1" s="73"/>
-      <c r="L1" s="73"/>
-      <c r="M1" s="73"/>
-      <c r="N1" s="73"/>
-      <c r="O1" s="73"/>
-      <c r="P1" s="73"/>
-      <c r="Q1" s="73"/>
-      <c r="R1" s="73"/>
-      <c r="S1" s="73"/>
-      <c r="T1" s="73"/>
-      <c r="U1" s="73"/>
-      <c r="V1" s="74"/>
+      <c r="K1" s="77"/>
+      <c r="L1" s="77"/>
+      <c r="M1" s="77"/>
+      <c r="N1" s="77"/>
+      <c r="O1" s="77"/>
+      <c r="P1" s="77"/>
+      <c r="Q1" s="77"/>
+      <c r="R1" s="77"/>
+      <c r="S1" s="77"/>
+      <c r="T1" s="77"/>
+      <c r="U1" s="77"/>
+      <c r="V1" s="78"/>
     </row>
     <row r="2" spans="1:22" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
@@ -2011,7 +2038,7 @@
       <c r="S3" s="44"/>
       <c r="T3" s="44"/>
       <c r="U3" s="44"/>
-      <c r="V3" s="75"/>
+      <c r="V3" s="79"/>
     </row>
     <row r="4" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
@@ -2039,7 +2066,7 @@
       <c r="S4" s="6"/>
       <c r="T4" s="6"/>
       <c r="U4" s="65"/>
-      <c r="V4" s="76"/>
+      <c r="V4" s="80"/>
     </row>
     <row r="5" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
@@ -2067,7 +2094,7 @@
       <c r="S5" s="5"/>
       <c r="T5" s="5"/>
       <c r="U5" s="5"/>
-      <c r="V5" s="76"/>
+      <c r="V5" s="80"/>
     </row>
     <row r="6" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
@@ -2091,7 +2118,7 @@
       <c r="S6" s="5"/>
       <c r="T6" s="5"/>
       <c r="U6" s="5"/>
-      <c r="V6" s="76"/>
+      <c r="V6" s="80"/>
     </row>
     <row r="7" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
@@ -2115,7 +2142,7 @@
       <c r="S7" s="45"/>
       <c r="T7" s="45"/>
       <c r="U7" s="45"/>
-      <c r="V7" s="76"/>
+      <c r="V7" s="80"/>
     </row>
     <row r="8" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
@@ -2139,7 +2166,7 @@
       <c r="S8" s="64"/>
       <c r="T8" s="64"/>
       <c r="U8" s="64"/>
-      <c r="V8" s="77"/>
+      <c r="V8" s="81"/>
     </row>
     <row r="9" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
@@ -2165,46 +2192,46 @@
         <v>132</v>
       </c>
       <c r="I9" s="20" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="J9" s="21" t="s">
         <v>153</v>
       </c>
       <c r="K9" s="20" t="s">
+        <v>204</v>
+      </c>
+      <c r="L9" s="20" t="s">
+        <v>195</v>
+      </c>
+      <c r="M9" s="20" t="s">
+        <v>206</v>
+      </c>
+      <c r="N9" s="41" t="s">
+        <v>208</v>
+      </c>
+      <c r="O9" s="20" t="s">
+        <v>205</v>
+      </c>
+      <c r="P9" s="20" t="s">
         <v>207</v>
       </c>
-      <c r="L9" s="20" t="s">
-        <v>198</v>
-      </c>
-      <c r="M9" s="20" t="s">
+      <c r="Q9" s="42" t="s">
         <v>209</v>
       </c>
-      <c r="N9" s="41" t="s">
+      <c r="R9" s="20" t="s">
+        <v>213</v>
+      </c>
+      <c r="S9" s="20" t="s">
+        <v>214</v>
+      </c>
+      <c r="T9" s="20" t="s">
+        <v>210</v>
+      </c>
+      <c r="U9" s="20" t="s">
         <v>211</v>
       </c>
-      <c r="O9" s="20" t="s">
-        <v>208</v>
-      </c>
-      <c r="P9" s="20" t="s">
-        <v>210</v>
-      </c>
-      <c r="Q9" s="42" t="s">
+      <c r="V9" s="41" t="s">
         <v>212</v>
-      </c>
-      <c r="R9" s="20" t="s">
-        <v>216</v>
-      </c>
-      <c r="S9" s="20" t="s">
-        <v>217</v>
-      </c>
-      <c r="T9" s="20" t="s">
-        <v>213</v>
-      </c>
-      <c r="U9" s="20" t="s">
-        <v>214</v>
-      </c>
-      <c r="V9" s="41" t="s">
-        <v>215</v>
       </c>
     </row>
     <row r="10" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -2214,29 +2241,29 @@
         <v>1</v>
       </c>
       <c r="C10" s="30" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="D10" s="31" t="s">
         <v>14</v>
       </c>
       <c r="E10" s="48" t="s">
+        <v>215</v>
+      </c>
+      <c r="F10" s="37" t="s">
+        <v>216</v>
+      </c>
+      <c r="G10" s="31" t="s">
+        <v>217</v>
+      </c>
+      <c r="H10" s="30" t="s">
         <v>218</v>
-      </c>
-      <c r="F10" s="37" t="s">
-        <v>219</v>
-      </c>
-      <c r="G10" s="31" t="s">
-        <v>220</v>
-      </c>
-      <c r="H10" s="30" t="s">
-        <v>221</v>
       </c>
       <c r="I10" s="31"/>
       <c r="J10" s="30" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="K10" s="31" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="L10" s="37">
         <v>2</v>
@@ -2255,7 +2282,7 @@
         <v>20</v>
       </c>
       <c r="Q10" s="68" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="R10" s="35">
         <v>0.29630000000000001</v>
@@ -2274,14 +2301,14 @@
     <row r="11" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="1"/>
       <c r="B11" s="26">
-        <f t="shared" ref="B11:B44" si="0">ROW(B11) - ROW($B$9)</f>
+        <f t="shared" ref="B11:B45" si="0">ROW(B11) - ROW($B$9)</f>
         <v>2</v>
       </c>
       <c r="C11" s="33" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="D11" s="34" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="E11" s="43" t="s">
         <v>46</v>
@@ -2300,7 +2327,7 @@
         <v>154</v>
       </c>
       <c r="K11" s="34" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="L11" s="33">
         <v>1</v>
@@ -2319,19 +2346,19 @@
         <v>100</v>
       </c>
       <c r="Q11" s="69" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="R11" s="36">
-        <v>5.1000000000000004E-3</v>
+        <v>5.1999999999999998E-3</v>
       </c>
       <c r="S11" s="36">
-        <v>0.51</v>
+        <v>0.52</v>
       </c>
       <c r="T11" s="36">
-        <v>5.1000000000000004E-3</v>
+        <v>5.1999999999999998E-3</v>
       </c>
       <c r="U11" s="36">
-        <v>0.51</v>
+        <v>0.52</v>
       </c>
       <c r="V11" s="46"/>
     </row>
@@ -2342,7 +2369,7 @@
         <v>3</v>
       </c>
       <c r="C12" s="30" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="D12" s="31" t="s">
         <v>15</v>
@@ -2364,7 +2391,7 @@
         <v>155</v>
       </c>
       <c r="K12" s="31" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="L12" s="47">
         <v>2</v>
@@ -2383,19 +2410,19 @@
         <v>50</v>
       </c>
       <c r="Q12" s="68" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="R12" s="35">
-        <v>1.78E-2</v>
+        <v>1.84E-2</v>
       </c>
       <c r="S12" s="35">
-        <v>0.89</v>
+        <v>0.92</v>
       </c>
       <c r="T12" s="35">
-        <v>1.78E-2</v>
+        <v>1.84E-2</v>
       </c>
       <c r="U12" s="35">
-        <v>0.89</v>
+        <v>0.92</v>
       </c>
       <c r="V12" s="32"/>
     </row>
@@ -2406,7 +2433,7 @@
         <v>4</v>
       </c>
       <c r="C13" s="33" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="D13" s="34" t="s">
         <v>16</v>
@@ -2428,7 +2455,7 @@
         <v>156</v>
       </c>
       <c r="K13" s="34" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="L13" s="33">
         <v>1</v>
@@ -2438,28 +2465,28 @@
         <v>5</v>
       </c>
       <c r="N13" s="34">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="O13" s="33">
         <v>10</v>
       </c>
       <c r="P13" s="66">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="Q13" s="69" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="R13" s="36">
-        <v>1.7100000000000001E-2</v>
+        <v>2.3599999999999999E-2</v>
       </c>
       <c r="S13" s="36">
-        <v>0.86</v>
+        <v>0.47</v>
       </c>
       <c r="T13" s="36">
-        <v>1.7100000000000001E-2</v>
+        <v>2.3599999999999999E-2</v>
       </c>
       <c r="U13" s="36">
-        <v>0.86</v>
+        <v>0.47</v>
       </c>
       <c r="V13" s="46"/>
     </row>
@@ -2470,7 +2497,7 @@
         <v>5</v>
       </c>
       <c r="C14" s="30" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="D14" s="31" t="s">
         <v>17</v>
@@ -2492,7 +2519,7 @@
         <v>157</v>
       </c>
       <c r="K14" s="31" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="L14" s="47">
         <v>1</v>
@@ -2511,19 +2538,19 @@
         <v>20</v>
       </c>
       <c r="Q14" s="68" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="R14" s="35">
-        <v>1.3299999999999999E-2</v>
+        <v>2.3900000000000001E-2</v>
       </c>
       <c r="S14" s="35">
-        <v>0.27</v>
+        <v>0.48</v>
       </c>
       <c r="T14" s="35">
-        <v>1.3299999999999999E-2</v>
+        <v>2.3900000000000001E-2</v>
       </c>
       <c r="U14" s="35">
-        <v>0.27</v>
+        <v>0.48</v>
       </c>
       <c r="V14" s="32"/>
     </row>
@@ -2534,7 +2561,7 @@
         <v>6</v>
       </c>
       <c r="C15" s="33" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="D15" s="34" t="s">
         <v>18</v>
@@ -2556,7 +2583,7 @@
         <v>158</v>
       </c>
       <c r="K15" s="34" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="L15" s="33">
         <v>2</v>
@@ -2575,19 +2602,19 @@
         <v>50</v>
       </c>
       <c r="Q15" s="69" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="R15" s="36">
-        <v>7.1999999999999998E-3</v>
+        <v>7.7000000000000002E-3</v>
       </c>
       <c r="S15" s="36">
-        <v>0.36</v>
+        <v>0.39</v>
       </c>
       <c r="T15" s="36">
-        <v>7.1999999999999998E-3</v>
+        <v>7.7000000000000002E-3</v>
       </c>
       <c r="U15" s="36">
-        <v>0.36</v>
+        <v>0.39</v>
       </c>
       <c r="V15" s="46"/>
     </row>
@@ -2598,7 +2625,7 @@
         <v>7</v>
       </c>
       <c r="C16" s="30" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="D16" s="31" t="s">
         <v>19</v>
@@ -2620,7 +2647,7 @@
         <v>159</v>
       </c>
       <c r="K16" s="31" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="L16" s="47">
         <v>1</v>
@@ -2639,19 +2666,19 @@
         <v>100</v>
       </c>
       <c r="Q16" s="68" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="R16" s="35">
-        <v>2.5999999999999999E-3</v>
+        <v>2.7000000000000001E-3</v>
       </c>
       <c r="S16" s="35">
-        <v>0.26</v>
+        <v>0.27</v>
       </c>
       <c r="T16" s="35">
-        <v>2.5999999999999999E-3</v>
+        <v>2.7000000000000001E-3</v>
       </c>
       <c r="U16" s="35">
-        <v>0.26</v>
+        <v>0.27</v>
       </c>
       <c r="V16" s="32"/>
     </row>
@@ -2662,10 +2689,10 @@
         <v>8</v>
       </c>
       <c r="C17" s="33" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="D17" s="33" t="s">
-        <v>243</v>
+        <v>240</v>
       </c>
       <c r="E17" s="43" t="s">
         <v>51</v>
@@ -2684,7 +2711,7 @@
         <v>160</v>
       </c>
       <c r="K17" s="34" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="L17" s="33">
         <v>2</v>
@@ -2703,19 +2730,19 @@
         <v>20</v>
       </c>
       <c r="Q17" s="69" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="R17" s="36">
-        <v>2.7199999999999998E-2</v>
+        <v>2.8000000000000001E-2</v>
       </c>
       <c r="S17" s="36">
-        <v>0.54</v>
+        <v>0.56000000000000005</v>
       </c>
       <c r="T17" s="36">
-        <v>2.7199999999999998E-2</v>
+        <v>2.8000000000000001E-2</v>
       </c>
       <c r="U17" s="36">
-        <v>0.54</v>
+        <v>0.56000000000000005</v>
       </c>
       <c r="V17" s="46"/>
     </row>
@@ -2726,7 +2753,7 @@
         <v>9</v>
       </c>
       <c r="C18" s="30" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="D18" s="31" t="s">
         <v>20</v>
@@ -2744,13 +2771,13 @@
         <v>136</v>
       </c>
       <c r="I18" s="30" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="J18" s="30" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="K18" s="31" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="L18" s="47">
         <v>3</v>
@@ -2769,19 +2796,19 @@
         <v>30</v>
       </c>
       <c r="Q18" s="68" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="R18" s="35">
-        <v>6.0299999999999999E-2</v>
+        <v>6.2399999999999997E-2</v>
       </c>
       <c r="S18" s="35">
-        <v>1.21</v>
+        <v>1.25</v>
       </c>
       <c r="T18" s="35">
-        <v>6.0299999999999999E-2</v>
+        <v>6.2399999999999997E-2</v>
       </c>
       <c r="U18" s="35">
-        <v>1.81</v>
+        <v>1.87</v>
       </c>
       <c r="V18" s="32"/>
     </row>
@@ -2792,7 +2819,7 @@
         <v>10</v>
       </c>
       <c r="C19" s="33" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="D19" s="34" t="s">
         <v>21</v>
@@ -2814,7 +2841,7 @@
         <v>161</v>
       </c>
       <c r="K19" s="34" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="L19" s="33">
         <v>3</v>
@@ -2833,19 +2860,19 @@
         <v>50</v>
       </c>
       <c r="Q19" s="69" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="R19" s="36">
-        <v>7.0000000000000001E-3</v>
+        <v>7.1000000000000004E-3</v>
       </c>
       <c r="S19" s="36">
-        <v>0.35</v>
+        <v>0.36</v>
       </c>
       <c r="T19" s="36">
-        <v>7.0000000000000001E-3</v>
+        <v>7.1000000000000004E-3</v>
       </c>
       <c r="U19" s="36">
-        <v>0.35</v>
+        <v>0.36</v>
       </c>
       <c r="V19" s="46"/>
     </row>
@@ -2856,7 +2883,7 @@
         <v>11</v>
       </c>
       <c r="C20" s="30" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="D20" s="31" t="s">
         <v>22</v>
@@ -2874,13 +2901,13 @@
         <v>138</v>
       </c>
       <c r="I20" s="30" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="J20" s="30" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="K20" s="31" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
       <c r="L20" s="47">
         <v>3</v>
@@ -2899,19 +2926,19 @@
         <v>100</v>
       </c>
       <c r="Q20" s="68" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="R20" s="35">
-        <v>4.1999999999999997E-3</v>
+        <v>4.4000000000000003E-3</v>
       </c>
       <c r="S20" s="35">
-        <v>0.42</v>
+        <v>0.44</v>
       </c>
       <c r="T20" s="35">
-        <v>4.1999999999999997E-3</v>
+        <v>4.4000000000000003E-3</v>
       </c>
       <c r="U20" s="35">
-        <v>0.42</v>
+        <v>0.44</v>
       </c>
       <c r="V20" s="32"/>
     </row>
@@ -2922,7 +2949,7 @@
         <v>12</v>
       </c>
       <c r="C21" s="33" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="D21" s="34" t="s">
         <v>23</v>
@@ -2944,7 +2971,7 @@
         <v>162</v>
       </c>
       <c r="K21" s="34" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="L21" s="33">
         <v>1</v>
@@ -2963,19 +2990,19 @@
         <v>100</v>
       </c>
       <c r="Q21" s="69" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="R21" s="36">
-        <v>8.9999999999999998E-4</v>
+        <v>1.1000000000000001E-3</v>
       </c>
       <c r="S21" s="36">
-        <v>0.09</v>
+        <v>0.11</v>
       </c>
       <c r="T21" s="36">
-        <v>8.9999999999999998E-4</v>
+        <v>1.1000000000000001E-3</v>
       </c>
       <c r="U21" s="36">
-        <v>0.09</v>
+        <v>0.11</v>
       </c>
       <c r="V21" s="46"/>
     </row>
@@ -2986,10 +3013,10 @@
         <v>13</v>
       </c>
       <c r="C22" s="30" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="D22" s="31" t="s">
-        <v>244</v>
+        <v>241</v>
       </c>
       <c r="E22" s="48" t="s">
         <v>56</v>
@@ -3008,7 +3035,7 @@
         <v>163</v>
       </c>
       <c r="K22" s="31" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="L22" s="47">
         <v>3</v>
@@ -3027,19 +3054,19 @@
         <v>40</v>
       </c>
       <c r="Q22" s="68" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="R22" s="35">
-        <v>2.2800000000000001E-2</v>
+        <v>2.0400000000000001E-2</v>
       </c>
       <c r="S22" s="35">
-        <v>0.46</v>
+        <v>0.41</v>
       </c>
       <c r="T22" s="35">
-        <v>2.2800000000000001E-2</v>
+        <v>2.0400000000000001E-2</v>
       </c>
       <c r="U22" s="35">
-        <v>0.91</v>
+        <v>0.82</v>
       </c>
       <c r="V22" s="32"/>
     </row>
@@ -3050,7 +3077,7 @@
         <v>14</v>
       </c>
       <c r="C23" s="33" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="D23" s="34" t="s">
         <v>29</v>
@@ -3061,20 +3088,20 @@
       <c r="F23" s="33" t="s">
         <v>90</v>
       </c>
-      <c r="G23" s="84">
+      <c r="G23" s="73">
         <v>61300611121</v>
       </c>
       <c r="H23" s="33" t="s">
         <v>138</v>
       </c>
       <c r="I23" s="34" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="J23" s="33" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="K23" s="34" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="L23" s="33">
         <v>1</v>
@@ -3093,16 +3120,16 @@
         <v>20</v>
       </c>
       <c r="Q23" s="69" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="R23" s="36">
-        <v>2.75E-2</v>
+        <v>2.76E-2</v>
       </c>
       <c r="S23" s="36">
         <v>0.55000000000000004</v>
       </c>
       <c r="T23" s="36">
-        <v>2.75E-2</v>
+        <v>2.76E-2</v>
       </c>
       <c r="U23" s="36">
         <v>0.55000000000000004</v>
@@ -3116,7 +3143,7 @@
         <v>15</v>
       </c>
       <c r="C24" s="30" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="D24" s="31" t="s">
         <v>31</v>
@@ -3127,20 +3154,20 @@
       <c r="F24" s="30" t="s">
         <v>92</v>
       </c>
-      <c r="G24" s="85">
+      <c r="G24" s="74">
         <v>61300211121</v>
       </c>
       <c r="H24" s="30" t="s">
         <v>138</v>
       </c>
       <c r="I24" s="31" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="J24" s="30" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="K24" s="31" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="L24" s="47">
         <v>1</v>
@@ -3159,19 +3186,19 @@
         <v>50</v>
       </c>
       <c r="Q24" s="68" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="R24" s="35">
-        <v>1.38E-2</v>
+        <v>1.3299999999999999E-2</v>
       </c>
       <c r="S24" s="35">
-        <v>0.69</v>
+        <v>0.67</v>
       </c>
       <c r="T24" s="35">
-        <v>1.38E-2</v>
+        <v>1.3299999999999999E-2</v>
       </c>
       <c r="U24" s="35">
-        <v>0.69</v>
+        <v>0.67</v>
       </c>
       <c r="V24" s="32"/>
     </row>
@@ -3182,7 +3209,7 @@
         <v>16</v>
       </c>
       <c r="C25" s="33" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="D25" s="34" t="s">
         <v>24</v>
@@ -3204,7 +3231,7 @@
         <v>164</v>
       </c>
       <c r="K25" s="34" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="L25" s="33">
         <v>1</v>
@@ -3223,19 +3250,19 @@
         <v>10</v>
       </c>
       <c r="Q25" s="69" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="R25" s="36">
-        <v>4.9399999999999999E-2</v>
+        <v>5.1200000000000002E-2</v>
       </c>
       <c r="S25" s="36">
-        <v>0.49</v>
+        <v>0.51</v>
       </c>
       <c r="T25" s="36">
-        <v>4.9399999999999999E-2</v>
+        <v>5.1200000000000002E-2</v>
       </c>
       <c r="U25" s="36">
-        <v>0.49</v>
+        <v>0.51</v>
       </c>
       <c r="V25" s="46"/>
     </row>
@@ -3246,7 +3273,7 @@
         <v>17</v>
       </c>
       <c r="C26" s="30" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="D26" s="31" t="s">
         <v>25</v>
@@ -3268,7 +3295,7 @@
         <v>165</v>
       </c>
       <c r="K26" s="31" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="L26" s="47">
         <v>1</v>
@@ -3287,16 +3314,16 @@
         <v>10</v>
       </c>
       <c r="Q26" s="68" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="R26" s="35">
-        <v>4.0599999999999997E-2</v>
+        <v>4.1000000000000002E-2</v>
       </c>
       <c r="S26" s="35">
         <v>0.41</v>
       </c>
       <c r="T26" s="35">
-        <v>4.0599999999999997E-2</v>
+        <v>4.1000000000000002E-2</v>
       </c>
       <c r="U26" s="35">
         <v>0.41</v>
@@ -3332,7 +3359,7 @@
         <v>166</v>
       </c>
       <c r="K27" s="34" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
       <c r="L27" s="33">
         <v>1</v>
@@ -3351,19 +3378,19 @@
         <v>10</v>
       </c>
       <c r="Q27" s="69" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="R27" s="36">
-        <v>0.26819999999999999</v>
+        <v>0.26979999999999998</v>
       </c>
       <c r="S27" s="36">
-        <v>1.34</v>
+        <v>1.35</v>
       </c>
       <c r="T27" s="36">
-        <v>0.26819999999999999</v>
+        <v>0.26979999999999998</v>
       </c>
       <c r="U27" s="36">
-        <v>2.68</v>
+        <v>2.7</v>
       </c>
       <c r="V27" s="46"/>
     </row>
@@ -3374,7 +3401,7 @@
         <v>19</v>
       </c>
       <c r="C28" s="30" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="D28" s="31" t="s">
         <v>27</v>
@@ -3396,7 +3423,7 @@
         <v>167</v>
       </c>
       <c r="K28" s="31" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="L28" s="47">
         <v>2</v>
@@ -3415,19 +3442,19 @@
         <v>20</v>
       </c>
       <c r="Q28" s="68" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="R28" s="35">
-        <v>7.3200000000000001E-2</v>
+        <v>6.3899999999999998E-2</v>
       </c>
       <c r="S28" s="35">
-        <v>0.73</v>
+        <v>0.64</v>
       </c>
       <c r="T28" s="35">
-        <v>7.3200000000000001E-2</v>
+        <v>6.3899999999999998E-2</v>
       </c>
       <c r="U28" s="35">
-        <v>1.46</v>
+        <v>1.28</v>
       </c>
       <c r="V28" s="32"/>
     </row>
@@ -3449,18 +3476,20 @@
       <c r="F29" s="33" t="s">
         <v>93</v>
       </c>
-      <c r="G29" s="34" t="s">
+      <c r="G29" s="76" t="s">
         <v>118</v>
       </c>
       <c r="H29" s="33" t="s">
         <v>142</v>
       </c>
-      <c r="I29" s="34"/>
+      <c r="I29" s="33" t="s">
+        <v>253</v>
+      </c>
       <c r="J29" s="33" t="s">
-        <v>168</v>
+        <v>254</v>
       </c>
       <c r="K29" s="34" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="L29" s="33">
         <v>6</v>
@@ -3479,19 +3508,19 @@
         <v>60</v>
       </c>
       <c r="Q29" s="69" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="R29" s="36">
-        <v>0.1668</v>
+        <v>0.57279999999999998</v>
       </c>
       <c r="S29" s="36">
-        <v>5</v>
+        <v>17.18</v>
       </c>
       <c r="T29" s="36">
-        <v>0.13439999999999999</v>
+        <v>0.57279999999999998</v>
       </c>
       <c r="U29" s="36">
-        <v>8.06</v>
+        <v>34.369999999999997</v>
       </c>
       <c r="V29" s="46"/>
     </row>
@@ -3513,7 +3542,7 @@
       <c r="F30" s="30" t="s">
         <v>95</v>
       </c>
-      <c r="G30" s="31" t="s">
+      <c r="G30" s="74" t="s">
         <v>119</v>
       </c>
       <c r="H30" s="30" t="s">
@@ -3521,10 +3550,10 @@
       </c>
       <c r="I30" s="31"/>
       <c r="J30" s="30" t="s">
-        <v>169</v>
+        <v>255</v>
       </c>
       <c r="K30" s="31" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="L30" s="47">
         <v>3</v>
@@ -3543,19 +3572,19 @@
         <v>100</v>
       </c>
       <c r="Q30" s="68" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="R30" s="35">
-        <v>1.5E-3</v>
+        <v>1E-3</v>
       </c>
       <c r="S30" s="35">
-        <v>0.15</v>
+        <v>0.1</v>
       </c>
       <c r="T30" s="35">
-        <v>1.5E-3</v>
+        <v>1E-3</v>
       </c>
       <c r="U30" s="35">
-        <v>0.15</v>
+        <v>0.1</v>
       </c>
       <c r="V30" s="32"/>
     </row>
@@ -3577,20 +3606,20 @@
       <c r="F31" s="33" t="s">
         <v>96</v>
       </c>
-      <c r="G31" s="87" t="s">
+      <c r="G31" s="76" t="s">
         <v>120</v>
       </c>
       <c r="H31" s="33" t="s">
         <v>143</v>
       </c>
       <c r="I31" s="34" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
       <c r="J31" s="33" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="K31" s="34" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="L31" s="33">
         <v>6</v>
@@ -3609,19 +3638,19 @@
         <v>60</v>
       </c>
       <c r="Q31" s="69" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="R31" s="36">
-        <v>3.1600000000000003E-2</v>
+        <v>3.0599999999999999E-2</v>
       </c>
       <c r="S31" s="36">
-        <v>1.26</v>
+        <v>1.22</v>
       </c>
       <c r="T31" s="36">
-        <v>3.1600000000000003E-2</v>
+        <v>3.0599999999999999E-2</v>
       </c>
       <c r="U31" s="36">
-        <v>1.9</v>
+        <v>1.84</v>
       </c>
       <c r="V31" s="46"/>
     </row>
@@ -3635,7 +3664,7 @@
         <v>11</v>
       </c>
       <c r="D32" s="31" t="s">
-        <v>245</v>
+        <v>242</v>
       </c>
       <c r="E32" s="48" t="s">
         <v>67</v>
@@ -3643,20 +3672,20 @@
       <c r="F32" s="30" t="s">
         <v>96</v>
       </c>
-      <c r="G32" s="85" t="s">
+      <c r="G32" s="74" t="s">
         <v>121</v>
       </c>
       <c r="H32" s="30" t="s">
         <v>144</v>
       </c>
       <c r="I32" s="31" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
       <c r="J32" s="30" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="K32" s="31" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="L32" s="47">
         <v>4</v>
@@ -3675,19 +3704,19 @@
         <v>100</v>
       </c>
       <c r="Q32" s="68" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="R32" s="35">
-        <v>1.6999999999999999E-3</v>
+        <v>1.6000000000000001E-3</v>
       </c>
       <c r="S32" s="35">
-        <v>0.17</v>
+        <v>0.16</v>
       </c>
       <c r="T32" s="35">
-        <v>1.6999999999999999E-3</v>
+        <v>1.6000000000000001E-3</v>
       </c>
       <c r="U32" s="35">
-        <v>0.17</v>
+        <v>0.16</v>
       </c>
       <c r="V32" s="32"/>
     </row>
@@ -3717,10 +3746,10 @@
       </c>
       <c r="I33" s="34"/>
       <c r="J33" s="33" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="K33" s="34" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
       <c r="L33" s="33">
         <v>3</v>
@@ -3739,19 +3768,19 @@
         <v>40</v>
       </c>
       <c r="Q33" s="69" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="R33" s="36">
-        <v>2.7900000000000001E-2</v>
+        <v>3.2199999999999999E-2</v>
       </c>
       <c r="S33" s="36">
-        <v>0.56000000000000005</v>
+        <v>0.64</v>
       </c>
       <c r="T33" s="36">
-        <v>2.7900000000000001E-2</v>
+        <v>3.2199999999999999E-2</v>
       </c>
       <c r="U33" s="36">
-        <v>1.1200000000000001</v>
+        <v>1.29</v>
       </c>
       <c r="V33" s="46"/>
     </row>
@@ -3781,10 +3810,10 @@
       </c>
       <c r="I34" s="31"/>
       <c r="J34" s="30" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="K34" s="31" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="L34" s="47">
         <v>3</v>
@@ -3803,19 +3832,19 @@
         <v>50</v>
       </c>
       <c r="Q34" s="68" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="R34" s="35">
-        <v>7.1999999999999998E-3</v>
+        <v>8.0999999999999996E-3</v>
       </c>
       <c r="S34" s="35">
-        <v>0.36</v>
+        <v>0.41</v>
       </c>
       <c r="T34" s="35">
-        <v>7.1999999999999998E-3</v>
+        <v>8.0999999999999996E-3</v>
       </c>
       <c r="U34" s="35">
-        <v>0.36</v>
+        <v>0.41</v>
       </c>
       <c r="V34" s="32"/>
     </row>
@@ -3837,7 +3866,7 @@
       <c r="F35" s="33" t="s">
         <v>94</v>
       </c>
-      <c r="G35" s="34" t="s">
+      <c r="G35" s="76" t="s">
         <v>124</v>
       </c>
       <c r="H35" s="33" t="s">
@@ -3845,10 +3874,10 @@
       </c>
       <c r="I35" s="34"/>
       <c r="J35" s="33" t="s">
-        <v>172</v>
+        <v>256</v>
       </c>
       <c r="K35" s="34" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="L35" s="33">
         <v>1</v>
@@ -3858,28 +3887,28 @@
         <v>5</v>
       </c>
       <c r="N35" s="34">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="O35" s="33">
         <v>10</v>
       </c>
       <c r="P35" s="66">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="Q35" s="69" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="R35" s="36">
-        <v>1.1599999999999999E-2</v>
+        <v>1.1999999999999999E-3</v>
       </c>
       <c r="S35" s="36">
-        <v>0.57999999999999996</v>
+        <v>0.12</v>
       </c>
       <c r="T35" s="36">
-        <v>1.1599999999999999E-2</v>
+        <v>1.1999999999999999E-3</v>
       </c>
       <c r="U35" s="36">
-        <v>0.57999999999999996</v>
+        <v>0.12</v>
       </c>
       <c r="V35" s="46"/>
     </row>
@@ -3901,20 +3930,20 @@
       <c r="F36" s="30" t="s">
         <v>97</v>
       </c>
-      <c r="G36" s="85" t="s">
+      <c r="G36" s="74" t="s">
         <v>125</v>
       </c>
       <c r="H36" s="30" t="s">
         <v>147</v>
       </c>
       <c r="I36" s="31" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="J36" s="30" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="K36" s="31" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="L36" s="47">
         <v>1</v>
@@ -3933,7 +3962,7 @@
         <v>100</v>
       </c>
       <c r="Q36" s="68" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="R36" s="35">
         <v>5.9999999999999995E-4</v>
@@ -3975,10 +4004,10 @@
       </c>
       <c r="I37" s="34"/>
       <c r="J37" s="33" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="K37" s="34" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="L37" s="33">
         <v>1</v>
@@ -3997,19 +4026,19 @@
         <v>10</v>
       </c>
       <c r="Q37" s="69" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="R37" s="36">
-        <v>6.4399999999999999E-2</v>
+        <v>4.53E-2</v>
       </c>
       <c r="S37" s="36">
-        <v>0.64</v>
+        <v>0.45</v>
       </c>
       <c r="T37" s="36">
-        <v>6.4399999999999999E-2</v>
+        <v>4.53E-2</v>
       </c>
       <c r="U37" s="36">
-        <v>0.64</v>
+        <v>0.45</v>
       </c>
       <c r="V37" s="46"/>
     </row>
@@ -4023,7 +4052,7 @@
         <v>11</v>
       </c>
       <c r="D38" s="31" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="E38" s="48" t="s">
         <v>73</v>
@@ -4039,10 +4068,10 @@
       </c>
       <c r="I38" s="31"/>
       <c r="J38" s="30" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="K38" s="31" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="L38" s="47">
         <v>1</v>
@@ -4061,7 +4090,7 @@
         <v>100</v>
       </c>
       <c r="Q38" s="68" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="R38" s="35">
         <v>1.1999999999999999E-3</v>
@@ -4079,129 +4108,126 @@
     </row>
     <row r="39" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A39" s="1"/>
-      <c r="B39" s="26">
-        <f>ROW(B39) - ROW($B$9)</f>
-        <v>30</v>
-      </c>
+      <c r="B39" s="26"/>
       <c r="C39" s="33" t="s">
-        <v>203</v>
-      </c>
-      <c r="D39" s="34" t="s">
-        <v>28</v>
-      </c>
-      <c r="E39" s="43" t="s">
-        <v>224</v>
+        <v>11</v>
+      </c>
+      <c r="D39" s="33" t="s">
+        <v>248</v>
+      </c>
+      <c r="E39" s="34" t="s">
+        <v>249</v>
       </c>
       <c r="F39" s="33" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="G39" s="34" t="s">
-        <v>225</v>
+        <v>250</v>
       </c>
       <c r="H39" s="33" t="s">
-        <v>225</v>
-      </c>
-      <c r="I39" s="34"/>
+        <v>133</v>
+      </c>
+      <c r="I39" s="33"/>
       <c r="J39" s="33" t="s">
-        <v>225</v>
-      </c>
-      <c r="K39" s="34" t="s">
-        <v>187</v>
-      </c>
-      <c r="L39" s="33" t="s">
-        <v>225</v>
-      </c>
-      <c r="M39" s="46" t="s">
-        <v>225</v>
-      </c>
-      <c r="N39" s="34" t="s">
-        <v>225</v>
-      </c>
-      <c r="O39" s="33" t="s">
-        <v>225</v>
-      </c>
-      <c r="P39" s="66" t="s">
-        <v>225</v>
-      </c>
-      <c r="Q39" s="69" t="s">
-        <v>225</v>
-      </c>
-      <c r="R39" s="36" t="s">
-        <v>225</v>
-      </c>
-      <c r="S39" s="36" t="s">
-        <v>225</v>
-      </c>
-      <c r="T39" s="36" t="s">
-        <v>225</v>
-      </c>
-      <c r="U39" s="36" t="s">
-        <v>225</v>
-      </c>
-      <c r="V39" s="46"/>
-    </row>
-    <row r="40" spans="1:22" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>252</v>
+      </c>
+      <c r="K39" s="33" t="s">
+        <v>251</v>
+      </c>
+      <c r="L39" s="34">
+        <v>1</v>
+      </c>
+      <c r="M39" s="33">
+        <v>5</v>
+      </c>
+      <c r="N39" s="33">
+        <v>100</v>
+      </c>
+      <c r="O39" s="33">
+        <v>10</v>
+      </c>
+      <c r="P39" s="66">
+        <v>100</v>
+      </c>
+      <c r="Q39" s="88" t="s">
+        <v>220</v>
+      </c>
+      <c r="R39" s="36">
+        <v>1.1000000000000001E-3</v>
+      </c>
+      <c r="S39" s="36">
+        <v>0.11</v>
+      </c>
+      <c r="T39" s="36">
+        <v>1.1000000000000001E-3</v>
+      </c>
+      <c r="U39" s="36">
+        <v>0.11</v>
+      </c>
+      <c r="V39" s="33"/>
+    </row>
+    <row r="40" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A40" s="1"/>
       <c r="B40" s="26">
         <f>ROW(B40) - ROW($B$9)</f>
         <v>31</v>
       </c>
       <c r="C40" s="30" t="s">
-        <v>204</v>
-      </c>
-      <c r="D40" s="31" t="s">
-        <v>30</v>
-      </c>
-      <c r="E40" s="48" t="s">
-        <v>62</v>
+        <v>200</v>
+      </c>
+      <c r="D40" s="30" t="s">
+        <v>28</v>
+      </c>
+      <c r="E40" s="30" t="s">
+        <v>221</v>
       </c>
       <c r="F40" s="30" t="s">
-        <v>91</v>
-      </c>
-      <c r="G40" s="31" t="s">
-        <v>225</v>
+        <v>89</v>
+      </c>
+      <c r="G40" s="30" t="s">
+        <v>222</v>
       </c>
       <c r="H40" s="30" t="s">
-        <v>225</v>
-      </c>
-      <c r="I40" s="31"/>
+        <v>222</v>
+      </c>
+      <c r="I40" s="30"/>
       <c r="J40" s="30" t="s">
-        <v>225</v>
-      </c>
-      <c r="K40" s="31" t="s">
-        <v>188</v>
-      </c>
-      <c r="L40" s="47" t="s">
-        <v>225</v>
-      </c>
-      <c r="M40" s="32" t="s">
-        <v>225</v>
-      </c>
-      <c r="N40" s="31" t="s">
-        <v>225</v>
+        <v>222</v>
+      </c>
+      <c r="K40" s="30" t="s">
+        <v>184</v>
+      </c>
+      <c r="L40" s="30" t="s">
+        <v>222</v>
+      </c>
+      <c r="M40" s="30" t="s">
+        <v>222</v>
+      </c>
+      <c r="N40" s="30" t="s">
+        <v>222</v>
       </c>
       <c r="O40" s="30" t="s">
-        <v>225</v>
-      </c>
-      <c r="P40" s="67" t="s">
-        <v>225</v>
-      </c>
-      <c r="Q40" s="68" t="s">
-        <v>225</v>
-      </c>
-      <c r="R40" s="35" t="s">
-        <v>225</v>
-      </c>
-      <c r="S40" s="35" t="s">
-        <v>225</v>
-      </c>
-      <c r="T40" s="35" t="s">
-        <v>225</v>
-      </c>
-      <c r="U40" s="35" t="s">
-        <v>225</v>
-      </c>
-      <c r="V40" s="32"/>
+        <v>222</v>
+      </c>
+      <c r="P40" s="30" t="s">
+        <v>222</v>
+      </c>
+      <c r="Q40" s="30" t="s">
+        <v>222</v>
+      </c>
+      <c r="R40" s="30" t="s">
+        <v>222</v>
+      </c>
+      <c r="S40" s="30" t="s">
+        <v>222</v>
+      </c>
+      <c r="T40" s="30" t="s">
+        <v>222</v>
+      </c>
+      <c r="U40" s="30" t="s">
+        <v>222</v>
+      </c>
+      <c r="V40" s="30"/>
     </row>
     <row r="41" spans="1:22" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A41" s="1"/>
@@ -4210,111 +4236,128 @@
         <v>32</v>
       </c>
       <c r="C41" s="33" t="s">
-        <v>205</v>
-      </c>
-      <c r="D41" s="34" t="s">
-        <v>40</v>
-      </c>
-      <c r="E41" s="43" t="s">
-        <v>74</v>
+        <v>201</v>
+      </c>
+      <c r="D41" s="33" t="s">
+        <v>30</v>
+      </c>
+      <c r="E41" s="33" t="s">
+        <v>62</v>
       </c>
       <c r="F41" s="33" t="s">
-        <v>99</v>
-      </c>
-      <c r="G41" s="34" t="s">
-        <v>128</v>
+        <v>91</v>
+      </c>
+      <c r="G41" s="33" t="s">
+        <v>222</v>
       </c>
       <c r="H41" s="33" t="s">
-        <v>149</v>
-      </c>
-      <c r="I41" s="34"/>
+        <v>222</v>
+      </c>
+      <c r="I41" s="33"/>
       <c r="J41" s="33" t="s">
-        <v>175</v>
-      </c>
-      <c r="K41" s="34" t="s">
-        <v>225</v>
-      </c>
-      <c r="L41" s="33">
-        <v>1</v>
-      </c>
-      <c r="M41" s="46">
-        <f>L41*5</f>
-        <v>5</v>
-      </c>
-      <c r="N41" s="34">
-        <v>10</v>
-      </c>
-      <c r="O41" s="33">
-        <v>10</v>
-      </c>
-      <c r="P41" s="66">
-        <v>10</v>
-      </c>
-      <c r="Q41" s="69" t="s">
-        <v>223</v>
-      </c>
-      <c r="R41" s="36">
-        <v>5.8200000000000002E-2</v>
-      </c>
-      <c r="S41" s="36">
-        <v>0.57999999999999996</v>
-      </c>
-      <c r="T41" s="36">
-        <v>5.8200000000000002E-2</v>
-      </c>
-      <c r="U41" s="36">
-        <v>0.57999999999999996</v>
-      </c>
-      <c r="V41" s="46"/>
+        <v>222</v>
+      </c>
+      <c r="K41" s="33" t="s">
+        <v>185</v>
+      </c>
+      <c r="L41" s="33" t="s">
+        <v>222</v>
+      </c>
+      <c r="M41" s="33" t="s">
+        <v>222</v>
+      </c>
+      <c r="N41" s="33" t="s">
+        <v>222</v>
+      </c>
+      <c r="O41" s="33" t="s">
+        <v>222</v>
+      </c>
+      <c r="P41" s="33" t="s">
+        <v>222</v>
+      </c>
+      <c r="Q41" s="33" t="s">
+        <v>222</v>
+      </c>
+      <c r="R41" s="33" t="s">
+        <v>222</v>
+      </c>
+      <c r="S41" s="33" t="s">
+        <v>222</v>
+      </c>
+      <c r="T41" s="33" t="s">
+        <v>222</v>
+      </c>
+      <c r="U41" s="33" t="s">
+        <v>222</v>
+      </c>
+      <c r="V41" s="33"/>
     </row>
     <row r="42" spans="1:22" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A42" s="1"/>
       <c r="B42" s="26">
-        <f t="shared" si="0"/>
+        <f>ROW(B42) - ROW($B$9)</f>
         <v>33</v>
       </c>
       <c r="C42" s="30" t="s">
-        <v>12</v>
-      </c>
-      <c r="D42" s="31" t="s">
-        <v>41</v>
-      </c>
-      <c r="E42" s="48" t="s">
-        <v>75</v>
+        <v>202</v>
+      </c>
+      <c r="D42" s="30" t="s">
+        <v>40</v>
+      </c>
+      <c r="E42" s="30" t="s">
+        <v>74</v>
       </c>
       <c r="F42" s="30" t="s">
-        <v>100</v>
-      </c>
-      <c r="G42" s="31" t="s">
-        <v>129</v>
+        <v>99</v>
+      </c>
+      <c r="G42" s="30" t="s">
+        <v>128</v>
       </c>
       <c r="H42" s="30" t="s">
-        <v>150</v>
-      </c>
-      <c r="I42" s="31"/>
-      <c r="J42" s="30"/>
-      <c r="K42" s="31" t="s">
-        <v>225</v>
-      </c>
-      <c r="L42" s="47">
+        <v>149</v>
+      </c>
+      <c r="I42" s="30"/>
+      <c r="J42" s="30" t="s">
+        <v>172</v>
+      </c>
+      <c r="K42" s="30" t="s">
+        <v>222</v>
+      </c>
+      <c r="L42" s="30">
         <v>1</v>
       </c>
-      <c r="M42" s="32">
-        <f t="shared" ref="M42:M43" si="14">L42*5</f>
+      <c r="M42" s="30">
+        <f>L42*5</f>
         <v>5</v>
       </c>
-      <c r="N42" s="31"/>
-      <c r="O42" s="30"/>
-      <c r="P42" s="67"/>
-      <c r="Q42" s="68"/>
-      <c r="R42" s="35"/>
-      <c r="S42" s="35"/>
-      <c r="T42" s="35"/>
-      <c r="U42" s="35"/>
-      <c r="V42" s="32"/>
-    </row>
-    <row r="43" spans="1:22" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A43" s="86"/>
+      <c r="N42" s="30">
+        <v>10</v>
+      </c>
+      <c r="O42" s="30">
+        <v>10</v>
+      </c>
+      <c r="P42" s="30">
+        <v>10</v>
+      </c>
+      <c r="Q42" s="68" t="s">
+        <v>220</v>
+      </c>
+      <c r="R42" s="35">
+        <v>5.7599999999999998E-2</v>
+      </c>
+      <c r="S42" s="35">
+        <v>0.57999999999999996</v>
+      </c>
+      <c r="T42" s="35">
+        <v>5.7599999999999998E-2</v>
+      </c>
+      <c r="U42" s="35">
+        <v>0.57999999999999996</v>
+      </c>
+      <c r="V42" s="30"/>
+    </row>
+    <row r="43" spans="1:22" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A43" s="1"/>
       <c r="B43" s="26">
         <f t="shared" si="0"/>
         <v>34</v>
@@ -4322,45 +4365,45 @@
       <c r="C43" s="33" t="s">
         <v>12</v>
       </c>
-      <c r="D43" s="34" t="s">
-        <v>42</v>
-      </c>
-      <c r="E43" s="43" t="s">
-        <v>247</v>
+      <c r="D43" s="33" t="s">
+        <v>41</v>
+      </c>
+      <c r="E43" s="33" t="s">
+        <v>75</v>
       </c>
       <c r="F43" s="33" t="s">
-        <v>248</v>
-      </c>
-      <c r="G43" s="34" t="s">
-        <v>249</v>
+        <v>100</v>
+      </c>
+      <c r="G43" s="33" t="s">
+        <v>129</v>
       </c>
       <c r="H43" s="33" t="s">
-        <v>250</v>
-      </c>
-      <c r="I43" s="34"/>
+        <v>150</v>
+      </c>
+      <c r="I43" s="33"/>
       <c r="J43" s="33"/>
-      <c r="K43" s="34" t="s">
-        <v>225</v>
+      <c r="K43" s="33" t="s">
+        <v>222</v>
       </c>
       <c r="L43" s="33">
         <v>1</v>
       </c>
-      <c r="M43" s="46">
-        <f t="shared" si="14"/>
+      <c r="M43" s="33">
+        <f t="shared" ref="M43:M44" si="14">L43*5</f>
         <v>5</v>
       </c>
-      <c r="N43" s="34"/>
+      <c r="N43" s="33"/>
       <c r="O43" s="33"/>
-      <c r="P43" s="66"/>
-      <c r="Q43" s="69"/>
-      <c r="R43" s="36"/>
-      <c r="S43" s="36"/>
-      <c r="T43" s="36"/>
-      <c r="U43" s="36"/>
-      <c r="V43" s="46"/>
-    </row>
-    <row r="44" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A44" s="1"/>
+      <c r="P43" s="33"/>
+      <c r="Q43" s="33"/>
+      <c r="R43" s="33"/>
+      <c r="S43" s="33"/>
+      <c r="T43" s="33"/>
+      <c r="U43" s="33"/>
+      <c r="V43" s="33"/>
+    </row>
+    <row r="44" spans="1:22" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A44" s="75"/>
       <c r="B44" s="26">
         <f t="shared" si="0"/>
         <v>35</v>
@@ -4368,196 +4411,242 @@
       <c r="C44" s="30" t="s">
         <v>12</v>
       </c>
-      <c r="D44" s="31" t="s">
-        <v>43</v>
-      </c>
-      <c r="E44" s="48" t="s">
-        <v>76</v>
+      <c r="D44" s="30" t="s">
+        <v>42</v>
+      </c>
+      <c r="E44" s="30" t="s">
+        <v>244</v>
       </c>
       <c r="F44" s="30" t="s">
-        <v>101</v>
-      </c>
-      <c r="G44" s="31" t="s">
-        <v>130</v>
+        <v>245</v>
+      </c>
+      <c r="G44" s="30" t="s">
+        <v>246</v>
       </c>
       <c r="H44" s="30" t="s">
-        <v>151</v>
-      </c>
-      <c r="I44" s="31"/>
-      <c r="J44" s="30" t="s">
-        <v>239</v>
-      </c>
-      <c r="K44" s="31" t="s">
-        <v>225</v>
-      </c>
-      <c r="L44" s="47">
+        <v>247</v>
+      </c>
+      <c r="I44" s="30"/>
+      <c r="J44" s="30"/>
+      <c r="K44" s="30" t="s">
+        <v>222</v>
+      </c>
+      <c r="L44" s="30">
         <v>1</v>
       </c>
-      <c r="M44" s="32">
-        <f t="shared" ref="M44" si="15">L44*5</f>
+      <c r="M44" s="30">
+        <f t="shared" si="14"/>
         <v>5</v>
       </c>
-      <c r="N44" s="31">
-        <v>5</v>
-      </c>
-      <c r="O44" s="30">
-        <v>10</v>
-      </c>
-      <c r="P44" s="67">
-        <v>10</v>
-      </c>
-      <c r="Q44" s="68" t="s">
-        <v>223</v>
-      </c>
-      <c r="R44" s="35">
-        <v>1.2198</v>
-      </c>
-      <c r="S44" s="35">
-        <v>6.1</v>
-      </c>
-      <c r="T44" s="35">
-        <v>1.0928</v>
-      </c>
-      <c r="U44" s="35">
-        <v>10.93</v>
-      </c>
-      <c r="V44" s="32"/>
-    </row>
-    <row r="45" spans="1:22" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="N44" s="30"/>
+      <c r="O44" s="30"/>
+      <c r="P44" s="30"/>
+      <c r="Q44" s="30"/>
+      <c r="R44" s="30"/>
+      <c r="S44" s="30"/>
+      <c r="T44" s="30"/>
+      <c r="U44" s="30"/>
+      <c r="V44" s="30"/>
+    </row>
+    <row r="45" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A45" s="1"/>
       <c r="B45" s="26">
-        <f>ROW(B45) - ROW($B$9)</f>
+        <f t="shared" si="0"/>
         <v>36</v>
       </c>
       <c r="C45" s="33" t="s">
         <v>12</v>
       </c>
-      <c r="D45" s="34" t="s">
-        <v>44</v>
-      </c>
-      <c r="E45" s="43" t="s">
-        <v>77</v>
+      <c r="D45" s="33" t="s">
+        <v>43</v>
+      </c>
+      <c r="E45" s="33" t="s">
+        <v>76</v>
       </c>
       <c r="F45" s="33" t="s">
-        <v>102</v>
-      </c>
-      <c r="G45" s="34" t="s">
-        <v>131</v>
+        <v>101</v>
+      </c>
+      <c r="G45" s="33" t="s">
+        <v>130</v>
       </c>
       <c r="H45" s="33" t="s">
-        <v>152</v>
-      </c>
-      <c r="I45" s="34"/>
+        <v>151</v>
+      </c>
+      <c r="I45" s="33"/>
       <c r="J45" s="33" t="s">
-        <v>176</v>
-      </c>
-      <c r="K45" s="34" t="s">
-        <v>225</v>
+        <v>236</v>
+      </c>
+      <c r="K45" s="33" t="s">
+        <v>222</v>
       </c>
       <c r="L45" s="33">
         <v>1</v>
       </c>
-      <c r="M45" s="46">
-        <f>L45*5</f>
+      <c r="M45" s="33">
+        <f t="shared" ref="M45" si="15">L45*5</f>
         <v>5</v>
       </c>
-      <c r="N45" s="34">
+      <c r="N45" s="33">
         <v>5</v>
       </c>
       <c r="O45" s="33">
         <v>10</v>
       </c>
-      <c r="P45" s="66">
+      <c r="P45" s="33">
         <v>10</v>
       </c>
-      <c r="Q45" s="69" t="s">
-        <v>223</v>
+      <c r="Q45" s="90" t="s">
+        <v>220</v>
       </c>
       <c r="R45" s="36">
-        <v>6.83E-2</v>
+        <v>1.2919</v>
       </c>
       <c r="S45" s="36">
-        <v>0.34</v>
+        <v>6.46</v>
       </c>
       <c r="T45" s="36">
-        <v>6.83E-2</v>
+        <v>1.2919</v>
       </c>
       <c r="U45" s="36">
-        <v>0.68</v>
-      </c>
-      <c r="V45" s="46"/>
-    </row>
-    <row r="46" spans="1:22" ht="15.75" x14ac:dyDescent="0.25">
+        <v>11.54</v>
+      </c>
+      <c r="V45" s="33"/>
+    </row>
+    <row r="46" spans="1:22" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A46" s="1"/>
-      <c r="B46" s="22"/>
-      <c r="C46" s="28"/>
-      <c r="D46" s="23"/>
-      <c r="E46" s="53"/>
-      <c r="F46" s="24"/>
-      <c r="G46" s="25"/>
-      <c r="H46" s="24"/>
-      <c r="I46" s="25"/>
-      <c r="J46" s="24"/>
-      <c r="K46" s="25"/>
-      <c r="L46" s="55"/>
-      <c r="M46" s="25"/>
-      <c r="N46" s="25"/>
-      <c r="O46" s="25"/>
-      <c r="P46" s="25"/>
-      <c r="Q46" s="80" t="s">
-        <v>240</v>
-      </c>
-      <c r="R46" s="81"/>
-      <c r="S46" s="71">
-        <f>SUM(S10:S45)</f>
-        <v>29.31</v>
-      </c>
-      <c r="T46" s="25"/>
-      <c r="U46" s="71">
-        <f>SUM(U10:U45)</f>
-        <v>44.829999999999991</v>
-      </c>
-      <c r="V46" s="78"/>
-    </row>
-    <row r="47" spans="1:22" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B46" s="26">
+        <f>ROW(B46) - ROW($B$9)</f>
+        <v>37</v>
+      </c>
+      <c r="C46" s="30" t="s">
+        <v>12</v>
+      </c>
+      <c r="D46" s="30" t="s">
+        <v>44</v>
+      </c>
+      <c r="E46" s="30" t="s">
+        <v>77</v>
+      </c>
+      <c r="F46" s="30" t="s">
+        <v>102</v>
+      </c>
+      <c r="G46" s="30" t="s">
+        <v>131</v>
+      </c>
+      <c r="H46" s="30" t="s">
+        <v>152</v>
+      </c>
+      <c r="I46" s="30"/>
+      <c r="J46" s="30" t="s">
+        <v>173</v>
+      </c>
+      <c r="K46" s="30" t="s">
+        <v>222</v>
+      </c>
+      <c r="L46" s="30">
+        <v>1</v>
+      </c>
+      <c r="M46" s="30">
+        <f>L46*5</f>
+        <v>5</v>
+      </c>
+      <c r="N46" s="30">
+        <v>5</v>
+      </c>
+      <c r="O46" s="30">
+        <v>10</v>
+      </c>
+      <c r="P46" s="30">
+        <v>10</v>
+      </c>
+      <c r="Q46" s="89" t="s">
+        <v>220</v>
+      </c>
+      <c r="R46" s="35">
+        <v>7.6300000000000007E-2</v>
+      </c>
+      <c r="S46" s="35">
+        <v>0.38</v>
+      </c>
+      <c r="T46" s="35">
+        <v>7.6300000000000007E-2</v>
+      </c>
+      <c r="U46" s="35">
+        <v>0.38</v>
+      </c>
+      <c r="V46" s="30"/>
+    </row>
+    <row r="47" spans="1:22" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A47" s="1"/>
-      <c r="B47" s="18"/>
-      <c r="C47" s="29"/>
-      <c r="D47" s="7"/>
-      <c r="E47" s="54"/>
-      <c r="F47" s="8"/>
-      <c r="G47" s="8"/>
-      <c r="H47" s="8"/>
-      <c r="I47" s="8"/>
-      <c r="J47" s="8"/>
-      <c r="K47" s="8"/>
-      <c r="L47" s="8"/>
-      <c r="M47" s="8"/>
-      <c r="N47" s="8"/>
-      <c r="O47" s="8"/>
-      <c r="P47" s="8"/>
-      <c r="Q47" s="82" t="s">
-        <v>241</v>
-      </c>
-      <c r="R47" s="83"/>
-      <c r="S47" s="72">
-        <f>(S46/5)</f>
-        <v>5.8620000000000001</v>
-      </c>
-      <c r="T47" s="8"/>
-      <c r="U47" s="72">
-        <f>(U46/10)</f>
-        <v>4.4829999999999988</v>
-      </c>
-      <c r="V47" s="79"/>
+      <c r="B47" s="22"/>
+      <c r="C47" s="28"/>
+      <c r="D47" s="23"/>
+      <c r="E47" s="53"/>
+      <c r="F47" s="24"/>
+      <c r="G47" s="25"/>
+      <c r="H47" s="24"/>
+      <c r="I47" s="25"/>
+      <c r="J47" s="24"/>
+      <c r="K47" s="25"/>
+      <c r="L47" s="55"/>
+      <c r="M47" s="25"/>
+      <c r="N47" s="25"/>
+      <c r="O47" s="25"/>
+      <c r="P47" s="25"/>
+      <c r="Q47" s="84" t="s">
+        <v>237</v>
+      </c>
+      <c r="R47" s="85"/>
+      <c r="S47" s="71">
+        <f>SUM(S10:S46)</f>
+        <v>41.26</v>
+      </c>
+      <c r="T47" s="25"/>
+      <c r="U47" s="71">
+        <f>SUM(U10:U46)</f>
+        <v>70.789999999999992</v>
+      </c>
+      <c r="V47" s="82"/>
+    </row>
+    <row r="48" spans="1:22" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A48" s="1"/>
+      <c r="B48" s="18"/>
+      <c r="C48" s="29"/>
+      <c r="D48" s="7"/>
+      <c r="E48" s="54"/>
+      <c r="F48" s="8"/>
+      <c r="G48" s="8"/>
+      <c r="H48" s="8"/>
+      <c r="I48" s="8"/>
+      <c r="J48" s="8"/>
+      <c r="K48" s="8"/>
+      <c r="L48" s="8"/>
+      <c r="M48" s="8"/>
+      <c r="N48" s="8"/>
+      <c r="O48" s="8"/>
+      <c r="P48" s="8"/>
+      <c r="Q48" s="86" t="s">
+        <v>238</v>
+      </c>
+      <c r="R48" s="87"/>
+      <c r="S48" s="72">
+        <f>(S47/5)</f>
+        <v>8.2519999999999989</v>
+      </c>
+      <c r="T48" s="8"/>
+      <c r="U48" s="72">
+        <f>(U47/10)</f>
+        <v>7.0789999999999988</v>
+      </c>
+      <c r="V48" s="83"/>
     </row>
   </sheetData>
   <mergeCells count="5">
     <mergeCell ref="K1:V1"/>
     <mergeCell ref="V3:V8"/>
-    <mergeCell ref="V46:V47"/>
-    <mergeCell ref="Q46:R46"/>
+    <mergeCell ref="V47:V48"/>
     <mergeCell ref="Q47:R47"/>
+    <mergeCell ref="Q48:R48"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="H10" r:id="rId1" display="https://www.lcsc.com/brand-detail/994.html"/>
@@ -4581,21 +4670,22 @@
     <hyperlink ref="Q27" r:id="rId19"/>
     <hyperlink ref="Q29" r:id="rId20"/>
     <hyperlink ref="Q28" r:id="rId21"/>
-    <hyperlink ref="Q41" r:id="rId22"/>
-    <hyperlink ref="Q30" r:id="rId23"/>
-    <hyperlink ref="Q31" r:id="rId24"/>
-    <hyperlink ref="Q32" r:id="rId25"/>
-    <hyperlink ref="Q33" r:id="rId26"/>
-    <hyperlink ref="Q34" r:id="rId27"/>
-    <hyperlink ref="Q35" r:id="rId28"/>
-    <hyperlink ref="Q36" r:id="rId29"/>
-    <hyperlink ref="Q37" r:id="rId30"/>
-    <hyperlink ref="Q38" r:id="rId31"/>
+    <hyperlink ref="Q30" r:id="rId22"/>
+    <hyperlink ref="Q31" r:id="rId23"/>
+    <hyperlink ref="Q32" r:id="rId24"/>
+    <hyperlink ref="Q33" r:id="rId25"/>
+    <hyperlink ref="Q34" r:id="rId26"/>
+    <hyperlink ref="Q35" r:id="rId27"/>
+    <hyperlink ref="Q36" r:id="rId28"/>
+    <hyperlink ref="Q37" r:id="rId29"/>
+    <hyperlink ref="Q38" r:id="rId30"/>
+    <hyperlink ref="Q46" r:id="rId31"/>
     <hyperlink ref="Q45" r:id="rId32"/>
-    <hyperlink ref="Q44" r:id="rId33"/>
+    <hyperlink ref="Q39" r:id="rId33"/>
+    <hyperlink ref="Q42" r:id="rId34"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId34"/>
-  <drawing r:id="rId35"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId35"/>
+  <drawing r:id="rId36"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
#34 BOM updated with updated headers and ICs
</commit_message>
<xml_diff>
--- a/Deliverables/BOM/PAC5527/eSpark_BOM.xlsx
+++ b/Deliverables/BOM/PAC5527/eSpark_BOM.xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="383" uniqueCount="257">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="387" uniqueCount="259">
   <si>
     <t>Component list</t>
   </si>
@@ -376,12 +376,6 @@
     <t>1N4148WS-7-F</t>
   </si>
   <si>
-    <t>B4B-XH-A(LF)(SN)</t>
-  </si>
-  <si>
-    <t>B3B-XH-A(LF)(SN)</t>
-  </si>
-  <si>
     <t>16-213/GHC-YR1S1/3T</t>
   </si>
   <si>
@@ -451,9 +445,6 @@
     <t>Diodes</t>
   </si>
   <si>
-    <t>JST</t>
-  </si>
-  <si>
     <t>Everlight Elec</t>
   </si>
   <si>
@@ -523,12 +514,6 @@
     <t>C60580</t>
   </si>
   <si>
-    <t>C144395</t>
-  </si>
-  <si>
-    <t>C144394</t>
-  </si>
-  <si>
     <t>C13754</t>
   </si>
   <si>
@@ -800,6 +785,27 @@
   </si>
   <si>
     <t>C105574</t>
+  </si>
+  <si>
+    <t>B-2100S04P-A110</t>
+  </si>
+  <si>
+    <t>B-2100S03P-A110</t>
+  </si>
+  <si>
+    <t>Ckmtw</t>
+  </si>
+  <si>
+    <t>C124378</t>
+  </si>
+  <si>
+    <t>C124376</t>
+  </si>
+  <si>
+    <t>Chipsmall</t>
+  </si>
+  <si>
+    <t>Buy from Chipsmall</t>
   </si>
 </sst>
 </file>
@@ -811,7 +817,7 @@
     <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.0000"/>
     <numFmt numFmtId="166" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="24" x14ac:knownFonts="1">
+  <fonts count="25" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -977,6 +983,14 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="7">
     <fill>
@@ -1346,7 +1360,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="91">
+  <cellXfs count="93">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1551,6 +1565,15 @@
     <xf numFmtId="0" fontId="20" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="165" fontId="19" fillId="4" borderId="17" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="16" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="4" borderId="17" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1586,13 +1609,10 @@
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="165" fontId="19" fillId="4" borderId="17" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="24" fillId="4" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="16" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="4" borderId="17" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="24" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1971,18 +1991,18 @@
       <c r="H1" s="2"/>
       <c r="I1" s="2"/>
       <c r="J1" s="2"/>
-      <c r="K1" s="77"/>
-      <c r="L1" s="77"/>
-      <c r="M1" s="77"/>
-      <c r="N1" s="77"/>
-      <c r="O1" s="77"/>
-      <c r="P1" s="77"/>
-      <c r="Q1" s="77"/>
-      <c r="R1" s="77"/>
-      <c r="S1" s="77"/>
-      <c r="T1" s="77"/>
-      <c r="U1" s="77"/>
-      <c r="V1" s="78"/>
+      <c r="K1" s="80"/>
+      <c r="L1" s="80"/>
+      <c r="M1" s="80"/>
+      <c r="N1" s="80"/>
+      <c r="O1" s="80"/>
+      <c r="P1" s="80"/>
+      <c r="Q1" s="80"/>
+      <c r="R1" s="80"/>
+      <c r="S1" s="80"/>
+      <c r="T1" s="80"/>
+      <c r="U1" s="80"/>
+      <c r="V1" s="81"/>
     </row>
     <row r="2" spans="1:22" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
@@ -2038,7 +2058,7 @@
       <c r="S3" s="44"/>
       <c r="T3" s="44"/>
       <c r="U3" s="44"/>
-      <c r="V3" s="79"/>
+      <c r="V3" s="82"/>
     </row>
     <row r="4" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
@@ -2066,7 +2086,7 @@
       <c r="S4" s="6"/>
       <c r="T4" s="6"/>
       <c r="U4" s="65"/>
-      <c r="V4" s="80"/>
+      <c r="V4" s="83"/>
     </row>
     <row r="5" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
@@ -2094,7 +2114,7 @@
       <c r="S5" s="5"/>
       <c r="T5" s="5"/>
       <c r="U5" s="5"/>
-      <c r="V5" s="80"/>
+      <c r="V5" s="83"/>
     </row>
     <row r="6" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
@@ -2118,7 +2138,7 @@
       <c r="S6" s="5"/>
       <c r="T6" s="5"/>
       <c r="U6" s="5"/>
-      <c r="V6" s="80"/>
+      <c r="V6" s="83"/>
     </row>
     <row r="7" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
@@ -2142,7 +2162,7 @@
       <c r="S7" s="45"/>
       <c r="T7" s="45"/>
       <c r="U7" s="45"/>
-      <c r="V7" s="80"/>
+      <c r="V7" s="83"/>
     </row>
     <row r="8" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
@@ -2166,7 +2186,7 @@
       <c r="S8" s="64"/>
       <c r="T8" s="64"/>
       <c r="U8" s="64"/>
-      <c r="V8" s="81"/>
+      <c r="V8" s="84"/>
     </row>
     <row r="9" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
@@ -2189,49 +2209,49 @@
         <v>103</v>
       </c>
       <c r="H9" s="20" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="I9" s="20" t="s">
+        <v>198</v>
+      </c>
+      <c r="J9" s="21" t="s">
+        <v>150</v>
+      </c>
+      <c r="K9" s="20" t="s">
+        <v>199</v>
+      </c>
+      <c r="L9" s="20" t="s">
+        <v>190</v>
+      </c>
+      <c r="M9" s="20" t="s">
+        <v>201</v>
+      </c>
+      <c r="N9" s="41" t="s">
         <v>203</v>
       </c>
-      <c r="J9" s="21" t="s">
-        <v>153</v>
-      </c>
-      <c r="K9" s="20" t="s">
+      <c r="O9" s="20" t="s">
+        <v>200</v>
+      </c>
+      <c r="P9" s="20" t="s">
+        <v>202</v>
+      </c>
+      <c r="Q9" s="42" t="s">
         <v>204</v>
       </c>
-      <c r="L9" s="20" t="s">
-        <v>195</v>
-      </c>
-      <c r="M9" s="20" t="s">
+      <c r="R9" s="20" t="s">
+        <v>208</v>
+      </c>
+      <c r="S9" s="20" t="s">
+        <v>209</v>
+      </c>
+      <c r="T9" s="20" t="s">
+        <v>205</v>
+      </c>
+      <c r="U9" s="20" t="s">
         <v>206</v>
       </c>
-      <c r="N9" s="41" t="s">
-        <v>208</v>
-      </c>
-      <c r="O9" s="20" t="s">
-        <v>205</v>
-      </c>
-      <c r="P9" s="20" t="s">
+      <c r="V9" s="41" t="s">
         <v>207</v>
-      </c>
-      <c r="Q9" s="42" t="s">
-        <v>209</v>
-      </c>
-      <c r="R9" s="20" t="s">
-        <v>213</v>
-      </c>
-      <c r="S9" s="20" t="s">
-        <v>214</v>
-      </c>
-      <c r="T9" s="20" t="s">
-        <v>210</v>
-      </c>
-      <c r="U9" s="20" t="s">
-        <v>211</v>
-      </c>
-      <c r="V9" s="41" t="s">
-        <v>212</v>
       </c>
     </row>
     <row r="10" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -2241,29 +2261,29 @@
         <v>1</v>
       </c>
       <c r="C10" s="30" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
       <c r="D10" s="31" t="s">
         <v>14</v>
       </c>
       <c r="E10" s="48" t="s">
-        <v>215</v>
+        <v>210</v>
       </c>
       <c r="F10" s="37" t="s">
-        <v>216</v>
+        <v>211</v>
       </c>
       <c r="G10" s="31" t="s">
-        <v>217</v>
+        <v>212</v>
       </c>
       <c r="H10" s="30" t="s">
-        <v>218</v>
+        <v>213</v>
       </c>
       <c r="I10" s="31"/>
       <c r="J10" s="30" t="s">
-        <v>219</v>
+        <v>214</v>
       </c>
       <c r="K10" s="31" t="s">
-        <v>174</v>
+        <v>169</v>
       </c>
       <c r="L10" s="37">
         <v>2</v>
@@ -2282,7 +2302,7 @@
         <v>20</v>
       </c>
       <c r="Q10" s="68" t="s">
-        <v>220</v>
+        <v>215</v>
       </c>
       <c r="R10" s="35">
         <v>0.29630000000000001</v>
@@ -2305,10 +2325,10 @@
         <v>2</v>
       </c>
       <c r="C11" s="33" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
       <c r="D11" s="34" t="s">
-        <v>239</v>
+        <v>234</v>
       </c>
       <c r="E11" s="43" t="s">
         <v>46</v>
@@ -2320,14 +2340,14 @@
         <v>104</v>
       </c>
       <c r="H11" s="33" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="I11" s="34"/>
       <c r="J11" s="33" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="K11" s="34" t="s">
-        <v>175</v>
+        <v>170</v>
       </c>
       <c r="L11" s="33">
         <v>1</v>
@@ -2346,7 +2366,7 @@
         <v>100</v>
       </c>
       <c r="Q11" s="69" t="s">
-        <v>220</v>
+        <v>215</v>
       </c>
       <c r="R11" s="36">
         <v>5.1999999999999998E-3</v>
@@ -2369,7 +2389,7 @@
         <v>3</v>
       </c>
       <c r="C12" s="30" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
       <c r="D12" s="31" t="s">
         <v>15</v>
@@ -2384,14 +2404,14 @@
         <v>105</v>
       </c>
       <c r="H12" s="30" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="I12" s="31"/>
       <c r="J12" s="30" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="K12" s="31" t="s">
-        <v>176</v>
+        <v>171</v>
       </c>
       <c r="L12" s="47">
         <v>2</v>
@@ -2410,7 +2430,7 @@
         <v>50</v>
       </c>
       <c r="Q12" s="68" t="s">
-        <v>220</v>
+        <v>215</v>
       </c>
       <c r="R12" s="35">
         <v>1.84E-2</v>
@@ -2433,7 +2453,7 @@
         <v>4</v>
       </c>
       <c r="C13" s="33" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
       <c r="D13" s="34" t="s">
         <v>16</v>
@@ -2448,14 +2468,14 @@
         <v>106</v>
       </c>
       <c r="H13" s="33" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="I13" s="34"/>
       <c r="J13" s="33" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="K13" s="34" t="s">
-        <v>177</v>
+        <v>172</v>
       </c>
       <c r="L13" s="33">
         <v>1</v>
@@ -2474,7 +2494,7 @@
         <v>20</v>
       </c>
       <c r="Q13" s="69" t="s">
-        <v>220</v>
+        <v>215</v>
       </c>
       <c r="R13" s="36">
         <v>2.3599999999999999E-2</v>
@@ -2497,7 +2517,7 @@
         <v>5</v>
       </c>
       <c r="C14" s="30" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
       <c r="D14" s="31" t="s">
         <v>17</v>
@@ -2512,14 +2532,14 @@
         <v>107</v>
       </c>
       <c r="H14" s="30" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="I14" s="31"/>
       <c r="J14" s="30" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="K14" s="31" t="s">
-        <v>178</v>
+        <v>173</v>
       </c>
       <c r="L14" s="47">
         <v>1</v>
@@ -2538,7 +2558,7 @@
         <v>20</v>
       </c>
       <c r="Q14" s="68" t="s">
-        <v>220</v>
+        <v>215</v>
       </c>
       <c r="R14" s="35">
         <v>2.3900000000000001E-2</v>
@@ -2561,7 +2581,7 @@
         <v>6</v>
       </c>
       <c r="C15" s="33" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
       <c r="D15" s="34" t="s">
         <v>18</v>
@@ -2576,14 +2596,14 @@
         <v>108</v>
       </c>
       <c r="H15" s="33" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="I15" s="34"/>
       <c r="J15" s="33" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="K15" s="34" t="s">
-        <v>176</v>
+        <v>171</v>
       </c>
       <c r="L15" s="33">
         <v>2</v>
@@ -2602,7 +2622,7 @@
         <v>50</v>
       </c>
       <c r="Q15" s="69" t="s">
-        <v>220</v>
+        <v>215</v>
       </c>
       <c r="R15" s="36">
         <v>7.7000000000000002E-3</v>
@@ -2625,7 +2645,7 @@
         <v>7</v>
       </c>
       <c r="C16" s="30" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
       <c r="D16" s="31" t="s">
         <v>19</v>
@@ -2640,14 +2660,14 @@
         <v>109</v>
       </c>
       <c r="H16" s="30" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="I16" s="31"/>
       <c r="J16" s="30" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="K16" s="31" t="s">
-        <v>175</v>
+        <v>170</v>
       </c>
       <c r="L16" s="47">
         <v>1</v>
@@ -2666,7 +2686,7 @@
         <v>100</v>
       </c>
       <c r="Q16" s="68" t="s">
-        <v>220</v>
+        <v>215</v>
       </c>
       <c r="R16" s="35">
         <v>2.7000000000000001E-3</v>
@@ -2689,10 +2709,10 @@
         <v>8</v>
       </c>
       <c r="C17" s="33" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
       <c r="D17" s="33" t="s">
-        <v>240</v>
+        <v>235</v>
       </c>
       <c r="E17" s="43" t="s">
         <v>51</v>
@@ -2704,14 +2724,14 @@
         <v>110</v>
       </c>
       <c r="H17" s="33" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="I17" s="34"/>
       <c r="J17" s="33" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="K17" s="34" t="s">
-        <v>179</v>
+        <v>174</v>
       </c>
       <c r="L17" s="33">
         <v>2</v>
@@ -2730,7 +2750,7 @@
         <v>20</v>
       </c>
       <c r="Q17" s="69" t="s">
-        <v>220</v>
+        <v>215</v>
       </c>
       <c r="R17" s="36">
         <v>2.8000000000000001E-2</v>
@@ -2753,7 +2773,7 @@
         <v>9</v>
       </c>
       <c r="C18" s="30" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
       <c r="D18" s="31" t="s">
         <v>20</v>
@@ -2768,16 +2788,16 @@
         <v>111</v>
       </c>
       <c r="H18" s="30" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="I18" s="30" t="s">
-        <v>223</v>
+        <v>218</v>
       </c>
       <c r="J18" s="30" t="s">
-        <v>224</v>
+        <v>219</v>
       </c>
       <c r="K18" s="31" t="s">
-        <v>177</v>
+        <v>172</v>
       </c>
       <c r="L18" s="47">
         <v>3</v>
@@ -2796,7 +2816,7 @@
         <v>30</v>
       </c>
       <c r="Q18" s="68" t="s">
-        <v>220</v>
+        <v>215</v>
       </c>
       <c r="R18" s="35">
         <v>6.2399999999999997E-2</v>
@@ -2819,7 +2839,7 @@
         <v>10</v>
       </c>
       <c r="C19" s="33" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
       <c r="D19" s="34" t="s">
         <v>21</v>
@@ -2834,14 +2854,14 @@
         <v>112</v>
       </c>
       <c r="H19" s="33" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="I19" s="34"/>
       <c r="J19" s="33" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="K19" s="34" t="s">
-        <v>180</v>
+        <v>175</v>
       </c>
       <c r="L19" s="33">
         <v>3</v>
@@ -2860,7 +2880,7 @@
         <v>50</v>
       </c>
       <c r="Q19" s="69" t="s">
-        <v>220</v>
+        <v>215</v>
       </c>
       <c r="R19" s="36">
         <v>7.1000000000000004E-3</v>
@@ -2883,7 +2903,7 @@
         <v>11</v>
       </c>
       <c r="C20" s="30" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
       <c r="D20" s="31" t="s">
         <v>22</v>
@@ -2898,16 +2918,16 @@
         <v>885012205080</v>
       </c>
       <c r="H20" s="30" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="I20" s="30" t="s">
-        <v>225</v>
+        <v>220</v>
       </c>
       <c r="J20" s="30" t="s">
-        <v>226</v>
+        <v>221</v>
       </c>
       <c r="K20" s="31" t="s">
-        <v>181</v>
+        <v>176</v>
       </c>
       <c r="L20" s="47">
         <v>3</v>
@@ -2926,7 +2946,7 @@
         <v>100</v>
       </c>
       <c r="Q20" s="68" t="s">
-        <v>220</v>
+        <v>215</v>
       </c>
       <c r="R20" s="35">
         <v>4.4000000000000003E-3</v>
@@ -2949,7 +2969,7 @@
         <v>12</v>
       </c>
       <c r="C21" s="33" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
       <c r="D21" s="34" t="s">
         <v>23</v>
@@ -2964,14 +2984,14 @@
         <v>113</v>
       </c>
       <c r="H21" s="33" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="I21" s="34"/>
       <c r="J21" s="33" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="K21" s="34" t="s">
-        <v>175</v>
+        <v>170</v>
       </c>
       <c r="L21" s="33">
         <v>1</v>
@@ -2990,7 +3010,7 @@
         <v>100</v>
       </c>
       <c r="Q21" s="69" t="s">
-        <v>220</v>
+        <v>215</v>
       </c>
       <c r="R21" s="36">
         <v>1.1000000000000001E-3</v>
@@ -3013,10 +3033,10 @@
         <v>13</v>
       </c>
       <c r="C22" s="30" t="s">
-        <v>197</v>
+        <v>192</v>
       </c>
       <c r="D22" s="31" t="s">
-        <v>241</v>
+        <v>236</v>
       </c>
       <c r="E22" s="48" t="s">
         <v>56</v>
@@ -3028,14 +3048,14 @@
         <v>114</v>
       </c>
       <c r="H22" s="30" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="I22" s="31"/>
       <c r="J22" s="30" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="K22" s="31" t="s">
-        <v>222</v>
+        <v>217</v>
       </c>
       <c r="L22" s="47">
         <v>3</v>
@@ -3054,7 +3074,7 @@
         <v>40</v>
       </c>
       <c r="Q22" s="68" t="s">
-        <v>220</v>
+        <v>215</v>
       </c>
       <c r="R22" s="35">
         <v>2.0400000000000001E-2</v>
@@ -3077,7 +3097,7 @@
         <v>14</v>
       </c>
       <c r="C23" s="33" t="s">
-        <v>198</v>
+        <v>193</v>
       </c>
       <c r="D23" s="34" t="s">
         <v>29</v>
@@ -3092,16 +3112,16 @@
         <v>61300611121</v>
       </c>
       <c r="H23" s="33" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="I23" s="34" t="s">
-        <v>227</v>
+        <v>222</v>
       </c>
       <c r="J23" s="33" t="s">
-        <v>227</v>
+        <v>222</v>
       </c>
       <c r="K23" s="34" t="s">
-        <v>222</v>
+        <v>217</v>
       </c>
       <c r="L23" s="33">
         <v>1</v>
@@ -3120,7 +3140,7 @@
         <v>20</v>
       </c>
       <c r="Q23" s="69" t="s">
-        <v>220</v>
+        <v>215</v>
       </c>
       <c r="R23" s="36">
         <v>2.76E-2</v>
@@ -3143,7 +3163,7 @@
         <v>15</v>
       </c>
       <c r="C24" s="30" t="s">
-        <v>198</v>
+        <v>193</v>
       </c>
       <c r="D24" s="31" t="s">
         <v>31</v>
@@ -3158,16 +3178,16 @@
         <v>61300211121</v>
       </c>
       <c r="H24" s="30" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="I24" s="31" t="s">
-        <v>228</v>
+        <v>223</v>
       </c>
       <c r="J24" s="30" t="s">
-        <v>229</v>
+        <v>224</v>
       </c>
       <c r="K24" s="31" t="s">
-        <v>222</v>
+        <v>217</v>
       </c>
       <c r="L24" s="47">
         <v>1</v>
@@ -3186,7 +3206,7 @@
         <v>50</v>
       </c>
       <c r="Q24" s="68" t="s">
-        <v>220</v>
+        <v>215</v>
       </c>
       <c r="R24" s="35">
         <v>1.3299999999999999E-2</v>
@@ -3209,7 +3229,7 @@
         <v>16</v>
       </c>
       <c r="C25" s="33" t="s">
-        <v>198</v>
+        <v>193</v>
       </c>
       <c r="D25" s="34" t="s">
         <v>24</v>
@@ -3221,17 +3241,17 @@
         <v>85</v>
       </c>
       <c r="G25" s="34" t="s">
-        <v>115</v>
+        <v>252</v>
       </c>
       <c r="H25" s="33" t="s">
-        <v>140</v>
+        <v>254</v>
       </c>
       <c r="I25" s="34"/>
       <c r="J25" s="33" t="s">
-        <v>164</v>
+        <v>255</v>
       </c>
       <c r="K25" s="34" t="s">
-        <v>222</v>
+        <v>217</v>
       </c>
       <c r="L25" s="33">
         <v>1</v>
@@ -3250,19 +3270,19 @@
         <v>10</v>
       </c>
       <c r="Q25" s="69" t="s">
-        <v>220</v>
+        <v>215</v>
       </c>
       <c r="R25" s="36">
-        <v>5.1200000000000002E-2</v>
+        <v>4.0500000000000001E-2</v>
       </c>
       <c r="S25" s="36">
-        <v>0.51</v>
+        <v>0.41</v>
       </c>
       <c r="T25" s="36">
-        <v>5.1200000000000002E-2</v>
+        <v>4.0500000000000001E-2</v>
       </c>
       <c r="U25" s="36">
-        <v>0.51</v>
+        <v>0.41</v>
       </c>
       <c r="V25" s="46"/>
     </row>
@@ -3273,7 +3293,7 @@
         <v>17</v>
       </c>
       <c r="C26" s="30" t="s">
-        <v>198</v>
+        <v>193</v>
       </c>
       <c r="D26" s="31" t="s">
         <v>25</v>
@@ -3285,17 +3305,17 @@
         <v>86</v>
       </c>
       <c r="G26" s="31" t="s">
-        <v>116</v>
+        <v>253</v>
       </c>
       <c r="H26" s="30" t="s">
-        <v>140</v>
+        <v>254</v>
       </c>
       <c r="I26" s="31"/>
       <c r="J26" s="30" t="s">
-        <v>165</v>
+        <v>256</v>
       </c>
       <c r="K26" s="31" t="s">
-        <v>222</v>
+        <v>217</v>
       </c>
       <c r="L26" s="47">
         <v>1</v>
@@ -3305,28 +3325,28 @@
         <v>5</v>
       </c>
       <c r="N26" s="31">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="O26" s="30">
         <v>10</v>
       </c>
       <c r="P26" s="67">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="Q26" s="68" t="s">
-        <v>220</v>
+        <v>215</v>
       </c>
       <c r="R26" s="35">
-        <v>4.1000000000000002E-2</v>
+        <v>2.3E-2</v>
       </c>
       <c r="S26" s="35">
-        <v>0.41</v>
+        <v>0.46</v>
       </c>
       <c r="T26" s="35">
-        <v>4.1000000000000002E-2</v>
+        <v>2.3E-2</v>
       </c>
       <c r="U26" s="35">
-        <v>0.41</v>
+        <v>0.46</v>
       </c>
       <c r="V26" s="32"/>
     </row>
@@ -3352,14 +3372,14 @@
         <v>87</v>
       </c>
       <c r="H27" s="33" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="I27" s="34"/>
       <c r="J27" s="33" t="s">
-        <v>166</v>
+        <v>161</v>
       </c>
       <c r="K27" s="34" t="s">
-        <v>182</v>
+        <v>177</v>
       </c>
       <c r="L27" s="33">
         <v>1</v>
@@ -3378,7 +3398,7 @@
         <v>10</v>
       </c>
       <c r="Q27" s="69" t="s">
-        <v>220</v>
+        <v>215</v>
       </c>
       <c r="R27" s="36">
         <v>0.26979999999999998</v>
@@ -3401,7 +3421,7 @@
         <v>19</v>
       </c>
       <c r="C28" s="30" t="s">
-        <v>199</v>
+        <v>194</v>
       </c>
       <c r="D28" s="31" t="s">
         <v>27</v>
@@ -3413,17 +3433,17 @@
         <v>88</v>
       </c>
       <c r="G28" s="31" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="H28" s="30" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="I28" s="31"/>
       <c r="J28" s="30" t="s">
-        <v>167</v>
+        <v>162</v>
       </c>
       <c r="K28" s="31" t="s">
-        <v>183</v>
+        <v>178</v>
       </c>
       <c r="L28" s="47">
         <v>2</v>
@@ -3442,7 +3462,7 @@
         <v>20</v>
       </c>
       <c r="Q28" s="68" t="s">
-        <v>220</v>
+        <v>215</v>
       </c>
       <c r="R28" s="35">
         <v>6.3899999999999998E-2</v>
@@ -3477,19 +3497,19 @@
         <v>93</v>
       </c>
       <c r="G29" s="76" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="H29" s="33" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="I29" s="33" t="s">
-        <v>253</v>
+        <v>248</v>
       </c>
       <c r="J29" s="33" t="s">
-        <v>254</v>
+        <v>249</v>
       </c>
       <c r="K29" s="34" t="s">
-        <v>222</v>
+        <v>217</v>
       </c>
       <c r="L29" s="33">
         <v>6</v>
@@ -3508,7 +3528,7 @@
         <v>60</v>
       </c>
       <c r="Q29" s="69" t="s">
-        <v>220</v>
+        <v>215</v>
       </c>
       <c r="R29" s="36">
         <v>0.57279999999999998</v>
@@ -3543,17 +3563,17 @@
         <v>95</v>
       </c>
       <c r="G30" s="74" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="H30" s="30" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="I30" s="31"/>
       <c r="J30" s="30" t="s">
-        <v>255</v>
+        <v>250</v>
       </c>
       <c r="K30" s="31" t="s">
-        <v>186</v>
+        <v>181</v>
       </c>
       <c r="L30" s="47">
         <v>3</v>
@@ -3572,7 +3592,7 @@
         <v>100</v>
       </c>
       <c r="Q30" s="68" t="s">
-        <v>220</v>
+        <v>215</v>
       </c>
       <c r="R30" s="35">
         <v>1E-3</v>
@@ -3607,19 +3627,19 @@
         <v>96</v>
       </c>
       <c r="G31" s="76" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="H31" s="33" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="I31" s="34" t="s">
-        <v>231</v>
+        <v>226</v>
       </c>
       <c r="J31" s="33" t="s">
-        <v>230</v>
+        <v>225</v>
       </c>
       <c r="K31" s="34" t="s">
-        <v>187</v>
+        <v>182</v>
       </c>
       <c r="L31" s="33">
         <v>6</v>
@@ -3638,7 +3658,7 @@
         <v>60</v>
       </c>
       <c r="Q31" s="69" t="s">
-        <v>220</v>
+        <v>215</v>
       </c>
       <c r="R31" s="36">
         <v>3.0599999999999999E-2</v>
@@ -3664,7 +3684,7 @@
         <v>11</v>
       </c>
       <c r="D32" s="31" t="s">
-        <v>242</v>
+        <v>237</v>
       </c>
       <c r="E32" s="48" t="s">
         <v>67</v>
@@ -3673,19 +3693,19 @@
         <v>96</v>
       </c>
       <c r="G32" s="74" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="H32" s="30" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="I32" s="31" t="s">
-        <v>232</v>
+        <v>227</v>
       </c>
       <c r="J32" s="30" t="s">
-        <v>233</v>
+        <v>228</v>
       </c>
       <c r="K32" s="31" t="s">
-        <v>188</v>
+        <v>183</v>
       </c>
       <c r="L32" s="47">
         <v>4</v>
@@ -3704,7 +3724,7 @@
         <v>100</v>
       </c>
       <c r="Q32" s="68" t="s">
-        <v>220</v>
+        <v>215</v>
       </c>
       <c r="R32" s="35">
         <v>1.6000000000000001E-3</v>
@@ -3739,17 +3759,17 @@
         <v>94</v>
       </c>
       <c r="G33" s="34" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="H33" s="33" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="I33" s="34"/>
       <c r="J33" s="33" t="s">
-        <v>168</v>
+        <v>163</v>
       </c>
       <c r="K33" s="34" t="s">
-        <v>189</v>
+        <v>184</v>
       </c>
       <c r="L33" s="33">
         <v>3</v>
@@ -3768,7 +3788,7 @@
         <v>40</v>
       </c>
       <c r="Q33" s="69" t="s">
-        <v>220</v>
+        <v>215</v>
       </c>
       <c r="R33" s="36">
         <v>3.2199999999999999E-2</v>
@@ -3803,17 +3823,17 @@
         <v>94</v>
       </c>
       <c r="G34" s="31" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="H34" s="30" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="I34" s="31"/>
       <c r="J34" s="30" t="s">
-        <v>169</v>
+        <v>164</v>
       </c>
       <c r="K34" s="31" t="s">
-        <v>190</v>
+        <v>185</v>
       </c>
       <c r="L34" s="47">
         <v>3</v>
@@ -3832,7 +3852,7 @@
         <v>50</v>
       </c>
       <c r="Q34" s="68" t="s">
-        <v>220</v>
+        <v>215</v>
       </c>
       <c r="R34" s="35">
         <v>8.0999999999999996E-3</v>
@@ -3867,17 +3887,17 @@
         <v>94</v>
       </c>
       <c r="G35" s="76" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="H35" s="33" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="I35" s="34"/>
       <c r="J35" s="33" t="s">
-        <v>256</v>
+        <v>251</v>
       </c>
       <c r="K35" s="34" t="s">
-        <v>191</v>
+        <v>186</v>
       </c>
       <c r="L35" s="33">
         <v>1</v>
@@ -3896,7 +3916,7 @@
         <v>100</v>
       </c>
       <c r="Q35" s="69" t="s">
-        <v>220</v>
+        <v>215</v>
       </c>
       <c r="R35" s="36">
         <v>1.1999999999999999E-3</v>
@@ -3931,19 +3951,19 @@
         <v>97</v>
       </c>
       <c r="G36" s="74" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="H36" s="30" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="I36" s="31" t="s">
-        <v>234</v>
+        <v>229</v>
       </c>
       <c r="J36" s="30" t="s">
-        <v>235</v>
+        <v>230</v>
       </c>
       <c r="K36" s="31" t="s">
-        <v>192</v>
+        <v>187</v>
       </c>
       <c r="L36" s="47">
         <v>1</v>
@@ -3962,7 +3982,7 @@
         <v>100</v>
       </c>
       <c r="Q36" s="68" t="s">
-        <v>220</v>
+        <v>215</v>
       </c>
       <c r="R36" s="35">
         <v>5.9999999999999995E-4</v>
@@ -3997,17 +4017,17 @@
         <v>98</v>
       </c>
       <c r="G37" s="34" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="H37" s="33" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="I37" s="34"/>
       <c r="J37" s="33" t="s">
-        <v>170</v>
+        <v>165</v>
       </c>
       <c r="K37" s="34" t="s">
-        <v>193</v>
+        <v>188</v>
       </c>
       <c r="L37" s="33">
         <v>1</v>
@@ -4026,7 +4046,7 @@
         <v>10</v>
       </c>
       <c r="Q37" s="69" t="s">
-        <v>220</v>
+        <v>215</v>
       </c>
       <c r="R37" s="36">
         <v>4.53E-2</v>
@@ -4052,7 +4072,7 @@
         <v>11</v>
       </c>
       <c r="D38" s="31" t="s">
-        <v>243</v>
+        <v>238</v>
       </c>
       <c r="E38" s="48" t="s">
         <v>73</v>
@@ -4061,17 +4081,17 @@
         <v>94</v>
       </c>
       <c r="G38" s="31" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="H38" s="30" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="I38" s="31"/>
       <c r="J38" s="30" t="s">
-        <v>171</v>
+        <v>166</v>
       </c>
       <c r="K38" s="31" t="s">
-        <v>194</v>
+        <v>189</v>
       </c>
       <c r="L38" s="47">
         <v>1</v>
@@ -4090,7 +4110,7 @@
         <v>100</v>
       </c>
       <c r="Q38" s="68" t="s">
-        <v>220</v>
+        <v>215</v>
       </c>
       <c r="R38" s="35">
         <v>1.1999999999999999E-3</v>
@@ -4113,26 +4133,26 @@
         <v>11</v>
       </c>
       <c r="D39" s="33" t="s">
-        <v>248</v>
+        <v>243</v>
       </c>
       <c r="E39" s="34" t="s">
-        <v>249</v>
+        <v>244</v>
       </c>
       <c r="F39" s="33" t="s">
         <v>94</v>
       </c>
       <c r="G39" s="34" t="s">
-        <v>250</v>
+        <v>245</v>
       </c>
       <c r="H39" s="33" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="I39" s="33"/>
       <c r="J39" s="33" t="s">
-        <v>252</v>
+        <v>247</v>
       </c>
       <c r="K39" s="33" t="s">
-        <v>251</v>
+        <v>246</v>
       </c>
       <c r="L39" s="34">
         <v>1</v>
@@ -4149,8 +4169,8 @@
       <c r="P39" s="66">
         <v>100</v>
       </c>
-      <c r="Q39" s="88" t="s">
-        <v>220</v>
+      <c r="Q39" s="77" t="s">
+        <v>215</v>
       </c>
       <c r="R39" s="36">
         <v>1.1000000000000001E-3</v>
@@ -4173,59 +4193,59 @@
         <v>31</v>
       </c>
       <c r="C40" s="30" t="s">
-        <v>200</v>
+        <v>195</v>
       </c>
       <c r="D40" s="30" t="s">
         <v>28</v>
       </c>
       <c r="E40" s="30" t="s">
-        <v>221</v>
+        <v>216</v>
       </c>
       <c r="F40" s="30" t="s">
         <v>89</v>
       </c>
       <c r="G40" s="30" t="s">
-        <v>222</v>
+        <v>217</v>
       </c>
       <c r="H40" s="30" t="s">
-        <v>222</v>
+        <v>217</v>
       </c>
       <c r="I40" s="30"/>
       <c r="J40" s="30" t="s">
-        <v>222</v>
+        <v>217</v>
       </c>
       <c r="K40" s="30" t="s">
-        <v>184</v>
+        <v>179</v>
       </c>
       <c r="L40" s="30" t="s">
-        <v>222</v>
+        <v>217</v>
       </c>
       <c r="M40" s="30" t="s">
-        <v>222</v>
+        <v>217</v>
       </c>
       <c r="N40" s="30" t="s">
-        <v>222</v>
+        <v>217</v>
       </c>
       <c r="O40" s="30" t="s">
-        <v>222</v>
+        <v>217</v>
       </c>
       <c r="P40" s="30" t="s">
-        <v>222</v>
+        <v>217</v>
       </c>
       <c r="Q40" s="30" t="s">
-        <v>222</v>
+        <v>217</v>
       </c>
       <c r="R40" s="30" t="s">
-        <v>222</v>
+        <v>217</v>
       </c>
       <c r="S40" s="30" t="s">
-        <v>222</v>
+        <v>217</v>
       </c>
       <c r="T40" s="30" t="s">
-        <v>222</v>
+        <v>217</v>
       </c>
       <c r="U40" s="30" t="s">
-        <v>222</v>
+        <v>217</v>
       </c>
       <c r="V40" s="30"/>
     </row>
@@ -4236,7 +4256,7 @@
         <v>32</v>
       </c>
       <c r="C41" s="33" t="s">
-        <v>201</v>
+        <v>196</v>
       </c>
       <c r="D41" s="33" t="s">
         <v>30</v>
@@ -4248,47 +4268,47 @@
         <v>91</v>
       </c>
       <c r="G41" s="33" t="s">
-        <v>222</v>
+        <v>217</v>
       </c>
       <c r="H41" s="33" t="s">
-        <v>222</v>
+        <v>217</v>
       </c>
       <c r="I41" s="33"/>
       <c r="J41" s="33" t="s">
-        <v>222</v>
+        <v>217</v>
       </c>
       <c r="K41" s="33" t="s">
-        <v>185</v>
+        <v>180</v>
       </c>
       <c r="L41" s="33" t="s">
-        <v>222</v>
+        <v>217</v>
       </c>
       <c r="M41" s="33" t="s">
-        <v>222</v>
+        <v>217</v>
       </c>
       <c r="N41" s="33" t="s">
-        <v>222</v>
+        <v>217</v>
       </c>
       <c r="O41" s="33" t="s">
-        <v>222</v>
+        <v>217</v>
       </c>
       <c r="P41" s="33" t="s">
-        <v>222</v>
+        <v>217</v>
       </c>
       <c r="Q41" s="33" t="s">
-        <v>222</v>
+        <v>217</v>
       </c>
       <c r="R41" s="33" t="s">
-        <v>222</v>
+        <v>217</v>
       </c>
       <c r="S41" s="33" t="s">
-        <v>222</v>
+        <v>217</v>
       </c>
       <c r="T41" s="33" t="s">
-        <v>222</v>
+        <v>217</v>
       </c>
       <c r="U41" s="33" t="s">
-        <v>222</v>
+        <v>217</v>
       </c>
       <c r="V41" s="33"/>
     </row>
@@ -4299,7 +4319,7 @@
         <v>33</v>
       </c>
       <c r="C42" s="30" t="s">
-        <v>202</v>
+        <v>197</v>
       </c>
       <c r="D42" s="30" t="s">
         <v>40</v>
@@ -4311,17 +4331,17 @@
         <v>99</v>
       </c>
       <c r="G42" s="30" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="H42" s="30" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="I42" s="30"/>
       <c r="J42" s="30" t="s">
-        <v>172</v>
+        <v>167</v>
       </c>
       <c r="K42" s="30" t="s">
-        <v>222</v>
+        <v>217</v>
       </c>
       <c r="L42" s="30">
         <v>1</v>
@@ -4340,7 +4360,7 @@
         <v>10</v>
       </c>
       <c r="Q42" s="68" t="s">
-        <v>220</v>
+        <v>215</v>
       </c>
       <c r="R42" s="35">
         <v>5.7599999999999998E-2</v>
@@ -4375,15 +4395,15 @@
         <v>100</v>
       </c>
       <c r="G43" s="33" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="H43" s="33" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="I43" s="33"/>
       <c r="J43" s="33"/>
       <c r="K43" s="33" t="s">
-        <v>222</v>
+        <v>217</v>
       </c>
       <c r="L43" s="33">
         <v>1</v>
@@ -4392,15 +4412,33 @@
         <f t="shared" ref="M43:M44" si="14">L43*5</f>
         <v>5</v>
       </c>
-      <c r="N43" s="33"/>
-      <c r="O43" s="33"/>
-      <c r="P43" s="33"/>
-      <c r="Q43" s="33"/>
-      <c r="R43" s="33"/>
-      <c r="S43" s="33"/>
-      <c r="T43" s="33"/>
-      <c r="U43" s="33"/>
-      <c r="V43" s="33"/>
+      <c r="N43" s="33">
+        <v>5</v>
+      </c>
+      <c r="O43" s="33">
+        <v>10</v>
+      </c>
+      <c r="P43" s="33">
+        <v>10</v>
+      </c>
+      <c r="Q43" s="33" t="s">
+        <v>257</v>
+      </c>
+      <c r="R43" s="36">
+        <v>6.5</v>
+      </c>
+      <c r="S43" s="36">
+        <v>32.5</v>
+      </c>
+      <c r="T43" s="36">
+        <v>6.5</v>
+      </c>
+      <c r="U43" s="36">
+        <v>65</v>
+      </c>
+      <c r="V43" s="91" t="s">
+        <v>258</v>
+      </c>
     </row>
     <row r="44" spans="1:22" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A44" s="75"/>
@@ -4415,21 +4453,21 @@
         <v>42</v>
       </c>
       <c r="E44" s="30" t="s">
-        <v>244</v>
+        <v>239</v>
       </c>
       <c r="F44" s="30" t="s">
-        <v>245</v>
+        <v>240</v>
       </c>
       <c r="G44" s="30" t="s">
-        <v>246</v>
+        <v>241</v>
       </c>
       <c r="H44" s="30" t="s">
-        <v>247</v>
+        <v>242</v>
       </c>
       <c r="I44" s="30"/>
       <c r="J44" s="30"/>
       <c r="K44" s="30" t="s">
-        <v>222</v>
+        <v>217</v>
       </c>
       <c r="L44" s="30">
         <v>1</v>
@@ -4438,15 +4476,33 @@
         <f t="shared" si="14"/>
         <v>5</v>
       </c>
-      <c r="N44" s="30"/>
-      <c r="O44" s="30"/>
-      <c r="P44" s="30"/>
-      <c r="Q44" s="30"/>
-      <c r="R44" s="30"/>
-      <c r="S44" s="30"/>
-      <c r="T44" s="30"/>
-      <c r="U44" s="30"/>
-      <c r="V44" s="30"/>
+      <c r="N44" s="30">
+        <v>5</v>
+      </c>
+      <c r="O44" s="30">
+        <v>10</v>
+      </c>
+      <c r="P44" s="30">
+        <v>10</v>
+      </c>
+      <c r="Q44" s="30" t="s">
+        <v>257</v>
+      </c>
+      <c r="R44" s="35">
+        <v>6.5</v>
+      </c>
+      <c r="S44" s="35">
+        <v>32.5</v>
+      </c>
+      <c r="T44" s="35">
+        <v>6.5</v>
+      </c>
+      <c r="U44" s="35">
+        <v>65</v>
+      </c>
+      <c r="V44" s="92" t="s">
+        <v>258</v>
+      </c>
     </row>
     <row r="45" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A45" s="1"/>
@@ -4467,17 +4523,17 @@
         <v>101</v>
       </c>
       <c r="G45" s="33" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="H45" s="33" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="I45" s="33"/>
       <c r="J45" s="33" t="s">
-        <v>236</v>
+        <v>231</v>
       </c>
       <c r="K45" s="33" t="s">
-        <v>222</v>
+        <v>217</v>
       </c>
       <c r="L45" s="33">
         <v>1</v>
@@ -4495,8 +4551,8 @@
       <c r="P45" s="33">
         <v>10</v>
       </c>
-      <c r="Q45" s="90" t="s">
-        <v>220</v>
+      <c r="Q45" s="79" t="s">
+        <v>215</v>
       </c>
       <c r="R45" s="36">
         <v>1.2919</v>
@@ -4531,17 +4587,17 @@
         <v>102</v>
       </c>
       <c r="G46" s="30" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="H46" s="30" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="I46" s="30"/>
       <c r="J46" s="30" t="s">
-        <v>173</v>
+        <v>168</v>
       </c>
       <c r="K46" s="30" t="s">
-        <v>222</v>
+        <v>217</v>
       </c>
       <c r="L46" s="30">
         <v>1</v>
@@ -4559,8 +4615,8 @@
       <c r="P46" s="30">
         <v>10</v>
       </c>
-      <c r="Q46" s="89" t="s">
-        <v>220</v>
+      <c r="Q46" s="78" t="s">
+        <v>215</v>
       </c>
       <c r="R46" s="35">
         <v>7.6300000000000007E-2</v>
@@ -4593,20 +4649,20 @@
       <c r="N47" s="25"/>
       <c r="O47" s="25"/>
       <c r="P47" s="25"/>
-      <c r="Q47" s="84" t="s">
-        <v>237</v>
-      </c>
-      <c r="R47" s="85"/>
+      <c r="Q47" s="87" t="s">
+        <v>232</v>
+      </c>
+      <c r="R47" s="88"/>
       <c r="S47" s="71">
         <f>SUM(S10:S46)</f>
-        <v>41.26</v>
+        <v>106.20999999999998</v>
       </c>
       <c r="T47" s="25"/>
       <c r="U47" s="71">
         <f>SUM(U10:U46)</f>
-        <v>70.789999999999992</v>
-      </c>
-      <c r="V47" s="82"/>
+        <v>200.73999999999998</v>
+      </c>
+      <c r="V47" s="85"/>
     </row>
     <row r="48" spans="1:22" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A48" s="1"/>
@@ -4625,20 +4681,20 @@
       <c r="N48" s="8"/>
       <c r="O48" s="8"/>
       <c r="P48" s="8"/>
-      <c r="Q48" s="86" t="s">
-        <v>238</v>
-      </c>
-      <c r="R48" s="87"/>
+      <c r="Q48" s="89" t="s">
+        <v>233</v>
+      </c>
+      <c r="R48" s="90"/>
       <c r="S48" s="72">
         <f>(S47/5)</f>
-        <v>8.2519999999999989</v>
+        <v>21.241999999999997</v>
       </c>
       <c r="T48" s="8"/>
       <c r="U48" s="72">
         <f>(U47/10)</f>
-        <v>7.0789999999999988</v>
-      </c>
-      <c r="V48" s="83"/>
+        <v>20.073999999999998</v>
+      </c>
+      <c r="V48" s="86"/>
     </row>
   </sheetData>
   <mergeCells count="5">

</xml_diff>